<commit_message>
Verhoog maximale rennerprijs naar 4500 BC
</commit_message>
<xml_diff>
--- a/outputs/vuelta-2026-20260818/Wielerpool_prijslijst_vuelta_2026.xlsx
+++ b/outputs/vuelta-2026-20260818/Wielerpool_prijslijst_vuelta_2026.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Renners" sheetId="1" r:id="Rdaffe2d8cb2c4eb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instellingen" sheetId="2" r:id="R2602df3a4f9e4831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Renners" sheetId="1" r:id="R6e81a16643b445c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instellingen" sheetId="2" r:id="R6f7f9a1daf8146a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -281,7 +281,7 @@
     <x:col min="12" max="12" width="8.75" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="15.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="9.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="10.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="11.75" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="53.5" hidden="0" customWidth="1"/>
   </x:cols>
@@ -404,12 +404,12 @@
       </x:c>
       <x:c r="L6" t="n">
         <x:f>IF(K6="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K6/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>475</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="M6"/>
       <x:c r="N6" t="n">
         <x:f>IF(L6="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L6+IF(M6="",0,M6))))</x:f>
-        <x:v>475</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="O6" t="str">
         <x:f>IF(N6="","",IF(N6&gt;='Instellingen'!$B$22,"Absolute top",IF(N6&gt;='Instellingen'!$B$23,"Kopman",IF(N6&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N6&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -462,12 +462,12 @@
       </x:c>
       <x:c r="L7" t="n">
         <x:f>IF(K7="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K7/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>482</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="M7"/>
       <x:c r="N7" t="n">
         <x:f>IF(L7="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L7+IF(M7="",0,M7))))</x:f>
-        <x:v>482</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="O7" t="str">
         <x:f>IF(N7="","",IF(N7&gt;='Instellingen'!$B$22,"Absolute top",IF(N7&gt;='Instellingen'!$B$23,"Kopman",IF(N7&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N7&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -520,12 +520,12 @@
       </x:c>
       <x:c r="L8" t="n">
         <x:f>IF(K8="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K8/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>400</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="M8"/>
       <x:c r="N8" t="n">
         <x:f>IF(L8="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L8+IF(M8="",0,M8))))</x:f>
-        <x:v>400</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="O8" t="str">
         <x:f>IF(N8="","",IF(N8&gt;='Instellingen'!$B$22,"Absolute top",IF(N8&gt;='Instellingen'!$B$23,"Kopman",IF(N8&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N8&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -578,12 +578,12 @@
       </x:c>
       <x:c r="L9" t="n">
         <x:f>IF(K9="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K9/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>445</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="M9"/>
       <x:c r="N9" t="n">
         <x:f>IF(L9="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L9+IF(M9="",0,M9))))</x:f>
-        <x:v>445</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="O9" t="str">
         <x:f>IF(N9="","",IF(N9&gt;='Instellingen'!$B$22,"Absolute top",IF(N9&gt;='Instellingen'!$B$23,"Kopman",IF(N9&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N9&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -636,16 +636,16 @@
       </x:c>
       <x:c r="L10" t="n">
         <x:f>IF(K10="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K10/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>587</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="M10"/>
       <x:c r="N10" t="n">
         <x:f>IF(L10="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L10+IF(M10="",0,M10))))</x:f>
-        <x:v>587</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="O10" t="str">
         <x:f>IF(N10="","",IF(N10&gt;='Instellingen'!$B$22,"Absolute top",IF(N10&gt;='Instellingen'!$B$23,"Kopman",IF(N10&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N10&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P10" t="str">
         <x:f>IF(A10="","",IF(D10="","Rol invullen","Compleet"))</x:f>
@@ -694,16 +694,16 @@
       </x:c>
       <x:c r="L11" t="n">
         <x:f>IF(K11="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K11/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>656</x:v>
+        <x:v>979</x:v>
       </x:c>
       <x:c r="M11"/>
       <x:c r="N11" t="n">
         <x:f>IF(L11="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L11+IF(M11="",0,M11))))</x:f>
-        <x:v>656</x:v>
+        <x:v>979</x:v>
       </x:c>
       <x:c r="O11" t="str">
         <x:f>IF(N11="","",IF(N11&gt;='Instellingen'!$B$22,"Absolute top",IF(N11&gt;='Instellingen'!$B$23,"Kopman",IF(N11&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N11&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P11" t="str">
         <x:f>IF(A11="","",IF(D11="","Rol invullen","Compleet"))</x:f>
@@ -752,16 +752,16 @@
       </x:c>
       <x:c r="L12" t="n">
         <x:f>IF(K12="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K12/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>744</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="M12"/>
       <x:c r="N12" t="n">
         <x:f>IF(L12="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L12+IF(M12="",0,M12))))</x:f>
-        <x:v>744</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="O12" t="str">
         <x:f>IF(N12="","",IF(N12&gt;='Instellingen'!$B$22,"Absolute top",IF(N12&gt;='Instellingen'!$B$23,"Kopman",IF(N12&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N12&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P12" t="str">
         <x:f>IF(A12="","",IF(D12="","Rol invullen","Compleet"))</x:f>
@@ -810,12 +810,12 @@
       </x:c>
       <x:c r="L13" t="n">
         <x:f>IF(K13="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K13/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>493</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="M13"/>
       <x:c r="N13" t="n">
         <x:f>IF(L13="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L13+IF(M13="",0,M13))))</x:f>
-        <x:v>493</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="O13" t="str">
         <x:f>IF(N13="","",IF(N13&gt;='Instellingen'!$B$22,"Absolute top",IF(N13&gt;='Instellingen'!$B$23,"Kopman",IF(N13&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N13&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -868,16 +868,16 @@
       </x:c>
       <x:c r="L14" t="n">
         <x:f>IF(K14="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K14/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>1054</x:v>
+        <x:v>1740</x:v>
       </x:c>
       <x:c r="M14"/>
       <x:c r="N14" t="n">
         <x:f>IF(L14="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L14+IF(M14="",0,M14))))</x:f>
-        <x:v>1054</x:v>
+        <x:v>1740</x:v>
       </x:c>
       <x:c r="O14" t="str">
         <x:f>IF(N14="","",IF(N14&gt;='Instellingen'!$B$22,"Absolute top",IF(N14&gt;='Instellingen'!$B$23,"Kopman",IF(N14&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N14&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Kopman</x:v>
       </x:c>
       <x:c r="P14" t="str">
         <x:f>IF(A14="","",IF(D14="","Rol invullen","Compleet"))</x:f>
@@ -926,12 +926,12 @@
       </x:c>
       <x:c r="L15" t="n">
         <x:f>IF(K15="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K15/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>377</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="M15"/>
       <x:c r="N15" t="n">
         <x:f>IF(L15="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L15+IF(M15="",0,M15))))</x:f>
-        <x:v>377</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="O15" t="str">
         <x:f>IF(N15="","",IF(N15&gt;='Instellingen'!$B$22,"Absolute top",IF(N15&gt;='Instellingen'!$B$23,"Kopman",IF(N15&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N15&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -984,16 +984,16 @@
       </x:c>
       <x:c r="L16" t="n">
         <x:f>IF(K16="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K16/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>999</x:v>
+        <x:v>1634</x:v>
       </x:c>
       <x:c r="M16"/>
       <x:c r="N16" t="n">
         <x:f>IF(L16="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L16+IF(M16="",0,M16))))</x:f>
-        <x:v>999</x:v>
+        <x:v>1634</x:v>
       </x:c>
       <x:c r="O16" t="str">
         <x:f>IF(N16="","",IF(N16&gt;='Instellingen'!$B$22,"Absolute top",IF(N16&gt;='Instellingen'!$B$23,"Kopman",IF(N16&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N16&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Kopman</x:v>
       </x:c>
       <x:c r="P16" t="str">
         <x:f>IF(A16="","",IF(D16="","Rol invullen","Compleet"))</x:f>
@@ -1042,12 +1042,12 @@
       </x:c>
       <x:c r="L17" t="n">
         <x:f>IF(K17="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K17/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>452</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="M17"/>
       <x:c r="N17" t="n">
         <x:f>IF(L17="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L17+IF(M17="",0,M17))))</x:f>
-        <x:v>452</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="O17" t="str">
         <x:f>IF(N17="","",IF(N17&gt;='Instellingen'!$B$22,"Absolute top",IF(N17&gt;='Instellingen'!$B$23,"Kopman",IF(N17&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N17&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -1100,16 +1100,16 @@
       </x:c>
       <x:c r="L18" t="n">
         <x:f>IF(K18="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K18/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>606</x:v>
+        <x:v>884</x:v>
       </x:c>
       <x:c r="M18"/>
       <x:c r="N18" t="n">
         <x:f>IF(L18="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L18+IF(M18="",0,M18))))</x:f>
-        <x:v>606</x:v>
+        <x:v>884</x:v>
       </x:c>
       <x:c r="O18" t="str">
         <x:f>IF(N18="","",IF(N18&gt;='Instellingen'!$B$22,"Absolute top",IF(N18&gt;='Instellingen'!$B$23,"Kopman",IF(N18&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N18&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P18" t="str">
         <x:f>IF(A18="","",IF(D18="","Rol invullen","Compleet"))</x:f>
@@ -1158,16 +1158,16 @@
       </x:c>
       <x:c r="L19" t="n">
         <x:f>IF(K19="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K19/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>588</x:v>
+        <x:v>850</x:v>
       </x:c>
       <x:c r="M19"/>
       <x:c r="N19" t="n">
         <x:f>IF(L19="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L19+IF(M19="",0,M19))))</x:f>
-        <x:v>588</x:v>
+        <x:v>850</x:v>
       </x:c>
       <x:c r="O19" t="str">
         <x:f>IF(N19="","",IF(N19&gt;='Instellingen'!$B$22,"Absolute top",IF(N19&gt;='Instellingen'!$B$23,"Kopman",IF(N19&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N19&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P19" t="str">
         <x:f>IF(A19="","",IF(D19="","Rol invullen","Compleet"))</x:f>
@@ -1216,16 +1216,16 @@
       </x:c>
       <x:c r="L20" t="n">
         <x:f>IF(K20="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K20/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>958</x:v>
+        <x:v>1557</x:v>
       </x:c>
       <x:c r="M20"/>
       <x:c r="N20" t="n">
         <x:f>IF(L20="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L20+IF(M20="",0,M20))))</x:f>
-        <x:v>958</x:v>
+        <x:v>1557</x:v>
       </x:c>
       <x:c r="O20" t="str">
         <x:f>IF(N20="","",IF(N20&gt;='Instellingen'!$B$22,"Absolute top",IF(N20&gt;='Instellingen'!$B$23,"Kopman",IF(N20&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N20&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P20" t="str">
         <x:f>IF(A20="","",IF(D20="","Rol invullen","Compleet"))</x:f>
@@ -1274,16 +1274,16 @@
       </x:c>
       <x:c r="L21" t="n">
         <x:f>IF(K21="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K21/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>522</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="M21"/>
       <x:c r="N21" t="n">
         <x:f>IF(L21="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L21+IF(M21="",0,M21))))</x:f>
-        <x:v>522</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="O21" t="str">
         <x:f>IF(N21="","",IF(N21&gt;='Instellingen'!$B$22,"Absolute top",IF(N21&gt;='Instellingen'!$B$23,"Kopman",IF(N21&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N21&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P21" t="str">
         <x:f>IF(A21="","",IF(D21="","Rol invullen","Compleet"))</x:f>
@@ -1332,16 +1332,16 @@
       </x:c>
       <x:c r="L22" t="n">
         <x:f>IF(K22="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K22/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>877</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="M22"/>
       <x:c r="N22" t="n">
         <x:f>IF(L22="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L22+IF(M22="",0,M22))))</x:f>
-        <x:v>877</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="O22" t="str">
         <x:f>IF(N22="","",IF(N22&gt;='Instellingen'!$B$22,"Absolute top",IF(N22&gt;='Instellingen'!$B$23,"Kopman",IF(N22&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N22&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P22" t="str">
         <x:f>IF(A22="","",IF(D22="","Rol invullen","Compleet"))</x:f>
@@ -1390,16 +1390,16 @@
       </x:c>
       <x:c r="L23" t="n">
         <x:f>IF(K23="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K23/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>830</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="M23"/>
       <x:c r="N23" t="n">
         <x:f>IF(L23="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L23+IF(M23="",0,M23))))</x:f>
-        <x:v>830</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="O23" t="str">
         <x:f>IF(N23="","",IF(N23&gt;='Instellingen'!$B$22,"Absolute top",IF(N23&gt;='Instellingen'!$B$23,"Kopman",IF(N23&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N23&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P23" t="str">
         <x:f>IF(A23="","",IF(D23="","Rol invullen","Compleet"))</x:f>
@@ -1448,12 +1448,12 @@
       </x:c>
       <x:c r="L24" t="n">
         <x:f>IF(K24="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K24/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>377</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="M24"/>
       <x:c r="N24" t="n">
         <x:f>IF(L24="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L24+IF(M24="",0,M24))))</x:f>
-        <x:v>377</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="O24" t="str">
         <x:f>IF(N24="","",IF(N24&gt;='Instellingen'!$B$22,"Absolute top",IF(N24&gt;='Instellingen'!$B$23,"Kopman",IF(N24&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N24&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -1506,16 +1506,16 @@
       </x:c>
       <x:c r="L25" t="n">
         <x:f>IF(K25="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K25/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>587</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="M25"/>
       <x:c r="N25" t="n">
         <x:f>IF(L25="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L25+IF(M25="",0,M25))))</x:f>
-        <x:v>587</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="O25" t="str">
         <x:f>IF(N25="","",IF(N25&gt;='Instellingen'!$B$22,"Absolute top",IF(N25&gt;='Instellingen'!$B$23,"Kopman",IF(N25&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N25&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P25" t="str">
         <x:f>IF(A25="","",IF(D25="","Rol invullen","Compleet"))</x:f>
@@ -1564,16 +1564,16 @@
       </x:c>
       <x:c r="L26" t="n">
         <x:f>IF(K26="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K26/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>892</x:v>
+        <x:v>1430</x:v>
       </x:c>
       <x:c r="M26"/>
       <x:c r="N26" t="n">
         <x:f>IF(L26="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L26+IF(M26="",0,M26))))</x:f>
-        <x:v>892</x:v>
+        <x:v>1430</x:v>
       </x:c>
       <x:c r="O26" t="str">
         <x:f>IF(N26="","",IF(N26&gt;='Instellingen'!$B$22,"Absolute top",IF(N26&gt;='Instellingen'!$B$23,"Kopman",IF(N26&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N26&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P26" t="str">
         <x:f>IF(A26="","",IF(D26="","Rol invullen","Compleet"))</x:f>
@@ -1622,12 +1622,12 @@
       </x:c>
       <x:c r="L27" t="n">
         <x:f>IF(K27="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K27/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>489</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="M27"/>
       <x:c r="N27" t="n">
         <x:f>IF(L27="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L27+IF(M27="",0,M27))))</x:f>
-        <x:v>489</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="O27" t="str">
         <x:f>IF(N27="","",IF(N27&gt;='Instellingen'!$B$22,"Absolute top",IF(N27&gt;='Instellingen'!$B$23,"Kopman",IF(N27&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N27&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -1680,12 +1680,12 @@
       </x:c>
       <x:c r="L28" t="n">
         <x:f>IF(K28="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K28/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>479</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="M28"/>
       <x:c r="N28" t="n">
         <x:f>IF(L28="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L28+IF(M28="",0,M28))))</x:f>
-        <x:v>479</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="O28" t="str">
         <x:f>IF(N28="","",IF(N28&gt;='Instellingen'!$B$22,"Absolute top",IF(N28&gt;='Instellingen'!$B$23,"Kopman",IF(N28&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N28&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -1738,12 +1738,12 @@
       </x:c>
       <x:c r="L29" t="n">
         <x:f>IF(K29="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K29/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>377</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="M29"/>
       <x:c r="N29" t="n">
         <x:f>IF(L29="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L29+IF(M29="",0,M29))))</x:f>
-        <x:v>377</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="O29" t="str">
         <x:f>IF(N29="","",IF(N29&gt;='Instellingen'!$B$22,"Absolute top",IF(N29&gt;='Instellingen'!$B$23,"Kopman",IF(N29&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N29&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -1796,12 +1796,12 @@
       </x:c>
       <x:c r="L30" t="n">
         <x:f>IF(K30="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K30/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>400</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="M30"/>
       <x:c r="N30" t="n">
         <x:f>IF(L30="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L30+IF(M30="",0,M30))))</x:f>
-        <x:v>400</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="O30" t="str">
         <x:f>IF(N30="","",IF(N30&gt;='Instellingen'!$B$22,"Absolute top",IF(N30&gt;='Instellingen'!$B$23,"Kopman",IF(N30&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N30&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -1854,16 +1854,16 @@
       </x:c>
       <x:c r="L31" t="n">
         <x:f>IF(K31="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K31/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>631</x:v>
+        <x:v>932</x:v>
       </x:c>
       <x:c r="M31"/>
       <x:c r="N31" t="n">
         <x:f>IF(L31="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L31+IF(M31="",0,M31))))</x:f>
-        <x:v>631</x:v>
+        <x:v>932</x:v>
       </x:c>
       <x:c r="O31" t="str">
         <x:f>IF(N31="","",IF(N31&gt;='Instellingen'!$B$22,"Absolute top",IF(N31&gt;='Instellingen'!$B$23,"Kopman",IF(N31&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N31&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P31" t="str">
         <x:f>IF(A31="","",IF(D31="","Rol invullen","Compleet"))</x:f>
@@ -1912,16 +1912,16 @@
       </x:c>
       <x:c r="L32" t="n">
         <x:f>IF(K32="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K32/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>562</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="M32"/>
       <x:c r="N32" t="n">
         <x:f>IF(L32="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L32+IF(M32="",0,M32))))</x:f>
-        <x:v>562</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="O32" t="str">
         <x:f>IF(N32="","",IF(N32&gt;='Instellingen'!$B$22,"Absolute top",IF(N32&gt;='Instellingen'!$B$23,"Kopman",IF(N32&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N32&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P32" t="str">
         <x:f>IF(A32="","",IF(D32="","Rol invullen","Compleet"))</x:f>
@@ -1970,12 +1970,12 @@
       </x:c>
       <x:c r="L33" t="n">
         <x:f>IF(K33="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K33/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>452</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="M33"/>
       <x:c r="N33" t="n">
         <x:f>IF(L33="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L33+IF(M33="",0,M33))))</x:f>
-        <x:v>452</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="O33" t="str">
         <x:f>IF(N33="","",IF(N33&gt;='Instellingen'!$B$22,"Absolute top",IF(N33&gt;='Instellingen'!$B$23,"Kopman",IF(N33&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N33&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -2028,12 +2028,12 @@
       </x:c>
       <x:c r="L34" t="n">
         <x:f>IF(K34="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K34/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>483</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="M34"/>
       <x:c r="N34" t="n">
         <x:f>IF(L34="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L34+IF(M34="",0,M34))))</x:f>
-        <x:v>483</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="O34" t="str">
         <x:f>IF(N34="","",IF(N34&gt;='Instellingen'!$B$22,"Absolute top",IF(N34&gt;='Instellingen'!$B$23,"Kopman",IF(N34&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N34&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -2086,16 +2086,16 @@
       </x:c>
       <x:c r="L35" t="n">
         <x:f>IF(K35="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K35/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>1089</x:v>
+        <x:v>1807</x:v>
       </x:c>
       <x:c r="M35"/>
       <x:c r="N35" t="n">
         <x:f>IF(L35="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L35+IF(M35="",0,M35))))</x:f>
-        <x:v>1089</x:v>
+        <x:v>1807</x:v>
       </x:c>
       <x:c r="O35" t="str">
         <x:f>IF(N35="","",IF(N35&gt;='Instellingen'!$B$22,"Absolute top",IF(N35&gt;='Instellingen'!$B$23,"Kopman",IF(N35&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N35&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Kopman</x:v>
       </x:c>
       <x:c r="P35" t="str">
         <x:f>IF(A35="","",IF(D35="","Rol invullen","Compleet"))</x:f>
@@ -2144,16 +2144,16 @@
       </x:c>
       <x:c r="L36" t="n">
         <x:f>IF(K36="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K36/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>599</x:v>
+        <x:v>872</x:v>
       </x:c>
       <x:c r="M36"/>
       <x:c r="N36" t="n">
         <x:f>IF(L36="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L36+IF(M36="",0,M36))))</x:f>
-        <x:v>599</x:v>
+        <x:v>872</x:v>
       </x:c>
       <x:c r="O36" t="str">
         <x:f>IF(N36="","",IF(N36&gt;='Instellingen'!$B$22,"Absolute top",IF(N36&gt;='Instellingen'!$B$23,"Kopman",IF(N36&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N36&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P36" t="str">
         <x:f>IF(A36="","",IF(D36="","Rol invullen","Compleet"))</x:f>
@@ -2202,16 +2202,16 @@
       </x:c>
       <x:c r="L37" t="n">
         <x:f>IF(K37="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K37/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>663</x:v>
+        <x:v>992</x:v>
       </x:c>
       <x:c r="M37"/>
       <x:c r="N37" t="n">
         <x:f>IF(L37="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L37+IF(M37="",0,M37))))</x:f>
-        <x:v>663</x:v>
+        <x:v>992</x:v>
       </x:c>
       <x:c r="O37" t="str">
         <x:f>IF(N37="","",IF(N37&gt;='Instellingen'!$B$22,"Absolute top",IF(N37&gt;='Instellingen'!$B$23,"Kopman",IF(N37&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N37&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P37" t="str">
         <x:f>IF(A37="","",IF(D37="","Rol invullen","Compleet"))</x:f>
@@ -2260,16 +2260,16 @@
       </x:c>
       <x:c r="L38" t="n">
         <x:f>IF(K38="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K38/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>515</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="M38"/>
       <x:c r="N38" t="n">
         <x:f>IF(L38="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L38+IF(M38="",0,M38))))</x:f>
-        <x:v>515</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="O38" t="str">
         <x:f>IF(N38="","",IF(N38&gt;='Instellingen'!$B$22,"Absolute top",IF(N38&gt;='Instellingen'!$B$23,"Kopman",IF(N38&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N38&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P38" t="str">
         <x:f>IF(A38="","",IF(D38="","Rol invullen","Compleet"))</x:f>
@@ -2318,16 +2318,16 @@
       </x:c>
       <x:c r="L39" t="n">
         <x:f>IF(K39="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K39/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>596</x:v>
+        <x:v>865</x:v>
       </x:c>
       <x:c r="M39"/>
       <x:c r="N39" t="n">
         <x:f>IF(L39="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L39+IF(M39="",0,M39))))</x:f>
-        <x:v>596</x:v>
+        <x:v>865</x:v>
       </x:c>
       <x:c r="O39" t="str">
         <x:f>IF(N39="","",IF(N39&gt;='Instellingen'!$B$22,"Absolute top",IF(N39&gt;='Instellingen'!$B$23,"Kopman",IF(N39&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N39&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P39" t="str">
         <x:f>IF(A39="","",IF(D39="","Rol invullen","Compleet"))</x:f>
@@ -2376,12 +2376,12 @@
       </x:c>
       <x:c r="L40" t="n">
         <x:f>IF(K40="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K40/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>351</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="M40"/>
       <x:c r="N40" t="n">
         <x:f>IF(L40="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L40+IF(M40="",0,M40))))</x:f>
-        <x:v>351</x:v>
+        <x:v>397</x:v>
       </x:c>
       <x:c r="O40" t="str">
         <x:f>IF(N40="","",IF(N40&gt;='Instellingen'!$B$22,"Absolute top",IF(N40&gt;='Instellingen'!$B$23,"Kopman",IF(N40&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N40&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -2434,16 +2434,16 @@
       </x:c>
       <x:c r="L41" t="n">
         <x:f>IF(K41="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K41/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>660</x:v>
+        <x:v>988</x:v>
       </x:c>
       <x:c r="M41"/>
       <x:c r="N41" t="n">
         <x:f>IF(L41="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L41+IF(M41="",0,M41))))</x:f>
-        <x:v>660</x:v>
+        <x:v>988</x:v>
       </x:c>
       <x:c r="O41" t="str">
         <x:f>IF(N41="","",IF(N41&gt;='Instellingen'!$B$22,"Absolute top",IF(N41&gt;='Instellingen'!$B$23,"Kopman",IF(N41&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N41&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P41" t="str">
         <x:f>IF(A41="","",IF(D41="","Rol invullen","Compleet"))</x:f>
@@ -2492,16 +2492,16 @@
       </x:c>
       <x:c r="L42" t="n">
         <x:f>IF(K42="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K42/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>890</x:v>
+        <x:v>1427</x:v>
       </x:c>
       <x:c r="M42"/>
       <x:c r="N42" t="n">
         <x:f>IF(L42="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L42+IF(M42="",0,M42))))</x:f>
-        <x:v>890</x:v>
+        <x:v>1427</x:v>
       </x:c>
       <x:c r="O42" t="str">
         <x:f>IF(N42="","",IF(N42&gt;='Instellingen'!$B$22,"Absolute top",IF(N42&gt;='Instellingen'!$B$23,"Kopman",IF(N42&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N42&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P42" t="str">
         <x:f>IF(A42="","",IF(D42="","Rol invullen","Compleet"))</x:f>
@@ -2550,16 +2550,16 @@
       </x:c>
       <x:c r="L43" t="n">
         <x:f>IF(K43="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K43/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>1678</x:v>
+        <x:v>2931</x:v>
       </x:c>
       <x:c r="M43"/>
       <x:c r="N43" t="n">
         <x:f>IF(L43="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L43+IF(M43="",0,M43))))</x:f>
-        <x:v>1678</x:v>
+        <x:v>2931</x:v>
       </x:c>
       <x:c r="O43" t="str">
         <x:f>IF(N43="","",IF(N43&gt;='Instellingen'!$B$22,"Absolute top",IF(N43&gt;='Instellingen'!$B$23,"Kopman",IF(N43&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N43&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Kopman</x:v>
+        <x:v>Absolute top</x:v>
       </x:c>
       <x:c r="P43" t="str">
         <x:f>IF(A43="","",IF(D43="","Rol invullen","Compleet"))</x:f>
@@ -2608,16 +2608,16 @@
       </x:c>
       <x:c r="L44" t="n">
         <x:f>IF(K44="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K44/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>560</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="M44"/>
       <x:c r="N44" t="n">
         <x:f>IF(L44="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L44+IF(M44="",0,M44))))</x:f>
-        <x:v>560</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="O44" t="str">
         <x:f>IF(N44="","",IF(N44&gt;='Instellingen'!$B$22,"Absolute top",IF(N44&gt;='Instellingen'!$B$23,"Kopman",IF(N44&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N44&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P44" t="str">
         <x:f>IF(A44="","",IF(D44="","Rol invullen","Compleet"))</x:f>
@@ -2666,12 +2666,12 @@
       </x:c>
       <x:c r="L45" t="n">
         <x:f>IF(K45="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K45/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>489</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="M45"/>
       <x:c r="N45" t="n">
         <x:f>IF(L45="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L45+IF(M45="",0,M45))))</x:f>
-        <x:v>489</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="O45" t="str">
         <x:f>IF(N45="","",IF(N45&gt;='Instellingen'!$B$22,"Absolute top",IF(N45&gt;='Instellingen'!$B$23,"Kopman",IF(N45&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N45&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -2724,16 +2724,16 @@
       </x:c>
       <x:c r="L46" t="n">
         <x:f>IF(K46="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K46/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>551</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="M46"/>
       <x:c r="N46" t="n">
         <x:f>IF(L46="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L46+IF(M46="",0,M46))))</x:f>
-        <x:v>551</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="O46" t="str">
         <x:f>IF(N46="","",IF(N46&gt;='Instellingen'!$B$22,"Absolute top",IF(N46&gt;='Instellingen'!$B$23,"Kopman",IF(N46&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N46&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P46" t="str">
         <x:f>IF(A46="","",IF(D46="","Rol invullen","Compleet"))</x:f>
@@ -2782,12 +2782,12 @@
       </x:c>
       <x:c r="L47" t="n">
         <x:f>IF(K47="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K47/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>500</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="M47"/>
       <x:c r="N47" t="n">
         <x:f>IF(L47="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L47+IF(M47="",0,M47))))</x:f>
-        <x:v>500</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="O47" t="str">
         <x:f>IF(N47="","",IF(N47&gt;='Instellingen'!$B$22,"Absolute top",IF(N47&gt;='Instellingen'!$B$23,"Kopman",IF(N47&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N47&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -2840,12 +2840,12 @@
       </x:c>
       <x:c r="L48" t="n">
         <x:f>IF(K48="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K48/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>465</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="M48"/>
       <x:c r="N48" t="n">
         <x:f>IF(L48="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L48+IF(M48="",0,M48))))</x:f>
-        <x:v>465</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="O48" t="str">
         <x:f>IF(N48="","",IF(N48&gt;='Instellingen'!$B$22,"Absolute top",IF(N48&gt;='Instellingen'!$B$23,"Kopman",IF(N48&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N48&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -2898,16 +2898,16 @@
       </x:c>
       <x:c r="L49" t="n">
         <x:f>IF(K49="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K49/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>520</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="M49"/>
       <x:c r="N49" t="n">
         <x:f>IF(L49="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L49+IF(M49="",0,M49))))</x:f>
-        <x:v>520</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="O49" t="str">
         <x:f>IF(N49="","",IF(N49&gt;='Instellingen'!$B$22,"Absolute top",IF(N49&gt;='Instellingen'!$B$23,"Kopman",IF(N49&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N49&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P49" t="str">
         <x:f>IF(A49="","",IF(D49="","Rol invullen","Compleet"))</x:f>
@@ -2956,16 +2956,16 @@
       </x:c>
       <x:c r="L50" t="n">
         <x:f>IF(K50="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K50/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>1250</x:v>
+        <x:v>2113</x:v>
       </x:c>
       <x:c r="M50"/>
       <x:c r="N50" t="n">
         <x:f>IF(L50="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L50+IF(M50="",0,M50))))</x:f>
-        <x:v>1250</x:v>
+        <x:v>2113</x:v>
       </x:c>
       <x:c r="O50" t="str">
         <x:f>IF(N50="","",IF(N50&gt;='Instellingen'!$B$22,"Absolute top",IF(N50&gt;='Instellingen'!$B$23,"Kopman",IF(N50&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N50&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Sterke keuze</x:v>
+        <x:v>Kopman</x:v>
       </x:c>
       <x:c r="P50" t="str">
         <x:f>IF(A50="","",IF(D50="","Rol invullen","Compleet"))</x:f>
@@ -3014,16 +3014,16 @@
       </x:c>
       <x:c r="L51" t="n">
         <x:f>IF(K51="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K51/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>605</x:v>
+        <x:v>881</x:v>
       </x:c>
       <x:c r="M51"/>
       <x:c r="N51" t="n">
         <x:f>IF(L51="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L51+IF(M51="",0,M51))))</x:f>
-        <x:v>605</x:v>
+        <x:v>881</x:v>
       </x:c>
       <x:c r="O51" t="str">
         <x:f>IF(N51="","",IF(N51&gt;='Instellingen'!$B$22,"Absolute top",IF(N51&gt;='Instellingen'!$B$23,"Kopman",IF(N51&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N51&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P51" t="str">
         <x:f>IF(A51="","",IF(D51="","Rol invullen","Compleet"))</x:f>
@@ -3072,12 +3072,12 @@
       </x:c>
       <x:c r="L52" t="n">
         <x:f>IF(K52="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K52/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>445</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="M52"/>
       <x:c r="N52" t="n">
         <x:f>IF(L52="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L52+IF(M52="",0,M52))))</x:f>
-        <x:v>445</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="O52" t="str">
         <x:f>IF(N52="","",IF(N52&gt;='Instellingen'!$B$22,"Absolute top",IF(N52&gt;='Instellingen'!$B$23,"Kopman",IF(N52&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N52&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3130,12 +3130,12 @@
       </x:c>
       <x:c r="L53" t="n">
         <x:f>IF(K53="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K53/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>482</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="M53"/>
       <x:c r="N53" t="n">
         <x:f>IF(L53="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L53+IF(M53="",0,M53))))</x:f>
-        <x:v>482</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="O53" t="str">
         <x:f>IF(N53="","",IF(N53&gt;='Instellingen'!$B$22,"Absolute top",IF(N53&gt;='Instellingen'!$B$23,"Kopman",IF(N53&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N53&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3188,12 +3188,12 @@
       </x:c>
       <x:c r="L54" t="n">
         <x:f>IF(K54="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K54/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>492</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="M54"/>
       <x:c r="N54" t="n">
         <x:f>IF(L54="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L54+IF(M54="",0,M54))))</x:f>
-        <x:v>492</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="O54" t="str">
         <x:f>IF(N54="","",IF(N54&gt;='Instellingen'!$B$22,"Absolute top",IF(N54&gt;='Instellingen'!$B$23,"Kopman",IF(N54&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N54&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3246,12 +3246,12 @@
       </x:c>
       <x:c r="L55" t="n">
         <x:f>IF(K55="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K55/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>343</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="M55"/>
       <x:c r="N55" t="n">
         <x:f>IF(L55="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L55+IF(M55="",0,M55))))</x:f>
-        <x:v>343</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="O55" t="str">
         <x:f>IF(N55="","",IF(N55&gt;='Instellingen'!$B$22,"Absolute top",IF(N55&gt;='Instellingen'!$B$23,"Kopman",IF(N55&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N55&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3304,12 +3304,12 @@
       </x:c>
       <x:c r="L56" t="n">
         <x:f>IF(K56="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K56/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>444</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="M56"/>
       <x:c r="N56" t="n">
         <x:f>IF(L56="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L56+IF(M56="",0,M56))))</x:f>
-        <x:v>444</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="O56" t="str">
         <x:f>IF(N56="","",IF(N56&gt;='Instellingen'!$B$22,"Absolute top",IF(N56&gt;='Instellingen'!$B$23,"Kopman",IF(N56&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N56&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3362,12 +3362,12 @@
       </x:c>
       <x:c r="L57" t="n">
         <x:f>IF(K57="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K57/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>443</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="M57"/>
       <x:c r="N57" t="n">
         <x:f>IF(L57="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L57+IF(M57="",0,M57))))</x:f>
-        <x:v>443</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="O57" t="str">
         <x:f>IF(N57="","",IF(N57&gt;='Instellingen'!$B$22,"Absolute top",IF(N57&gt;='Instellingen'!$B$23,"Kopman",IF(N57&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N57&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3420,12 +3420,12 @@
       </x:c>
       <x:c r="L58" t="n">
         <x:f>IF(K58="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K58/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>457</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="M58"/>
       <x:c r="N58" t="n">
         <x:f>IF(L58="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L58+IF(M58="",0,M58))))</x:f>
-        <x:v>457</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="O58" t="str">
         <x:f>IF(N58="","",IF(N58&gt;='Instellingen'!$B$22,"Absolute top",IF(N58&gt;='Instellingen'!$B$23,"Kopman",IF(N58&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N58&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3478,12 +3478,12 @@
       </x:c>
       <x:c r="L59" t="n">
         <x:f>IF(K59="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K59/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>327</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="M59"/>
       <x:c r="N59" t="n">
         <x:f>IF(L59="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L59+IF(M59="",0,M59))))</x:f>
-        <x:v>327</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="O59" t="str">
         <x:f>IF(N59="","",IF(N59&gt;='Instellingen'!$B$22,"Absolute top",IF(N59&gt;='Instellingen'!$B$23,"Kopman",IF(N59&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N59&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3536,12 +3536,12 @@
       </x:c>
       <x:c r="L60" t="n">
         <x:f>IF(K60="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K60/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>476</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="M60"/>
       <x:c r="N60" t="n">
         <x:f>IF(L60="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L60+IF(M60="",0,M60))))</x:f>
-        <x:v>476</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="O60" t="str">
         <x:f>IF(N60="","",IF(N60&gt;='Instellingen'!$B$22,"Absolute top",IF(N60&gt;='Instellingen'!$B$23,"Kopman",IF(N60&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N60&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3594,12 +3594,12 @@
       </x:c>
       <x:c r="L61" t="n">
         <x:f>IF(K61="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K61/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>324</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="M61"/>
       <x:c r="N61" t="n">
         <x:f>IF(L61="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L61+IF(M61="",0,M61))))</x:f>
-        <x:v>324</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="O61" t="str">
         <x:f>IF(N61="","",IF(N61&gt;='Instellingen'!$B$22,"Absolute top",IF(N61&gt;='Instellingen'!$B$23,"Kopman",IF(N61&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N61&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3652,12 +3652,12 @@
       </x:c>
       <x:c r="L62" t="n">
         <x:f>IF(K62="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K62/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>450</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="M62"/>
       <x:c r="N62" t="n">
         <x:f>IF(L62="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L62+IF(M62="",0,M62))))</x:f>
-        <x:v>450</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="O62" t="str">
         <x:f>IF(N62="","",IF(N62&gt;='Instellingen'!$B$22,"Absolute top",IF(N62&gt;='Instellingen'!$B$23,"Kopman",IF(N62&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N62&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3710,12 +3710,12 @@
       </x:c>
       <x:c r="L63" t="n">
         <x:f>IF(K63="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K63/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>443</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="M63"/>
       <x:c r="N63" t="n">
         <x:f>IF(L63="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L63+IF(M63="",0,M63))))</x:f>
-        <x:v>443</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="O63" t="str">
         <x:f>IF(N63="","",IF(N63&gt;='Instellingen'!$B$22,"Absolute top",IF(N63&gt;='Instellingen'!$B$23,"Kopman",IF(N63&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N63&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3768,12 +3768,12 @@
       </x:c>
       <x:c r="L64" t="n">
         <x:f>IF(K64="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K64/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>368</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="M64"/>
       <x:c r="N64" t="n">
         <x:f>IF(L64="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L64+IF(M64="",0,M64))))</x:f>
-        <x:v>368</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="O64" t="str">
         <x:f>IF(N64="","",IF(N64&gt;='Instellingen'!$B$22,"Absolute top",IF(N64&gt;='Instellingen'!$B$23,"Kopman",IF(N64&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N64&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3826,12 +3826,12 @@
       </x:c>
       <x:c r="L65" t="n">
         <x:f>IF(K65="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K65/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>359</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="M65"/>
       <x:c r="N65" t="n">
         <x:f>IF(L65="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L65+IF(M65="",0,M65))))</x:f>
-        <x:v>359</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="O65" t="str">
         <x:f>IF(N65="","",IF(N65&gt;='Instellingen'!$B$22,"Absolute top",IF(N65&gt;='Instellingen'!$B$23,"Kopman",IF(N65&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N65&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3884,12 +3884,12 @@
       </x:c>
       <x:c r="L66" t="n">
         <x:f>IF(K66="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K66/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>443</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="M66"/>
       <x:c r="N66" t="n">
         <x:f>IF(L66="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L66+IF(M66="",0,M66))))</x:f>
-        <x:v>443</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="O66" t="str">
         <x:f>IF(N66="","",IF(N66&gt;='Instellingen'!$B$22,"Absolute top",IF(N66&gt;='Instellingen'!$B$23,"Kopman",IF(N66&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N66&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -3942,12 +3942,12 @@
       </x:c>
       <x:c r="L67" t="n">
         <x:f>IF(K67="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K67/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>496</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="M67"/>
       <x:c r="N67" t="n">
         <x:f>IF(L67="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L67+IF(M67="",0,M67))))</x:f>
-        <x:v>496</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="O67" t="str">
         <x:f>IF(N67="","",IF(N67&gt;='Instellingen'!$B$22,"Absolute top",IF(N67&gt;='Instellingen'!$B$23,"Kopman",IF(N67&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N67&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4000,16 +4000,16 @@
       </x:c>
       <x:c r="L68" t="n">
         <x:f>IF(K68="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K68/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>1044</x:v>
+        <x:v>1720</x:v>
       </x:c>
       <x:c r="M68"/>
       <x:c r="N68" t="n">
         <x:f>IF(L68="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L68+IF(M68="",0,M68))))</x:f>
-        <x:v>1044</x:v>
+        <x:v>1720</x:v>
       </x:c>
       <x:c r="O68" t="str">
         <x:f>IF(N68="","",IF(N68&gt;='Instellingen'!$B$22,"Absolute top",IF(N68&gt;='Instellingen'!$B$23,"Kopman",IF(N68&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N68&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Kopman</x:v>
       </x:c>
       <x:c r="P68" t="str">
         <x:f>IF(A68="","",IF(D68="","Rol invullen","Compleet"))</x:f>
@@ -4058,16 +4058,16 @@
       </x:c>
       <x:c r="L69" t="n">
         <x:f>IF(K69="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K69/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>657</x:v>
+        <x:v>981</x:v>
       </x:c>
       <x:c r="M69"/>
       <x:c r="N69" t="n">
         <x:f>IF(L69="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L69+IF(M69="",0,M69))))</x:f>
-        <x:v>657</x:v>
+        <x:v>981</x:v>
       </x:c>
       <x:c r="O69" t="str">
         <x:f>IF(N69="","",IF(N69&gt;='Instellingen'!$B$22,"Absolute top",IF(N69&gt;='Instellingen'!$B$23,"Kopman",IF(N69&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N69&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P69" t="str">
         <x:f>IF(A69="","",IF(D69="","Rol invullen","Compleet"))</x:f>
@@ -4116,16 +4116,16 @@
       </x:c>
       <x:c r="L70" t="n">
         <x:f>IF(K70="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K70/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>515</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="M70"/>
       <x:c r="N70" t="n">
         <x:f>IF(L70="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L70+IF(M70="",0,M70))))</x:f>
-        <x:v>515</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="O70" t="str">
         <x:f>IF(N70="","",IF(N70&gt;='Instellingen'!$B$22,"Absolute top",IF(N70&gt;='Instellingen'!$B$23,"Kopman",IF(N70&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N70&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P70" t="str">
         <x:f>IF(A70="","",IF(D70="","Rol invullen","Compleet"))</x:f>
@@ -4174,16 +4174,16 @@
       </x:c>
       <x:c r="L71" t="n">
         <x:f>IF(K71="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K71/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>649</x:v>
+        <x:v>965</x:v>
       </x:c>
       <x:c r="M71"/>
       <x:c r="N71" t="n">
         <x:f>IF(L71="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L71+IF(M71="",0,M71))))</x:f>
-        <x:v>649</x:v>
+        <x:v>965</x:v>
       </x:c>
       <x:c r="O71" t="str">
         <x:f>IF(N71="","",IF(N71&gt;='Instellingen'!$B$22,"Absolute top",IF(N71&gt;='Instellingen'!$B$23,"Kopman",IF(N71&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N71&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P71" t="str">
         <x:f>IF(A71="","",IF(D71="","Rol invullen","Compleet"))</x:f>
@@ -4232,16 +4232,16 @@
       </x:c>
       <x:c r="L72" t="n">
         <x:f>IF(K72="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K72/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>955</x:v>
+        <x:v>1551</x:v>
       </x:c>
       <x:c r="M72"/>
       <x:c r="N72" t="n">
         <x:f>IF(L72="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L72+IF(M72="",0,M72))))</x:f>
-        <x:v>955</x:v>
+        <x:v>1551</x:v>
       </x:c>
       <x:c r="O72" t="str">
         <x:f>IF(N72="","",IF(N72&gt;='Instellingen'!$B$22,"Absolute top",IF(N72&gt;='Instellingen'!$B$23,"Kopman",IF(N72&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N72&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P72" t="str">
         <x:f>IF(A72="","",IF(D72="","Rol invullen","Compleet"))</x:f>
@@ -4290,16 +4290,16 @@
       </x:c>
       <x:c r="L73" t="n">
         <x:f>IF(K73="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K73/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>777</x:v>
+        <x:v>1211</x:v>
       </x:c>
       <x:c r="M73"/>
       <x:c r="N73" t="n">
         <x:f>IF(L73="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L73+IF(M73="",0,M73))))</x:f>
-        <x:v>777</x:v>
+        <x:v>1211</x:v>
       </x:c>
       <x:c r="O73" t="str">
         <x:f>IF(N73="","",IF(N73&gt;='Instellingen'!$B$22,"Absolute top",IF(N73&gt;='Instellingen'!$B$23,"Kopman",IF(N73&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N73&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P73" t="str">
         <x:f>IF(A73="","",IF(D73="","Rol invullen","Compleet"))</x:f>
@@ -4348,16 +4348,16 @@
       </x:c>
       <x:c r="L74" t="n">
         <x:f>IF(K74="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K74/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>2066</x:v>
+        <x:v>3671</x:v>
       </x:c>
       <x:c r="M74"/>
       <x:c r="N74" t="n">
         <x:f>IF(L74="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L74+IF(M74="",0,M74))))</x:f>
-        <x:v>2066</x:v>
+        <x:v>3671</x:v>
       </x:c>
       <x:c r="O74" t="str">
         <x:f>IF(N74="","",IF(N74&gt;='Instellingen'!$B$22,"Absolute top",IF(N74&gt;='Instellingen'!$B$23,"Kopman",IF(N74&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N74&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Kopman</x:v>
+        <x:v>Absolute top</x:v>
       </x:c>
       <x:c r="P74" t="str">
         <x:f>IF(A74="","",IF(D74="","Rol invullen","Compleet"))</x:f>
@@ -4406,16 +4406,16 @@
       </x:c>
       <x:c r="L75" t="n">
         <x:f>IF(K75="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K75/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>1096</x:v>
+        <x:v>1819</x:v>
       </x:c>
       <x:c r="M75"/>
       <x:c r="N75" t="n">
         <x:f>IF(L75="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L75+IF(M75="",0,M75))))</x:f>
-        <x:v>1096</x:v>
+        <x:v>1819</x:v>
       </x:c>
       <x:c r="O75" t="str">
         <x:f>IF(N75="","",IF(N75&gt;='Instellingen'!$B$22,"Absolute top",IF(N75&gt;='Instellingen'!$B$23,"Kopman",IF(N75&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N75&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Kopman</x:v>
       </x:c>
       <x:c r="P75" t="str">
         <x:f>IF(A75="","",IF(D75="","Rol invullen","Compleet"))</x:f>
@@ -4464,16 +4464,16 @@
       </x:c>
       <x:c r="L76" t="n">
         <x:f>IF(K76="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K76/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>527</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="M76"/>
       <x:c r="N76" t="n">
         <x:f>IF(L76="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L76+IF(M76="",0,M76))))</x:f>
-        <x:v>527</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="O76" t="str">
         <x:f>IF(N76="","",IF(N76&gt;='Instellingen'!$B$22,"Absolute top",IF(N76&gt;='Instellingen'!$B$23,"Kopman",IF(N76&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N76&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P76" t="str">
         <x:f>IF(A76="","",IF(D76="","Rol invullen","Compleet"))</x:f>
@@ -4522,16 +4522,16 @@
       </x:c>
       <x:c r="L77" t="n">
         <x:f>IF(K77="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K77/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>769</x:v>
+        <x:v>1195</x:v>
       </x:c>
       <x:c r="M77"/>
       <x:c r="N77" t="n">
         <x:f>IF(L77="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L77+IF(M77="",0,M77))))</x:f>
-        <x:v>769</x:v>
+        <x:v>1195</x:v>
       </x:c>
       <x:c r="O77" t="str">
         <x:f>IF(N77="","",IF(N77&gt;='Instellingen'!$B$22,"Absolute top",IF(N77&gt;='Instellingen'!$B$23,"Kopman",IF(N77&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N77&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P77" t="str">
         <x:f>IF(A77="","",IF(D77="","Rol invullen","Compleet"))</x:f>
@@ -4580,12 +4580,12 @@
       </x:c>
       <x:c r="L78" t="n">
         <x:f>IF(K78="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K78/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>477</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="M78"/>
       <x:c r="N78" t="n">
         <x:f>IF(L78="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L78+IF(M78="",0,M78))))</x:f>
-        <x:v>477</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="O78" t="str">
         <x:f>IF(N78="","",IF(N78&gt;='Instellingen'!$B$22,"Absolute top",IF(N78&gt;='Instellingen'!$B$23,"Kopman",IF(N78&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N78&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4638,12 +4638,12 @@
       </x:c>
       <x:c r="L79" t="n">
         <x:f>IF(K79="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K79/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>459</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="M79"/>
       <x:c r="N79" t="n">
         <x:f>IF(L79="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L79+IF(M79="",0,M79))))</x:f>
-        <x:v>459</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="O79" t="str">
         <x:f>IF(N79="","",IF(N79&gt;='Instellingen'!$B$22,"Absolute top",IF(N79&gt;='Instellingen'!$B$23,"Kopman",IF(N79&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N79&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4696,12 +4696,12 @@
       </x:c>
       <x:c r="L80" t="n">
         <x:f>IF(K80="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K80/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>406</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="M80"/>
       <x:c r="N80" t="n">
         <x:f>IF(L80="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L80+IF(M80="",0,M80))))</x:f>
-        <x:v>406</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="O80" t="str">
         <x:f>IF(N80="","",IF(N80&gt;='Instellingen'!$B$22,"Absolute top",IF(N80&gt;='Instellingen'!$B$23,"Kopman",IF(N80&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N80&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4754,12 +4754,12 @@
       </x:c>
       <x:c r="L81" t="n">
         <x:f>IF(K81="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K81/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>363</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="M81"/>
       <x:c r="N81" t="n">
         <x:f>IF(L81="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L81+IF(M81="",0,M81))))</x:f>
-        <x:v>363</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="O81" t="str">
         <x:f>IF(N81="","",IF(N81&gt;='Instellingen'!$B$22,"Absolute top",IF(N81&gt;='Instellingen'!$B$23,"Kopman",IF(N81&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N81&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4812,12 +4812,12 @@
       </x:c>
       <x:c r="L82" t="n">
         <x:f>IF(K82="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K82/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>701</x:v>
+        <x:v>1065</x:v>
       </x:c>
       <x:c r="M82"/>
       <x:c r="N82" t="n">
         <x:f>IF(L82="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L82+IF(M82="",0,M82))))</x:f>
-        <x:v>701</x:v>
+        <x:v>1065</x:v>
       </x:c>
       <x:c r="O82" t="str">
         <x:f>IF(N82="","",IF(N82&gt;='Instellingen'!$B$22,"Absolute top",IF(N82&gt;='Instellingen'!$B$23,"Kopman",IF(N82&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N82&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4870,12 +4870,12 @@
       </x:c>
       <x:c r="L83" t="n">
         <x:f>IF(K83="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K83/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>456</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="M83"/>
       <x:c r="N83" t="n">
         <x:f>IF(L83="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L83+IF(M83="",0,M83))))</x:f>
-        <x:v>456</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="O83" t="str">
         <x:f>IF(N83="","",IF(N83&gt;='Instellingen'!$B$22,"Absolute top",IF(N83&gt;='Instellingen'!$B$23,"Kopman",IF(N83&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N83&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4928,12 +4928,12 @@
       </x:c>
       <x:c r="L84" t="n">
         <x:f>IF(K84="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K84/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>485</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="M84"/>
       <x:c r="N84" t="n">
         <x:f>IF(L84="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L84+IF(M84="",0,M84))))</x:f>
-        <x:v>485</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="O84" t="str">
         <x:f>IF(N84="","",IF(N84&gt;='Instellingen'!$B$22,"Absolute top",IF(N84&gt;='Instellingen'!$B$23,"Kopman",IF(N84&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N84&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -4986,12 +4986,12 @@
       </x:c>
       <x:c r="L85" t="n">
         <x:f>IF(K85="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K85/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>421</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="M85"/>
       <x:c r="N85" t="n">
         <x:f>IF(L85="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L85+IF(M85="",0,M85))))</x:f>
-        <x:v>421</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="O85" t="str">
         <x:f>IF(N85="","",IF(N85&gt;='Instellingen'!$B$22,"Absolute top",IF(N85&gt;='Instellingen'!$B$23,"Kopman",IF(N85&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N85&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5044,12 +5044,12 @@
       </x:c>
       <x:c r="L86" t="n">
         <x:f>IF(K86="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K86/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>496</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="M86"/>
       <x:c r="N86" t="n">
         <x:f>IF(L86="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L86+IF(M86="",0,M86))))</x:f>
-        <x:v>496</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="O86" t="str">
         <x:f>IF(N86="","",IF(N86&gt;='Instellingen'!$B$22,"Absolute top",IF(N86&gt;='Instellingen'!$B$23,"Kopman",IF(N86&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N86&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5102,12 +5102,12 @@
       </x:c>
       <x:c r="L87" t="n">
         <x:f>IF(K87="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K87/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>481</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="M87"/>
       <x:c r="N87" t="n">
         <x:f>IF(L87="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L87+IF(M87="",0,M87))))</x:f>
-        <x:v>481</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="O87" t="str">
         <x:f>IF(N87="","",IF(N87&gt;='Instellingen'!$B$22,"Absolute top",IF(N87&gt;='Instellingen'!$B$23,"Kopman",IF(N87&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N87&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5160,16 +5160,16 @@
       </x:c>
       <x:c r="L88" t="n">
         <x:f>IF(K88="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K88/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>543</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="M88"/>
       <x:c r="N88" t="n">
         <x:f>IF(L88="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L88+IF(M88="",0,M88))))</x:f>
-        <x:v>543</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="O88" t="str">
         <x:f>IF(N88="","",IF(N88&gt;='Instellingen'!$B$22,"Absolute top",IF(N88&gt;='Instellingen'!$B$23,"Kopman",IF(N88&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N88&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P88" t="str">
         <x:f>IF(A88="","",IF(D88="","Rol invullen","Compleet"))</x:f>
@@ -5218,16 +5218,16 @@
       </x:c>
       <x:c r="L89" t="n">
         <x:f>IF(K89="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K89/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>565</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="M89"/>
       <x:c r="N89" t="n">
         <x:f>IF(L89="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L89+IF(M89="",0,M89))))</x:f>
-        <x:v>565</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="O89" t="str">
         <x:f>IF(N89="","",IF(N89&gt;='Instellingen'!$B$22,"Absolute top",IF(N89&gt;='Instellingen'!$B$23,"Kopman",IF(N89&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N89&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P89" t="str">
         <x:f>IF(A89="","",IF(D89="","Rol invullen","Compleet"))</x:f>
@@ -5276,12 +5276,12 @@
       </x:c>
       <x:c r="L90" t="n">
         <x:f>IF(K90="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K90/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>364</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="M90"/>
       <x:c r="N90" t="n">
         <x:f>IF(L90="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L90+IF(M90="",0,M90))))</x:f>
-        <x:v>364</x:v>
+        <x:v>421</x:v>
       </x:c>
       <x:c r="O90" t="str">
         <x:f>IF(N90="","",IF(N90&gt;='Instellingen'!$B$22,"Absolute top",IF(N90&gt;='Instellingen'!$B$23,"Kopman",IF(N90&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N90&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5334,12 +5334,12 @@
       </x:c>
       <x:c r="L91" t="n">
         <x:f>IF(K91="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K91/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>450</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="M91"/>
       <x:c r="N91" t="n">
         <x:f>IF(L91="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L91+IF(M91="",0,M91))))</x:f>
-        <x:v>450</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="O91" t="str">
         <x:f>IF(N91="","",IF(N91&gt;='Instellingen'!$B$22,"Absolute top",IF(N91&gt;='Instellingen'!$B$23,"Kopman",IF(N91&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N91&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5392,12 +5392,12 @@
       </x:c>
       <x:c r="L92" t="n">
         <x:f>IF(K92="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K92/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>481</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="M92"/>
       <x:c r="N92" t="n">
         <x:f>IF(L92="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L92+IF(M92="",0,M92))))</x:f>
-        <x:v>481</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="O92" t="str">
         <x:f>IF(N92="","",IF(N92&gt;='Instellingen'!$B$22,"Absolute top",IF(N92&gt;='Instellingen'!$B$23,"Kopman",IF(N92&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N92&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5450,12 +5450,12 @@
       </x:c>
       <x:c r="L93" t="n">
         <x:f>IF(K93="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K93/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>479</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="M93"/>
       <x:c r="N93" t="n">
         <x:f>IF(L93="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L93+IF(M93="",0,M93))))</x:f>
-        <x:v>479</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="O93" t="str">
         <x:f>IF(N93="","",IF(N93&gt;='Instellingen'!$B$22,"Absolute top",IF(N93&gt;='Instellingen'!$B$23,"Kopman",IF(N93&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N93&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5508,16 +5508,16 @@
       </x:c>
       <x:c r="L94" t="n">
         <x:f>IF(K94="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K94/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>603</x:v>
+        <x:v>878</x:v>
       </x:c>
       <x:c r="M94"/>
       <x:c r="N94" t="n">
         <x:f>IF(L94="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L94+IF(M94="",0,M94))))</x:f>
-        <x:v>603</x:v>
+        <x:v>878</x:v>
       </x:c>
       <x:c r="O94" t="str">
         <x:f>IF(N94="","",IF(N94&gt;='Instellingen'!$B$22,"Absolute top",IF(N94&gt;='Instellingen'!$B$23,"Kopman",IF(N94&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N94&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P94" t="str">
         <x:f>IF(A94="","",IF(D94="","Rol invullen","Compleet"))</x:f>
@@ -5566,16 +5566,16 @@
       </x:c>
       <x:c r="L95" t="n">
         <x:f>IF(K95="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K95/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>776</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="M95"/>
       <x:c r="N95" t="n">
         <x:f>IF(L95="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L95+IF(M95="",0,M95))))</x:f>
-        <x:v>776</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="O95" t="str">
         <x:f>IF(N95="","",IF(N95&gt;='Instellingen'!$B$22,"Absolute top",IF(N95&gt;='Instellingen'!$B$23,"Kopman",IF(N95&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N95&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P95" t="str">
         <x:f>IF(A95="","",IF(D95="","Rol invullen","Compleet"))</x:f>
@@ -5624,16 +5624,16 @@
       </x:c>
       <x:c r="L96" t="n">
         <x:f>IF(K96="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K96/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>800</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="M96"/>
       <x:c r="N96" t="n">
         <x:f>IF(L96="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L96+IF(M96="",0,M96))))</x:f>
-        <x:v>800</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="O96" t="str">
         <x:f>IF(N96="","",IF(N96&gt;='Instellingen'!$B$22,"Absolute top",IF(N96&gt;='Instellingen'!$B$23,"Kopman",IF(N96&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N96&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P96" t="str">
         <x:f>IF(A96="","",IF(D96="","Rol invullen","Compleet"))</x:f>
@@ -5682,16 +5682,16 @@
       </x:c>
       <x:c r="L97" t="n">
         <x:f>IF(K97="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K97/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>824</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="M97"/>
       <x:c r="N97" t="n">
         <x:f>IF(L97="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L97+IF(M97="",0,M97))))</x:f>
-        <x:v>824</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="O97" t="str">
         <x:f>IF(N97="","",IF(N97&gt;='Instellingen'!$B$22,"Absolute top",IF(N97&gt;='Instellingen'!$B$23,"Kopman",IF(N97&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N97&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P97" t="str">
         <x:f>IF(A97="","",IF(D97="","Rol invullen","Compleet"))</x:f>
@@ -5740,12 +5740,12 @@
       </x:c>
       <x:c r="L98" t="n">
         <x:f>IF(K98="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K98/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>488</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="M98"/>
       <x:c r="N98" t="n">
         <x:f>IF(L98="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L98+IF(M98="",0,M98))))</x:f>
-        <x:v>488</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="O98" t="str">
         <x:f>IF(N98="","",IF(N98&gt;='Instellingen'!$B$22,"Absolute top",IF(N98&gt;='Instellingen'!$B$23,"Kopman",IF(N98&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N98&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5798,12 +5798,12 @@
       </x:c>
       <x:c r="L99" t="n">
         <x:f>IF(K99="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K99/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>497</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="M99"/>
       <x:c r="N99" t="n">
         <x:f>IF(L99="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L99+IF(M99="",0,M99))))</x:f>
-        <x:v>497</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="O99" t="str">
         <x:f>IF(N99="","",IF(N99&gt;='Instellingen'!$B$22,"Absolute top",IF(N99&gt;='Instellingen'!$B$23,"Kopman",IF(N99&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N99&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5856,12 +5856,12 @@
       </x:c>
       <x:c r="L100" t="n">
         <x:f>IF(K100="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K100/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>435</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="M100"/>
       <x:c r="N100" t="n">
         <x:f>IF(L100="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L100+IF(M100="",0,M100))))</x:f>
-        <x:v>435</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="O100" t="str">
         <x:f>IF(N100="","",IF(N100&gt;='Instellingen'!$B$22,"Absolute top",IF(N100&gt;='Instellingen'!$B$23,"Kopman",IF(N100&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N100&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5914,12 +5914,12 @@
       </x:c>
       <x:c r="L101" t="n">
         <x:f>IF(K101="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K101/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>350</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="M101"/>
       <x:c r="N101" t="n">
         <x:f>IF(L101="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L101+IF(M101="",0,M101))))</x:f>
-        <x:v>350</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="O101" t="str">
         <x:f>IF(N101="","",IF(N101&gt;='Instellingen'!$B$22,"Absolute top",IF(N101&gt;='Instellingen'!$B$23,"Kopman",IF(N101&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N101&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -5972,12 +5972,12 @@
       </x:c>
       <x:c r="L102" t="n">
         <x:f>IF(K102="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K102/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>477</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="M102"/>
       <x:c r="N102" t="n">
         <x:f>IF(L102="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L102+IF(M102="",0,M102))))</x:f>
-        <x:v>477</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="O102" t="str">
         <x:f>IF(N102="","",IF(N102&gt;='Instellingen'!$B$22,"Absolute top",IF(N102&gt;='Instellingen'!$B$23,"Kopman",IF(N102&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N102&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6030,12 +6030,12 @@
       </x:c>
       <x:c r="L103" t="n">
         <x:f>IF(K103="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K103/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>354</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="M103"/>
       <x:c r="N103" t="n">
         <x:f>IF(L103="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L103+IF(M103="",0,M103))))</x:f>
-        <x:v>354</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="O103" t="str">
         <x:f>IF(N103="","",IF(N103&gt;='Instellingen'!$B$22,"Absolute top",IF(N103&gt;='Instellingen'!$B$23,"Kopman",IF(N103&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N103&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6088,12 +6088,12 @@
       </x:c>
       <x:c r="L104" t="n">
         <x:f>IF(K104="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K104/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>354</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="M104"/>
       <x:c r="N104" t="n">
         <x:f>IF(L104="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L104+IF(M104="",0,M104))))</x:f>
-        <x:v>354</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="O104" t="str">
         <x:f>IF(N104="","",IF(N104&gt;='Instellingen'!$B$22,"Absolute top",IF(N104&gt;='Instellingen'!$B$23,"Kopman",IF(N104&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N104&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6146,16 +6146,16 @@
       </x:c>
       <x:c r="L105" t="n">
         <x:f>IF(K105="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K105/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>771</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="M105"/>
       <x:c r="N105" t="n">
         <x:f>IF(L105="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L105+IF(M105="",0,M105))))</x:f>
-        <x:v>771</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="O105" t="str">
         <x:f>IF(N105="","",IF(N105&gt;='Instellingen'!$B$22,"Absolute top",IF(N105&gt;='Instellingen'!$B$23,"Kopman",IF(N105&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N105&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P105" t="str">
         <x:f>IF(A105="","",IF(D105="","Rol invullen","Compleet"))</x:f>
@@ -6204,12 +6204,12 @@
       </x:c>
       <x:c r="L106" t="n">
         <x:f>IF(K106="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K106/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>485</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="M106"/>
       <x:c r="N106" t="n">
         <x:f>IF(L106="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L106+IF(M106="",0,M106))))</x:f>
-        <x:v>485</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="O106" t="str">
         <x:f>IF(N106="","",IF(N106&gt;='Instellingen'!$B$22,"Absolute top",IF(N106&gt;='Instellingen'!$B$23,"Kopman",IF(N106&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N106&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6262,12 +6262,12 @@
       </x:c>
       <x:c r="L107" t="n">
         <x:f>IF(K107="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K107/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>474</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="M107"/>
       <x:c r="N107" t="n">
         <x:f>IF(L107="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L107+IF(M107="",0,M107))))</x:f>
-        <x:v>474</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="O107" t="str">
         <x:f>IF(N107="","",IF(N107&gt;='Instellingen'!$B$22,"Absolute top",IF(N107&gt;='Instellingen'!$B$23,"Kopman",IF(N107&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N107&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6320,12 +6320,12 @@
       </x:c>
       <x:c r="L108" t="n">
         <x:f>IF(K108="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K108/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>443</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="M108"/>
       <x:c r="N108" t="n">
         <x:f>IF(L108="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L108+IF(M108="",0,M108))))</x:f>
-        <x:v>443</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="O108" t="str">
         <x:f>IF(N108="","",IF(N108&gt;='Instellingen'!$B$22,"Absolute top",IF(N108&gt;='Instellingen'!$B$23,"Kopman",IF(N108&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N108&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6378,12 +6378,12 @@
       </x:c>
       <x:c r="L109" t="n">
         <x:f>IF(K109="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K109/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>351</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="M109"/>
       <x:c r="N109" t="n">
         <x:f>IF(L109="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L109+IF(M109="",0,M109))))</x:f>
-        <x:v>351</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="O109" t="str">
         <x:f>IF(N109="","",IF(N109&gt;='Instellingen'!$B$22,"Absolute top",IF(N109&gt;='Instellingen'!$B$23,"Kopman",IF(N109&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N109&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6436,12 +6436,12 @@
       </x:c>
       <x:c r="L110" t="n">
         <x:f>IF(K110="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K110/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>323</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="M110"/>
       <x:c r="N110" t="n">
         <x:f>IF(L110="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L110+IF(M110="",0,M110))))</x:f>
-        <x:v>323</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="O110" t="str">
         <x:f>IF(N110="","",IF(N110&gt;='Instellingen'!$B$22,"Absolute top",IF(N110&gt;='Instellingen'!$B$23,"Kopman",IF(N110&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N110&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6494,12 +6494,12 @@
       </x:c>
       <x:c r="L111" t="n">
         <x:f>IF(K111="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K111/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>354</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="M111"/>
       <x:c r="N111" t="n">
         <x:f>IF(L111="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L111+IF(M111="",0,M111))))</x:f>
-        <x:v>354</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="O111" t="str">
         <x:f>IF(N111="","",IF(N111&gt;='Instellingen'!$B$22,"Absolute top",IF(N111&gt;='Instellingen'!$B$23,"Kopman",IF(N111&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N111&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6552,12 +6552,12 @@
       </x:c>
       <x:c r="L112" t="n">
         <x:f>IF(K112="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K112/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>321</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="M112"/>
       <x:c r="N112" t="n">
         <x:f>IF(L112="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L112+IF(M112="",0,M112))))</x:f>
-        <x:v>321</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="O112" t="str">
         <x:f>IF(N112="","",IF(N112&gt;='Instellingen'!$B$22,"Absolute top",IF(N112&gt;='Instellingen'!$B$23,"Kopman",IF(N112&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N112&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6610,12 +6610,12 @@
       </x:c>
       <x:c r="L113" t="n">
         <x:f>IF(K113="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K113/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>347</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="M113"/>
       <x:c r="N113" t="n">
         <x:f>IF(L113="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L113+IF(M113="",0,M113))))</x:f>
-        <x:v>347</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="O113" t="str">
         <x:f>IF(N113="","",IF(N113&gt;='Instellingen'!$B$22,"Absolute top",IF(N113&gt;='Instellingen'!$B$23,"Kopman",IF(N113&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N113&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6668,16 +6668,16 @@
       </x:c>
       <x:c r="L114" t="n">
         <x:f>IF(K114="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K114/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>513</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="M114"/>
       <x:c r="N114" t="n">
         <x:f>IF(L114="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L114+IF(M114="",0,M114))))</x:f>
-        <x:v>513</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="O114" t="str">
         <x:f>IF(N114="","",IF(N114&gt;='Instellingen'!$B$22,"Absolute top",IF(N114&gt;='Instellingen'!$B$23,"Kopman",IF(N114&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N114&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P114" t="str">
         <x:f>IF(A114="","",IF(D114="","Rol invullen","Compleet"))</x:f>
@@ -6726,12 +6726,12 @@
       </x:c>
       <x:c r="L115" t="n">
         <x:f>IF(K115="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K115/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>353</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="M115"/>
       <x:c r="N115" t="n">
         <x:f>IF(L115="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L115+IF(M115="",0,M115))))</x:f>
-        <x:v>353</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="O115" t="str">
         <x:f>IF(N115="","",IF(N115&gt;='Instellingen'!$B$22,"Absolute top",IF(N115&gt;='Instellingen'!$B$23,"Kopman",IF(N115&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N115&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6784,12 +6784,12 @@
       </x:c>
       <x:c r="L116" t="n">
         <x:f>IF(K116="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K116/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>370</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="M116"/>
       <x:c r="N116" t="n">
         <x:f>IF(L116="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L116+IF(M116="",0,M116))))</x:f>
-        <x:v>370</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="O116" t="str">
         <x:f>IF(N116="","",IF(N116&gt;='Instellingen'!$B$22,"Absolute top",IF(N116&gt;='Instellingen'!$B$23,"Kopman",IF(N116&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N116&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6842,12 +6842,12 @@
       </x:c>
       <x:c r="L117" t="n">
         <x:f>IF(K117="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K117/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>370</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="M117"/>
       <x:c r="N117" t="n">
         <x:f>IF(L117="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L117+IF(M117="",0,M117))))</x:f>
-        <x:v>370</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="O117" t="str">
         <x:f>IF(N117="","",IF(N117&gt;='Instellingen'!$B$22,"Absolute top",IF(N117&gt;='Instellingen'!$B$23,"Kopman",IF(N117&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N117&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6900,12 +6900,12 @@
       </x:c>
       <x:c r="L118" t="n">
         <x:f>IF(K118="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K118/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>323</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="M118"/>
       <x:c r="N118" t="n">
         <x:f>IF(L118="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L118+IF(M118="",0,M118))))</x:f>
-        <x:v>323</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="O118" t="str">
         <x:f>IF(N118="","",IF(N118&gt;='Instellingen'!$B$22,"Absolute top",IF(N118&gt;='Instellingen'!$B$23,"Kopman",IF(N118&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N118&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -6958,12 +6958,12 @@
       </x:c>
       <x:c r="L119" t="n">
         <x:f>IF(K119="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K119/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>355</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="M119"/>
       <x:c r="N119" t="n">
         <x:f>IF(L119="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L119+IF(M119="",0,M119))))</x:f>
-        <x:v>355</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="O119" t="str">
         <x:f>IF(N119="","",IF(N119&gt;='Instellingen'!$B$22,"Absolute top",IF(N119&gt;='Instellingen'!$B$23,"Kopman",IF(N119&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N119&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7016,16 +7016,16 @@
       </x:c>
       <x:c r="L120" t="n">
         <x:f>IF(K120="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K120/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>539</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="M120"/>
       <x:c r="N120" t="n">
         <x:f>IF(L120="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L120+IF(M120="",0,M120))))</x:f>
-        <x:v>539</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="O120" t="str">
         <x:f>IF(N120="","",IF(N120&gt;='Instellingen'!$B$22,"Absolute top",IF(N120&gt;='Instellingen'!$B$23,"Kopman",IF(N120&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N120&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P120" t="str">
         <x:f>IF(A120="","",IF(D120="","Rol invullen","Compleet"))</x:f>
@@ -7074,12 +7074,12 @@
       </x:c>
       <x:c r="L121" t="n">
         <x:f>IF(K121="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K121/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>446</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="M121"/>
       <x:c r="N121" t="n">
         <x:f>IF(L121="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L121+IF(M121="",0,M121))))</x:f>
-        <x:v>446</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="O121" t="str">
         <x:f>IF(N121="","",IF(N121&gt;='Instellingen'!$B$22,"Absolute top",IF(N121&gt;='Instellingen'!$B$23,"Kopman",IF(N121&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N121&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7132,12 +7132,12 @@
       </x:c>
       <x:c r="L122" t="n">
         <x:f>IF(K122="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K122/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>484</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="M122"/>
       <x:c r="N122" t="n">
         <x:f>IF(L122="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L122+IF(M122="",0,M122))))</x:f>
-        <x:v>484</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="O122" t="str">
         <x:f>IF(N122="","",IF(N122&gt;='Instellingen'!$B$22,"Absolute top",IF(N122&gt;='Instellingen'!$B$23,"Kopman",IF(N122&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N122&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7190,12 +7190,12 @@
       </x:c>
       <x:c r="L123" t="n">
         <x:f>IF(K123="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K123/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>483</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="M123"/>
       <x:c r="N123" t="n">
         <x:f>IF(L123="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L123+IF(M123="",0,M123))))</x:f>
-        <x:v>483</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="O123" t="str">
         <x:f>IF(N123="","",IF(N123&gt;='Instellingen'!$B$22,"Absolute top",IF(N123&gt;='Instellingen'!$B$23,"Kopman",IF(N123&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N123&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7248,12 +7248,12 @@
       </x:c>
       <x:c r="L124" t="n">
         <x:f>IF(K124="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K124/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>509</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="M124"/>
       <x:c r="N124" t="n">
         <x:f>IF(L124="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L124+IF(M124="",0,M124))))</x:f>
-        <x:v>509</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="O124" t="str">
         <x:f>IF(N124="","",IF(N124&gt;='Instellingen'!$B$22,"Absolute top",IF(N124&gt;='Instellingen'!$B$23,"Kopman",IF(N124&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N124&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7306,12 +7306,12 @@
       </x:c>
       <x:c r="L125" t="n">
         <x:f>IF(K125="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K125/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>405</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="M125"/>
       <x:c r="N125" t="n">
         <x:f>IF(L125="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L125+IF(M125="",0,M125))))</x:f>
-        <x:v>405</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="O125" t="str">
         <x:f>IF(N125="","",IF(N125&gt;='Instellingen'!$B$22,"Absolute top",IF(N125&gt;='Instellingen'!$B$23,"Kopman",IF(N125&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N125&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7364,16 +7364,16 @@
       </x:c>
       <x:c r="L126" t="n">
         <x:f>IF(K126="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K126/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>528</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="M126"/>
       <x:c r="N126" t="n">
         <x:f>IF(L126="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L126+IF(M126="",0,M126))))</x:f>
-        <x:v>528</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="O126" t="str">
         <x:f>IF(N126="","",IF(N126&gt;='Instellingen'!$B$22,"Absolute top",IF(N126&gt;='Instellingen'!$B$23,"Kopman",IF(N126&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N126&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P126" t="str">
         <x:f>IF(A126="","",IF(D126="","Rol invullen","Compleet"))</x:f>
@@ -7422,12 +7422,12 @@
       </x:c>
       <x:c r="L127" t="n">
         <x:f>IF(K127="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K127/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>509</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="M127"/>
       <x:c r="N127" t="n">
         <x:f>IF(L127="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L127+IF(M127="",0,M127))))</x:f>
-        <x:v>509</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="O127" t="str">
         <x:f>IF(N127="","",IF(N127&gt;='Instellingen'!$B$22,"Absolute top",IF(N127&gt;='Instellingen'!$B$23,"Kopman",IF(N127&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N127&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7480,12 +7480,12 @@
       </x:c>
       <x:c r="L128" t="n">
         <x:f>IF(K128="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K128/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>339</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="M128"/>
       <x:c r="N128" t="n">
         <x:f>IF(L128="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L128+IF(M128="",0,M128))))</x:f>
-        <x:v>339</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="O128" t="str">
         <x:f>IF(N128="","",IF(N128&gt;='Instellingen'!$B$22,"Absolute top",IF(N128&gt;='Instellingen'!$B$23,"Kopman",IF(N128&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N128&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7538,12 +7538,12 @@
       </x:c>
       <x:c r="L129" t="n">
         <x:f>IF(K129="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K129/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>445</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="M129"/>
       <x:c r="N129" t="n">
         <x:f>IF(L129="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L129+IF(M129="",0,M129))))</x:f>
-        <x:v>445</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="O129" t="str">
         <x:f>IF(N129="","",IF(N129&gt;='Instellingen'!$B$22,"Absolute top",IF(N129&gt;='Instellingen'!$B$23,"Kopman",IF(N129&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N129&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7596,12 +7596,12 @@
       </x:c>
       <x:c r="L130" t="n">
         <x:f>IF(K130="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K130/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>345</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="M130"/>
       <x:c r="N130" t="n">
         <x:f>IF(L130="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L130+IF(M130="",0,M130))))</x:f>
-        <x:v>345</x:v>
+        <x:v>387</x:v>
       </x:c>
       <x:c r="O130" t="str">
         <x:f>IF(N130="","",IF(N130&gt;='Instellingen'!$B$22,"Absolute top",IF(N130&gt;='Instellingen'!$B$23,"Kopman",IF(N130&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N130&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7654,12 +7654,12 @@
       </x:c>
       <x:c r="L131" t="n">
         <x:f>IF(K131="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K131/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>476</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="M131"/>
       <x:c r="N131" t="n">
         <x:f>IF(L131="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L131+IF(M131="",0,M131))))</x:f>
-        <x:v>476</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="O131" t="str">
         <x:f>IF(N131="","",IF(N131&gt;='Instellingen'!$B$22,"Absolute top",IF(N131&gt;='Instellingen'!$B$23,"Kopman",IF(N131&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N131&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7712,12 +7712,12 @@
       </x:c>
       <x:c r="L132" t="n">
         <x:f>IF(K132="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K132/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>496</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="M132"/>
       <x:c r="N132" t="n">
         <x:f>IF(L132="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L132+IF(M132="",0,M132))))</x:f>
-        <x:v>496</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="O132" t="str">
         <x:f>IF(N132="","",IF(N132&gt;='Instellingen'!$B$22,"Absolute top",IF(N132&gt;='Instellingen'!$B$23,"Kopman",IF(N132&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N132&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7770,12 +7770,12 @@
       </x:c>
       <x:c r="L133" t="n">
         <x:f>IF(K133="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K133/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>362</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="M133"/>
       <x:c r="N133" t="n">
         <x:f>IF(L133="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L133+IF(M133="",0,M133))))</x:f>
-        <x:v>362</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="O133" t="str">
         <x:f>IF(N133="","",IF(N133&gt;='Instellingen'!$B$22,"Absolute top",IF(N133&gt;='Instellingen'!$B$23,"Kopman",IF(N133&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N133&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7828,16 +7828,16 @@
       </x:c>
       <x:c r="L134" t="n">
         <x:f>IF(K134="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K134/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>527</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="M134"/>
       <x:c r="N134" t="n">
         <x:f>IF(L134="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L134+IF(M134="",0,M134))))</x:f>
-        <x:v>527</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="O134" t="str">
         <x:f>IF(N134="","",IF(N134&gt;='Instellingen'!$B$22,"Absolute top",IF(N134&gt;='Instellingen'!$B$23,"Kopman",IF(N134&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N134&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P134" t="str">
         <x:f>IF(A134="","",IF(D134="","Rol invullen","Compleet"))</x:f>
@@ -7886,12 +7886,12 @@
       </x:c>
       <x:c r="L135" t="n">
         <x:f>IF(K135="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K135/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>489</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="M135"/>
       <x:c r="N135" t="n">
         <x:f>IF(L135="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L135+IF(M135="",0,M135))))</x:f>
-        <x:v>489</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="O135" t="str">
         <x:f>IF(N135="","",IF(N135&gt;='Instellingen'!$B$22,"Absolute top",IF(N135&gt;='Instellingen'!$B$23,"Kopman",IF(N135&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N135&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -7944,12 +7944,12 @@
       </x:c>
       <x:c r="L136" t="n">
         <x:f>IF(K136="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K136/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>445</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="M136"/>
       <x:c r="N136" t="n">
         <x:f>IF(L136="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L136+IF(M136="",0,M136))))</x:f>
-        <x:v>445</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="O136" t="str">
         <x:f>IF(N136="","",IF(N136&gt;='Instellingen'!$B$22,"Absolute top",IF(N136&gt;='Instellingen'!$B$23,"Kopman",IF(N136&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N136&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8002,12 +8002,12 @@
       </x:c>
       <x:c r="L137" t="n">
         <x:f>IF(K137="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K137/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>482</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="M137"/>
       <x:c r="N137" t="n">
         <x:f>IF(L137="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L137+IF(M137="",0,M137))))</x:f>
-        <x:v>482</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="O137" t="str">
         <x:f>IF(N137="","",IF(N137&gt;='Instellingen'!$B$22,"Absolute top",IF(N137&gt;='Instellingen'!$B$23,"Kopman",IF(N137&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N137&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8060,16 +8060,16 @@
       </x:c>
       <x:c r="L138" t="n">
         <x:f>IF(K138="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K138/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>513</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="M138"/>
       <x:c r="N138" t="n">
         <x:f>IF(L138="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L138+IF(M138="",0,M138))))</x:f>
-        <x:v>513</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="O138" t="str">
         <x:f>IF(N138="","",IF(N138&gt;='Instellingen'!$B$22,"Absolute top",IF(N138&gt;='Instellingen'!$B$23,"Kopman",IF(N138&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N138&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P138" t="str">
         <x:f>IF(A138="","",IF(D138="","Rol invullen","Compleet"))</x:f>
@@ -8118,12 +8118,12 @@
       </x:c>
       <x:c r="L139" t="n">
         <x:f>IF(K139="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K139/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>446</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="M139"/>
       <x:c r="N139" t="n">
         <x:f>IF(L139="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L139+IF(M139="",0,M139))))</x:f>
-        <x:v>446</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="O139" t="str">
         <x:f>IF(N139="","",IF(N139&gt;='Instellingen'!$B$22,"Absolute top",IF(N139&gt;='Instellingen'!$B$23,"Kopman",IF(N139&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N139&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8176,12 +8176,12 @@
       </x:c>
       <x:c r="L140" t="n">
         <x:f>IF(K140="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K140/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>419</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="M140"/>
       <x:c r="N140" t="n">
         <x:f>IF(L140="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L140+IF(M140="",0,M140))))</x:f>
-        <x:v>419</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="O140" t="str">
         <x:f>IF(N140="","",IF(N140&gt;='Instellingen'!$B$22,"Absolute top",IF(N140&gt;='Instellingen'!$B$23,"Kopman",IF(N140&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N140&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8234,16 +8234,16 @@
       </x:c>
       <x:c r="L141" t="n">
         <x:f>IF(K141="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K141/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>537</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="M141"/>
       <x:c r="N141" t="n">
         <x:f>IF(L141="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L141+IF(M141="",0,M141))))</x:f>
-        <x:v>537</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="O141" t="str">
         <x:f>IF(N141="","",IF(N141&gt;='Instellingen'!$B$22,"Absolute top",IF(N141&gt;='Instellingen'!$B$23,"Kopman",IF(N141&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N141&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P141" t="str">
         <x:f>IF(A141="","",IF(D141="","Rol invullen","Compleet"))</x:f>
@@ -8292,12 +8292,12 @@
       </x:c>
       <x:c r="L142" t="n">
         <x:f>IF(K142="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K142/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>479</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="M142"/>
       <x:c r="N142" t="n">
         <x:f>IF(L142="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L142+IF(M142="",0,M142))))</x:f>
-        <x:v>479</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="O142" t="str">
         <x:f>IF(N142="","",IF(N142&gt;='Instellingen'!$B$22,"Absolute top",IF(N142&gt;='Instellingen'!$B$23,"Kopman",IF(N142&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N142&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8350,16 +8350,16 @@
       </x:c>
       <x:c r="L143" t="n">
         <x:f>IF(K143="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K143/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>692</x:v>
+        <x:v>1048</x:v>
       </x:c>
       <x:c r="M143"/>
       <x:c r="N143" t="n">
         <x:f>IF(L143="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L143+IF(M143="",0,M143))))</x:f>
-        <x:v>692</x:v>
+        <x:v>1048</x:v>
       </x:c>
       <x:c r="O143" t="str">
         <x:f>IF(N143="","",IF(N143&gt;='Instellingen'!$B$22,"Absolute top",IF(N143&gt;='Instellingen'!$B$23,"Kopman",IF(N143&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N143&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P143" t="str">
         <x:f>IF(A143="","",IF(D143="","Rol invullen","Compleet"))</x:f>
@@ -8408,12 +8408,12 @@
       </x:c>
       <x:c r="L144" t="n">
         <x:f>IF(K144="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K144/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>438</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="M144"/>
       <x:c r="N144" t="n">
         <x:f>IF(L144="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L144+IF(M144="",0,M144))))</x:f>
-        <x:v>438</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="O144" t="str">
         <x:f>IF(N144="","",IF(N144&gt;='Instellingen'!$B$22,"Absolute top",IF(N144&gt;='Instellingen'!$B$23,"Kopman",IF(N144&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N144&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8466,12 +8466,12 @@
       </x:c>
       <x:c r="L145" t="n">
         <x:f>IF(K145="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K145/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>437</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="M145"/>
       <x:c r="N145" t="n">
         <x:f>IF(L145="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L145+IF(M145="",0,M145))))</x:f>
-        <x:v>437</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="O145" t="str">
         <x:f>IF(N145="","",IF(N145&gt;='Instellingen'!$B$22,"Absolute top",IF(N145&gt;='Instellingen'!$B$23,"Kopman",IF(N145&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N145&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8524,16 +8524,16 @@
       </x:c>
       <x:c r="L146" t="n">
         <x:f>IF(K146="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K146/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>523</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="M146"/>
       <x:c r="N146" t="n">
         <x:f>IF(L146="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L146+IF(M146="",0,M146))))</x:f>
-        <x:v>523</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="O146" t="str">
         <x:f>IF(N146="","",IF(N146&gt;='Instellingen'!$B$22,"Absolute top",IF(N146&gt;='Instellingen'!$B$23,"Kopman",IF(N146&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N146&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P146" t="str">
         <x:f>IF(A146="","",IF(D146="","Rol invullen","Compleet"))</x:f>
@@ -8582,16 +8582,16 @@
       </x:c>
       <x:c r="L147" t="n">
         <x:f>IF(K147="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K147/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>791</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="M147"/>
       <x:c r="N147" t="n">
         <x:f>IF(L147="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L147+IF(M147="",0,M147))))</x:f>
-        <x:v>791</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="O147" t="str">
         <x:f>IF(N147="","",IF(N147&gt;='Instellingen'!$B$22,"Absolute top",IF(N147&gt;='Instellingen'!$B$23,"Kopman",IF(N147&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N147&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P147" t="str">
         <x:f>IF(A147="","",IF(D147="","Rol invullen","Compleet"))</x:f>
@@ -8640,12 +8640,12 @@
       </x:c>
       <x:c r="L148" t="n">
         <x:f>IF(K148="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K148/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>376</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="M148"/>
       <x:c r="N148" t="n">
         <x:f>IF(L148="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L148+IF(M148="",0,M148))))</x:f>
-        <x:v>376</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="O148" t="str">
         <x:f>IF(N148="","",IF(N148&gt;='Instellingen'!$B$22,"Absolute top",IF(N148&gt;='Instellingen'!$B$23,"Kopman",IF(N148&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N148&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -8698,16 +8698,16 @@
       </x:c>
       <x:c r="L149" t="n">
         <x:f>IF(K149="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K149/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>520</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="M149"/>
       <x:c r="N149" t="n">
         <x:f>IF(L149="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L149+IF(M149="",0,M149))))</x:f>
-        <x:v>520</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="O149" t="str">
         <x:f>IF(N149="","",IF(N149&gt;='Instellingen'!$B$22,"Absolute top",IF(N149&gt;='Instellingen'!$B$23,"Kopman",IF(N149&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N149&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P149" t="str">
         <x:f>IF(A149="","",IF(D149="","Rol invullen","Compleet"))</x:f>
@@ -8756,16 +8756,16 @@
       </x:c>
       <x:c r="L150" t="n">
         <x:f>IF(K150="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K150/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>592</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="M150"/>
       <x:c r="N150" t="n">
         <x:f>IF(L150="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L150+IF(M150="",0,M150))))</x:f>
-        <x:v>592</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="O150" t="str">
         <x:f>IF(N150="","",IF(N150&gt;='Instellingen'!$B$22,"Absolute top",IF(N150&gt;='Instellingen'!$B$23,"Kopman",IF(N150&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N150&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P150" t="str">
         <x:f>IF(A150="","",IF(D150="","Rol invullen","Compleet"))</x:f>
@@ -8814,16 +8814,16 @@
       </x:c>
       <x:c r="L151" t="n">
         <x:f>IF(K151="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K151/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>623</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="M151"/>
       <x:c r="N151" t="n">
         <x:f>IF(L151="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L151+IF(M151="",0,M151))))</x:f>
-        <x:v>623</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="O151" t="str">
         <x:f>IF(N151="","",IF(N151&gt;='Instellingen'!$B$22,"Absolute top",IF(N151&gt;='Instellingen'!$B$23,"Kopman",IF(N151&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N151&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P151" t="str">
         <x:f>IF(A151="","",IF(D151="","Rol invullen","Compleet"))</x:f>
@@ -8872,16 +8872,16 @@
       </x:c>
       <x:c r="L152" t="n">
         <x:f>IF(K152="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K152/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>604</x:v>
+        <x:v>880</x:v>
       </x:c>
       <x:c r="M152"/>
       <x:c r="N152" t="n">
         <x:f>IF(L152="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L152+IF(M152="",0,M152))))</x:f>
-        <x:v>604</x:v>
+        <x:v>880</x:v>
       </x:c>
       <x:c r="O152" t="str">
         <x:f>IF(N152="","",IF(N152&gt;='Instellingen'!$B$22,"Absolute top",IF(N152&gt;='Instellingen'!$B$23,"Kopman",IF(N152&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N152&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P152" t="str">
         <x:f>IF(A152="","",IF(D152="","Rol invullen","Compleet"))</x:f>
@@ -8930,16 +8930,16 @@
       </x:c>
       <x:c r="L153" t="n">
         <x:f>IF(K153="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K153/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>578</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="M153"/>
       <x:c r="N153" t="n">
         <x:f>IF(L153="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L153+IF(M153="",0,M153))))</x:f>
-        <x:v>578</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="O153" t="str">
         <x:f>IF(N153="","",IF(N153&gt;='Instellingen'!$B$22,"Absolute top",IF(N153&gt;='Instellingen'!$B$23,"Kopman",IF(N153&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N153&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P153" t="str">
         <x:f>IF(A153="","",IF(D153="","Rol invullen","Compleet"))</x:f>
@@ -8988,12 +8988,12 @@
       </x:c>
       <x:c r="L154" t="n">
         <x:f>IF(K154="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K154/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>470</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="M154"/>
       <x:c r="N154" t="n">
         <x:f>IF(L154="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L154+IF(M154="",0,M154))))</x:f>
-        <x:v>470</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="O154" t="str">
         <x:f>IF(N154="","",IF(N154&gt;='Instellingen'!$B$22,"Absolute top",IF(N154&gt;='Instellingen'!$B$23,"Kopman",IF(N154&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N154&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9046,16 +9046,16 @@
       </x:c>
       <x:c r="L155" t="n">
         <x:f>IF(K155="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K155/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>528</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="M155"/>
       <x:c r="N155" t="n">
         <x:f>IF(L155="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L155+IF(M155="",0,M155))))</x:f>
-        <x:v>528</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="O155" t="str">
         <x:f>IF(N155="","",IF(N155&gt;='Instellingen'!$B$22,"Absolute top",IF(N155&gt;='Instellingen'!$B$23,"Kopman",IF(N155&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N155&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P155" t="str">
         <x:f>IF(A155="","",IF(D155="","Rol invullen","Compleet"))</x:f>
@@ -9104,12 +9104,12 @@
       </x:c>
       <x:c r="L156" t="n">
         <x:f>IF(K156="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K156/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>480</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="M156"/>
       <x:c r="N156" t="n">
         <x:f>IF(L156="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L156+IF(M156="",0,M156))))</x:f>
-        <x:v>480</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="O156" t="str">
         <x:f>IF(N156="","",IF(N156&gt;='Instellingen'!$B$22,"Absolute top",IF(N156&gt;='Instellingen'!$B$23,"Kopman",IF(N156&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N156&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9162,16 +9162,16 @@
       </x:c>
       <x:c r="L157" t="n">
         <x:f>IF(K157="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K157/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>825</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="M157"/>
       <x:c r="N157" t="n">
         <x:f>IF(L157="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L157+IF(M157="",0,M157))))</x:f>
-        <x:v>825</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="O157" t="str">
         <x:f>IF(N157="","",IF(N157&gt;='Instellingen'!$B$22,"Absolute top",IF(N157&gt;='Instellingen'!$B$23,"Kopman",IF(N157&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N157&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Bruikbaar</x:v>
+        <x:v>Sterke keuze</x:v>
       </x:c>
       <x:c r="P157" t="str">
         <x:f>IF(A157="","",IF(D157="","Rol invullen","Compleet"))</x:f>
@@ -9220,12 +9220,12 @@
       </x:c>
       <x:c r="L158" t="n">
         <x:f>IF(K158="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K158/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>706</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="M158"/>
       <x:c r="N158" t="n">
         <x:f>IF(L158="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L158+IF(M158="",0,M158))))</x:f>
-        <x:v>706</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="O158" t="str">
         <x:f>IF(N158="","",IF(N158&gt;='Instellingen'!$B$22,"Absolute top",IF(N158&gt;='Instellingen'!$B$23,"Kopman",IF(N158&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N158&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9278,16 +9278,16 @@
       </x:c>
       <x:c r="L159" t="n">
         <x:f>IF(K159="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K159/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>528</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="M159"/>
       <x:c r="N159" t="n">
         <x:f>IF(L159="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L159+IF(M159="",0,M159))))</x:f>
-        <x:v>528</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="O159" t="str">
         <x:f>IF(N159="","",IF(N159&gt;='Instellingen'!$B$22,"Absolute top",IF(N159&gt;='Instellingen'!$B$23,"Kopman",IF(N159&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N159&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
-        <x:v>Gok</x:v>
+        <x:v>Bruikbaar</x:v>
       </x:c>
       <x:c r="P159" t="str">
         <x:f>IF(A159="","",IF(D159="","Rol invullen","Compleet"))</x:f>
@@ -9336,12 +9336,12 @@
       </x:c>
       <x:c r="L160" t="n">
         <x:f>IF(K160="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K160/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>476</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="M160"/>
       <x:c r="N160" t="n">
         <x:f>IF(L160="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L160+IF(M160="",0,M160))))</x:f>
-        <x:v>476</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="O160" t="str">
         <x:f>IF(N160="","",IF(N160&gt;='Instellingen'!$B$22,"Absolute top",IF(N160&gt;='Instellingen'!$B$23,"Kopman",IF(N160&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N160&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9394,12 +9394,12 @@
       </x:c>
       <x:c r="L161" t="n">
         <x:f>IF(K161="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K161/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>480</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="M161"/>
       <x:c r="N161" t="n">
         <x:f>IF(L161="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L161+IF(M161="",0,M161))))</x:f>
-        <x:v>480</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="O161" t="str">
         <x:f>IF(N161="","",IF(N161&gt;='Instellingen'!$B$22,"Absolute top",IF(N161&gt;='Instellingen'!$B$23,"Kopman",IF(N161&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N161&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9452,12 +9452,12 @@
       </x:c>
       <x:c r="L162" t="n">
         <x:f>IF(K162="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K162/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>428</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="M162"/>
       <x:c r="N162" t="n">
         <x:f>IF(L162="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L162+IF(M162="",0,M162))))</x:f>
-        <x:v>428</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="O162" t="str">
         <x:f>IF(N162="","",IF(N162&gt;='Instellingen'!$B$22,"Absolute top",IF(N162&gt;='Instellingen'!$B$23,"Kopman",IF(N162&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N162&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9510,12 +9510,12 @@
       </x:c>
       <x:c r="L163" t="n">
         <x:f>IF(K163="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K163/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>347</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="M163"/>
       <x:c r="N163" t="n">
         <x:f>IF(L163="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L163+IF(M163="",0,M163))))</x:f>
-        <x:v>347</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="O163" t="str">
         <x:f>IF(N163="","",IF(N163&gt;='Instellingen'!$B$22,"Absolute top",IF(N163&gt;='Instellingen'!$B$23,"Kopman",IF(N163&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N163&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9568,12 +9568,12 @@
       </x:c>
       <x:c r="L164" t="n">
         <x:f>IF(K164="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K164/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>359</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="M164"/>
       <x:c r="N164" t="n">
         <x:f>IF(L164="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L164+IF(M164="",0,M164))))</x:f>
-        <x:v>359</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="O164" t="str">
         <x:f>IF(N164="","",IF(N164&gt;='Instellingen'!$B$22,"Absolute top",IF(N164&gt;='Instellingen'!$B$23,"Kopman",IF(N164&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N164&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9626,12 +9626,12 @@
       </x:c>
       <x:c r="L165" t="n">
         <x:f>IF(K165="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K165/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>451</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="M165"/>
       <x:c r="N165" t="n">
         <x:f>IF(L165="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L165+IF(M165="",0,M165))))</x:f>
-        <x:v>451</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="O165" t="str">
         <x:f>IF(N165="","",IF(N165&gt;='Instellingen'!$B$22,"Absolute top",IF(N165&gt;='Instellingen'!$B$23,"Kopman",IF(N165&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N165&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9684,12 +9684,12 @@
       </x:c>
       <x:c r="L166" t="n">
         <x:f>IF(K166="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K166/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>445</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="M166"/>
       <x:c r="N166" t="n">
         <x:f>IF(L166="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L166+IF(M166="",0,M166))))</x:f>
-        <x:v>445</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="O166" t="str">
         <x:f>IF(N166="","",IF(N166&gt;='Instellingen'!$B$22,"Absolute top",IF(N166&gt;='Instellingen'!$B$23,"Kopman",IF(N166&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N166&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9742,12 +9742,12 @@
       </x:c>
       <x:c r="L167" t="n">
         <x:f>IF(K167="","",ROUND(('Instellingen'!$B$16+('Instellingen'!$B$17-'Instellingen'!$B$16)*POWER(K167/100,'Instellingen'!$B$18))/'Instellingen'!$B$19,0)*'Instellingen'!$B$19)</x:f>
-        <x:v>449</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="M167"/>
       <x:c r="N167" t="n">
         <x:f>IF(L167="","",MAX('Instellingen'!$B$16,MIN('Instellingen'!$B$17,L167+IF(M167="",0,M167))))</x:f>
-        <x:v>449</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="O167" t="str">
         <x:f>IF(N167="","",IF(N167&gt;='Instellingen'!$B$22,"Absolute top",IF(N167&gt;='Instellingen'!$B$23,"Kopman",IF(N167&gt;='Instellingen'!$B$24,"Sterke keuze",IF(N167&gt;='Instellingen'!$B$25,"Bruikbaar","Gok")))))</x:f>
@@ -9971,7 +9971,7 @@
         <x:v>Maximumprijs</x:v>
       </x:c>
       <x:c r="B17" t="n">
-        <x:v>2500</x:v>
+        <x:v>4500</x:v>
       </x:c>
       <x:c r="C17"/>
       <x:c r="D17"/>

</xml_diff>

<commit_message>
Verlaag maximale Vuelta-prijsschaal naar 4000 BC
</commit_message>
<xml_diff>
--- a/outputs/vuelta-2026-20260818/Wielerpool_prijslijst_vuelta_2026.xlsx
+++ b/outputs/vuelta-2026-20260818/Wielerpool_prijslijst_vuelta_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kejes\Documents\Codex\Projecten\_gedeelde-logica\outputs\vuelta-2026-20260818\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C97EFEAD-1455-454A-AEB4-A83AF792C2D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA8DD42-18FC-455B-A3D0-6FCD03B88B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Renners" sheetId="1" r:id="rId1"/>
@@ -1776,11 +1776,11 @@
       </c>
       <c r="L6">
         <f>IF(K6="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K6/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>3671</v>
+        <v>3270</v>
       </c>
       <c r="N6">
         <f>IF(L6="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L6+IF(M6="",0,M6))))</f>
-        <v>3671</v>
+        <v>3270</v>
       </c>
       <c r="O6" t="str">
         <f>IF(N6="","",IF(N6&gt;=Instellingen!$B$22,"Absolute top",IF(N6&gt;=Instellingen!$B$23,"Kopman",IF(N6&gt;=Instellingen!$B$24,"Sterke keuze",IF(N6&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -1833,11 +1833,11 @@
       </c>
       <c r="L7">
         <f>IF(K7="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K7/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>2931</v>
+        <v>2618</v>
       </c>
       <c r="N7">
         <f>IF(L7="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L7+IF(M7="",0,M7))))</f>
-        <v>2931</v>
+        <v>2618</v>
       </c>
       <c r="O7" t="str">
         <f>IF(N7="","",IF(N7&gt;=Instellingen!$B$22,"Absolute top",IF(N7&gt;=Instellingen!$B$23,"Kopman",IF(N7&gt;=Instellingen!$B$24,"Sterke keuze",IF(N7&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -1890,11 +1890,11 @@
       </c>
       <c r="L8">
         <f>IF(K8="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K8/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>2113</v>
+        <v>1897</v>
       </c>
       <c r="N8">
         <f>IF(L8="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L8+IF(M8="",0,M8))))</f>
-        <v>2113</v>
+        <v>1897</v>
       </c>
       <c r="O8" t="str">
         <f>IF(N8="","",IF(N8&gt;=Instellingen!$B$22,"Absolute top",IF(N8&gt;=Instellingen!$B$23,"Kopman",IF(N8&gt;=Instellingen!$B$24,"Sterke keuze",IF(N8&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -1947,11 +1947,11 @@
       </c>
       <c r="L9">
         <f>IF(K9="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K9/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1852</v>
+        <v>1667</v>
       </c>
       <c r="N9">
         <f>IF(L9="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L9+IF(M9="",0,M9))))</f>
-        <v>1852</v>
+        <v>1667</v>
       </c>
       <c r="O9" t="str">
         <f>IF(N9="","",IF(N9&gt;=Instellingen!$B$22,"Absolute top",IF(N9&gt;=Instellingen!$B$23,"Kopman",IF(N9&gt;=Instellingen!$B$24,"Sterke keuze",IF(N9&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2004,18 +2004,18 @@
       </c>
       <c r="L10">
         <f>IF(K10="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K10/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1819</v>
+        <v>1638</v>
       </c>
       <c r="M10">
         <v>-200</v>
       </c>
       <c r="N10">
         <f>IF(L10="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L10+IF(M10="",0,M10))))</f>
-        <v>1619</v>
+        <v>1438</v>
       </c>
       <c r="O10" t="str">
         <f>IF(N10="","",IF(N10&gt;=Instellingen!$B$22,"Absolute top",IF(N10&gt;=Instellingen!$B$23,"Kopman",IF(N10&gt;=Instellingen!$B$24,"Sterke keuze",IF(N10&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Kopman</v>
+        <v>Sterke keuze</v>
       </c>
       <c r="P10" t="str">
         <f>IF(A10="","",IF(D10="","Rol invullen","Compleet"))</f>
@@ -2064,11 +2064,11 @@
       </c>
       <c r="L11">
         <f>IF(K11="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K11/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1807</v>
+        <v>1627</v>
       </c>
       <c r="N11">
         <f>IF(L11="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L11+IF(M11="",0,M11))))</f>
-        <v>1807</v>
+        <v>1627</v>
       </c>
       <c r="O11" t="str">
         <f>IF(N11="","",IF(N11&gt;=Instellingen!$B$22,"Absolute top",IF(N11&gt;=Instellingen!$B$23,"Kopman",IF(N11&gt;=Instellingen!$B$24,"Sterke keuze",IF(N11&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2121,15 +2121,15 @@
       </c>
       <c r="L12">
         <f>IF(K12="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K12/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1740</v>
+        <v>1568</v>
       </c>
       <c r="N12">
         <f>IF(L12="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L12+IF(M12="",0,M12))))</f>
-        <v>1740</v>
+        <v>1568</v>
       </c>
       <c r="O12" t="str">
         <f>IF(N12="","",IF(N12&gt;=Instellingen!$B$22,"Absolute top",IF(N12&gt;=Instellingen!$B$23,"Kopman",IF(N12&gt;=Instellingen!$B$24,"Sterke keuze",IF(N12&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Kopman</v>
+        <v>Sterke keuze</v>
       </c>
       <c r="P12" t="str">
         <f>IF(A12="","",IF(D12="","Rol invullen","Compleet"))</f>
@@ -2178,15 +2178,15 @@
       </c>
       <c r="L13">
         <f>IF(K13="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K13/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1720</v>
+        <v>1551</v>
       </c>
       <c r="N13">
         <f>IF(L13="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L13+IF(M13="",0,M13))))</f>
-        <v>1720</v>
+        <v>1551</v>
       </c>
       <c r="O13" t="str">
         <f>IF(N13="","",IF(N13&gt;=Instellingen!$B$22,"Absolute top",IF(N13&gt;=Instellingen!$B$23,"Kopman",IF(N13&gt;=Instellingen!$B$24,"Sterke keuze",IF(N13&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Kopman</v>
+        <v>Sterke keuze</v>
       </c>
       <c r="P13" t="str">
         <f>IF(A13="","",IF(D13="","Rol invullen","Compleet"))</f>
@@ -2235,15 +2235,15 @@
       </c>
       <c r="L14">
         <f>IF(K14="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K14/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1634</v>
+        <v>1475</v>
       </c>
       <c r="N14">
         <f>IF(L14="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L14+IF(M14="",0,M14))))</f>
-        <v>1634</v>
+        <v>1475</v>
       </c>
       <c r="O14" t="str">
         <f>IF(N14="","",IF(N14&gt;=Instellingen!$B$22,"Absolute top",IF(N14&gt;=Instellingen!$B$23,"Kopman",IF(N14&gt;=Instellingen!$B$24,"Sterke keuze",IF(N14&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Kopman</v>
+        <v>Sterke keuze</v>
       </c>
       <c r="P14" t="str">
         <f>IF(A14="","",IF(D14="","Rol invullen","Compleet"))</f>
@@ -2292,11 +2292,11 @@
       </c>
       <c r="L15">
         <f>IF(K15="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K15/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1557</v>
+        <v>1407</v>
       </c>
       <c r="N15">
         <f>IF(L15="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L15+IF(M15="",0,M15))))</f>
-        <v>1557</v>
+        <v>1407</v>
       </c>
       <c r="O15" t="str">
         <f>IF(N15="","",IF(N15&gt;=Instellingen!$B$22,"Absolute top",IF(N15&gt;=Instellingen!$B$23,"Kopman",IF(N15&gt;=Instellingen!$B$24,"Sterke keuze",IF(N15&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2349,14 +2349,14 @@
       </c>
       <c r="L16">
         <f>IF(K16="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K16/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1551</v>
+        <v>1402</v>
       </c>
       <c r="M16">
         <v>-200</v>
       </c>
       <c r="N16">
         <f>IF(L16="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L16+IF(M16="",0,M16))))</f>
-        <v>1351</v>
+        <v>1202</v>
       </c>
       <c r="O16" t="str">
         <f>IF(N16="","",IF(N16&gt;=Instellingen!$B$22,"Absolute top",IF(N16&gt;=Instellingen!$B$23,"Kopman",IF(N16&gt;=Instellingen!$B$24,"Sterke keuze",IF(N16&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2409,11 +2409,11 @@
       </c>
       <c r="L17">
         <f>IF(K17="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K17/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1430</v>
+        <v>1295</v>
       </c>
       <c r="N17">
         <f>IF(L17="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L17+IF(M17="",0,M17))))</f>
-        <v>1430</v>
+        <v>1295</v>
       </c>
       <c r="O17" t="str">
         <f>IF(N17="","",IF(N17&gt;=Instellingen!$B$22,"Absolute top",IF(N17&gt;=Instellingen!$B$23,"Kopman",IF(N17&gt;=Instellingen!$B$24,"Sterke keuze",IF(N17&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2466,11 +2466,11 @@
       </c>
       <c r="L18">
         <f>IF(K18="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K18/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1427</v>
+        <v>1293</v>
       </c>
       <c r="N18">
         <f>IF(L18="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L18+IF(M18="",0,M18))))</f>
-        <v>1427</v>
+        <v>1293</v>
       </c>
       <c r="O18" t="str">
         <f>IF(N18="","",IF(N18&gt;=Instellingen!$B$22,"Absolute top",IF(N18&gt;=Instellingen!$B$23,"Kopman",IF(N18&gt;=Instellingen!$B$24,"Sterke keuze",IF(N18&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2523,11 +2523,11 @@
       </c>
       <c r="L19">
         <f>IF(K19="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K19/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1402</v>
+        <v>1271</v>
       </c>
       <c r="N19">
         <f>IF(L19="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L19+IF(M19="",0,M19))))</f>
-        <v>1402</v>
+        <v>1271</v>
       </c>
       <c r="O19" t="str">
         <f>IF(N19="","",IF(N19&gt;=Instellingen!$B$22,"Absolute top",IF(N19&gt;=Instellingen!$B$23,"Kopman",IF(N19&gt;=Instellingen!$B$24,"Sterke keuze",IF(N19&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2580,11 +2580,11 @@
       </c>
       <c r="L20">
         <f>IF(K20="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K20/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1360</v>
+        <v>1234</v>
       </c>
       <c r="N20">
         <f>IF(L20="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L20+IF(M20="",0,M20))))</f>
-        <v>1360</v>
+        <v>1234</v>
       </c>
       <c r="O20" t="str">
         <f>IF(N20="","",IF(N20&gt;=Instellingen!$B$22,"Absolute top",IF(N20&gt;=Instellingen!$B$23,"Kopman",IF(N20&gt;=Instellingen!$B$24,"Sterke keuze",IF(N20&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2637,11 +2637,11 @@
       </c>
       <c r="L21">
         <f>IF(K21="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K21/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1311</v>
+        <v>1191</v>
       </c>
       <c r="N21">
         <f>IF(L21="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L21+IF(M21="",0,M21))))</f>
-        <v>1311</v>
+        <v>1191</v>
       </c>
       <c r="O21" t="str">
         <f>IF(N21="","",IF(N21&gt;=Instellingen!$B$22,"Absolute top",IF(N21&gt;=Instellingen!$B$23,"Kopman",IF(N21&gt;=Instellingen!$B$24,"Sterke keuze",IF(N21&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2694,11 +2694,11 @@
       </c>
       <c r="L22">
         <f>IF(K22="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K22/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1301</v>
+        <v>1182</v>
       </c>
       <c r="N22">
         <f>IF(L22="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L22+IF(M22="",0,M22))))</f>
-        <v>1301</v>
+        <v>1182</v>
       </c>
       <c r="O22" t="str">
         <f>IF(N22="","",IF(N22&gt;=Instellingen!$B$22,"Absolute top",IF(N22&gt;=Instellingen!$B$23,"Kopman",IF(N22&gt;=Instellingen!$B$24,"Sterke keuze",IF(N22&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2751,11 +2751,11 @@
       </c>
       <c r="L23">
         <f>IF(K23="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K23/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1301</v>
+        <v>1182</v>
       </c>
       <c r="N23">
         <f>IF(L23="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L23+IF(M23="",0,M23))))</f>
-        <v>1301</v>
+        <v>1182</v>
       </c>
       <c r="O23" t="str">
         <f>IF(N23="","",IF(N23&gt;=Instellingen!$B$22,"Absolute top",IF(N23&gt;=Instellingen!$B$23,"Kopman",IF(N23&gt;=Instellingen!$B$24,"Sterke keuze",IF(N23&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2808,11 +2808,11 @@
       </c>
       <c r="L24">
         <f>IF(K24="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K24/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1255</v>
+        <v>1141</v>
       </c>
       <c r="N24">
         <f>IF(L24="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L24+IF(M24="",0,M24))))</f>
-        <v>1255</v>
+        <v>1141</v>
       </c>
       <c r="O24" t="str">
         <f>IF(N24="","",IF(N24&gt;=Instellingen!$B$22,"Absolute top",IF(N24&gt;=Instellingen!$B$23,"Kopman",IF(N24&gt;=Instellingen!$B$24,"Sterke keuze",IF(N24&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2865,11 +2865,11 @@
       </c>
       <c r="L25">
         <f>IF(K25="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K25/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1226</v>
+        <v>1115</v>
       </c>
       <c r="N25">
         <f>IF(L25="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L25+IF(M25="",0,M25))))</f>
-        <v>1226</v>
+        <v>1115</v>
       </c>
       <c r="O25" t="str">
         <f>IF(N25="","",IF(N25&gt;=Instellingen!$B$22,"Absolute top",IF(N25&gt;=Instellingen!$B$23,"Kopman",IF(N25&gt;=Instellingen!$B$24,"Sterke keuze",IF(N25&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2922,11 +2922,11 @@
       </c>
       <c r="L26">
         <f>IF(K26="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K26/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1211</v>
+        <v>1103</v>
       </c>
       <c r="N26">
         <f>IF(L26="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L26+IF(M26="",0,M26))))</f>
-        <v>1211</v>
+        <v>1103</v>
       </c>
       <c r="O26" t="str">
         <f>IF(N26="","",IF(N26&gt;=Instellingen!$B$22,"Absolute top",IF(N26&gt;=Instellingen!$B$23,"Kopman",IF(N26&gt;=Instellingen!$B$24,"Sterke keuze",IF(N26&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -2979,11 +2979,11 @@
       </c>
       <c r="L27">
         <f>IF(K27="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K27/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1209</v>
+        <v>1101</v>
       </c>
       <c r="N27">
         <f>IF(L27="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L27+IF(M27="",0,M27))))</f>
-        <v>1209</v>
+        <v>1101</v>
       </c>
       <c r="O27" t="str">
         <f>IF(N27="","",IF(N27&gt;=Instellingen!$B$22,"Absolute top",IF(N27&gt;=Instellingen!$B$23,"Kopman",IF(N27&gt;=Instellingen!$B$24,"Sterke keuze",IF(N27&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3036,15 +3036,15 @@
       </c>
       <c r="L28">
         <f>IF(K28="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K28/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1200</v>
+        <v>1092</v>
       </c>
       <c r="N28">
         <f>IF(L28="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L28+IF(M28="",0,M28))))</f>
-        <v>1200</v>
+        <v>1092</v>
       </c>
       <c r="O28" t="str">
         <f>IF(N28="","",IF(N28&gt;=Instellingen!$B$22,"Absolute top",IF(N28&gt;=Instellingen!$B$23,"Kopman",IF(N28&gt;=Instellingen!$B$24,"Sterke keuze",IF(N28&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Sterke keuze</v>
+        <v>Bruikbaar</v>
       </c>
       <c r="P28" t="str">
         <f>IF(A28="","",IF(D28="","Rol invullen","Compleet"))</f>
@@ -3093,15 +3093,15 @@
       </c>
       <c r="L29">
         <f>IF(K29="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K29/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1195</v>
+        <v>1088</v>
       </c>
       <c r="N29">
         <f>IF(L29="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L29+IF(M29="",0,M29))))</f>
-        <v>1195</v>
+        <v>1088</v>
       </c>
       <c r="O29" t="str">
         <f>IF(N29="","",IF(N29&gt;=Instellingen!$B$22,"Absolute top",IF(N29&gt;=Instellingen!$B$23,"Kopman",IF(N29&gt;=Instellingen!$B$24,"Sterke keuze",IF(N29&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Sterke keuze</v>
+        <v>Bruikbaar</v>
       </c>
       <c r="P29" t="str">
         <f>IF(A29="","",IF(D29="","Rol invullen","Compleet"))</f>
@@ -3150,18 +3150,18 @@
       </c>
       <c r="L30">
         <f>IF(K30="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K30/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1147</v>
+        <v>1046</v>
       </c>
       <c r="M30">
         <v>500</v>
       </c>
       <c r="N30">
         <f>IF(L30="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L30+IF(M30="",0,M30))))</f>
-        <v>1647</v>
+        <v>1546</v>
       </c>
       <c r="O30" t="str">
         <f>IF(N30="","",IF(N30&gt;=Instellingen!$B$22,"Absolute top",IF(N30&gt;=Instellingen!$B$23,"Kopman",IF(N30&gt;=Instellingen!$B$24,"Sterke keuze",IF(N30&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Kopman</v>
+        <v>Sterke keuze</v>
       </c>
       <c r="P30" t="str">
         <f>IF(A30="","",IF(D30="","Rol invullen","Compleet"))</f>
@@ -3210,14 +3210,14 @@
       </c>
       <c r="L31">
         <f>IF(K31="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K31/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1076</v>
+        <v>983</v>
       </c>
       <c r="M31">
         <v>400</v>
       </c>
       <c r="N31">
         <f>IF(L31="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L31+IF(M31="",0,M31))))</f>
-        <v>1476</v>
+        <v>1383</v>
       </c>
       <c r="O31" t="str">
         <f>IF(N31="","",IF(N31&gt;=Instellingen!$B$22,"Absolute top",IF(N31&gt;=Instellingen!$B$23,"Kopman",IF(N31&gt;=Instellingen!$B$24,"Sterke keuze",IF(N31&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3270,11 +3270,11 @@
       </c>
       <c r="L32">
         <f>IF(K32="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K32/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1065</v>
+        <v>974</v>
       </c>
       <c r="N32">
         <f>IF(L32="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L32+IF(M32="",0,M32))))</f>
-        <v>1065</v>
+        <v>974</v>
       </c>
       <c r="O32" t="str">
         <f>IF(N32="","",IF(N32&gt;=Instellingen!$B$22,"Absolute top",IF(N32&gt;=Instellingen!$B$23,"Kopman",IF(N32&gt;=Instellingen!$B$24,"Sterke keuze",IF(N32&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3327,11 +3327,11 @@
       </c>
       <c r="L33">
         <f>IF(K33="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K33/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>1048</v>
+        <v>959</v>
       </c>
       <c r="N33">
         <f>IF(L33="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L33+IF(M33="",0,M33))))</f>
-        <v>1048</v>
+        <v>959</v>
       </c>
       <c r="O33" t="str">
         <f>IF(N33="","",IF(N33&gt;=Instellingen!$B$22,"Absolute top",IF(N33&gt;=Instellingen!$B$23,"Kopman",IF(N33&gt;=Instellingen!$B$24,"Sterke keuze",IF(N33&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3384,11 +3384,11 @@
       </c>
       <c r="L34">
         <f>IF(K34="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K34/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>992</v>
+        <v>910</v>
       </c>
       <c r="N34">
         <f>IF(L34="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L34+IF(M34="",0,M34))))</f>
-        <v>992</v>
+        <v>910</v>
       </c>
       <c r="O34" t="str">
         <f>IF(N34="","",IF(N34&gt;=Instellingen!$B$22,"Absolute top",IF(N34&gt;=Instellingen!$B$23,"Kopman",IF(N34&gt;=Instellingen!$B$24,"Sterke keuze",IF(N34&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3441,11 +3441,11 @@
       </c>
       <c r="L35">
         <f>IF(K35="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K35/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>988</v>
+        <v>906</v>
       </c>
       <c r="N35">
         <f>IF(L35="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L35+IF(M35="",0,M35))))</f>
-        <v>988</v>
+        <v>906</v>
       </c>
       <c r="O35" t="str">
         <f>IF(N35="","",IF(N35&gt;=Instellingen!$B$22,"Absolute top",IF(N35&gt;=Instellingen!$B$23,"Kopman",IF(N35&gt;=Instellingen!$B$24,"Sterke keuze",IF(N35&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3498,11 +3498,11 @@
       </c>
       <c r="L36">
         <f>IF(K36="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K36/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>981</v>
+        <v>900</v>
       </c>
       <c r="N36">
         <f>IF(L36="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L36+IF(M36="",0,M36))))</f>
-        <v>981</v>
+        <v>900</v>
       </c>
       <c r="O36" t="str">
         <f>IF(N36="","",IF(N36&gt;=Instellingen!$B$22,"Absolute top",IF(N36&gt;=Instellingen!$B$23,"Kopman",IF(N36&gt;=Instellingen!$B$24,"Sterke keuze",IF(N36&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3555,11 +3555,11 @@
       </c>
       <c r="L37">
         <f>IF(K37="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K37/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>979</v>
+        <v>898</v>
       </c>
       <c r="N37">
         <f>IF(L37="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L37+IF(M37="",0,M37))))</f>
-        <v>979</v>
+        <v>898</v>
       </c>
       <c r="O37" t="str">
         <f>IF(N37="","",IF(N37&gt;=Instellingen!$B$22,"Absolute top",IF(N37&gt;=Instellingen!$B$23,"Kopman",IF(N37&gt;=Instellingen!$B$24,"Sterke keuze",IF(N37&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3612,11 +3612,11 @@
       </c>
       <c r="L38">
         <f>IF(K38="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K38/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>965</v>
+        <v>886</v>
       </c>
       <c r="N38">
         <f>IF(L38="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L38+IF(M38="",0,M38))))</f>
-        <v>965</v>
+        <v>886</v>
       </c>
       <c r="O38" t="str">
         <f>IF(N38="","",IF(N38&gt;=Instellingen!$B$22,"Absolute top",IF(N38&gt;=Instellingen!$B$23,"Kopman",IF(N38&gt;=Instellingen!$B$24,"Sterke keuze",IF(N38&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3669,11 +3669,11 @@
       </c>
       <c r="L39">
         <f>IF(K39="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K39/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>932</v>
+        <v>857</v>
       </c>
       <c r="N39">
         <f>IF(L39="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L39+IF(M39="",0,M39))))</f>
-        <v>932</v>
+        <v>857</v>
       </c>
       <c r="O39" t="str">
         <f>IF(N39="","",IF(N39&gt;=Instellingen!$B$22,"Absolute top",IF(N39&gt;=Instellingen!$B$23,"Kopman",IF(N39&gt;=Instellingen!$B$24,"Sterke keuze",IF(N39&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3726,11 +3726,11 @@
       </c>
       <c r="L40">
         <f>IF(K40="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K40/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>927</v>
+        <v>852</v>
       </c>
       <c r="N40">
         <f>IF(L40="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L40+IF(M40="",0,M40))))</f>
-        <v>927</v>
+        <v>852</v>
       </c>
       <c r="O40" t="str">
         <f>IF(N40="","",IF(N40&gt;=Instellingen!$B$22,"Absolute top",IF(N40&gt;=Instellingen!$B$23,"Kopman",IF(N40&gt;=Instellingen!$B$24,"Sterke keuze",IF(N40&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3783,11 +3783,11 @@
       </c>
       <c r="L41">
         <f>IF(K41="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K41/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>917</v>
+        <v>843</v>
       </c>
       <c r="N41">
         <f>IF(L41="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L41+IF(M41="",0,M41))))</f>
-        <v>917</v>
+        <v>843</v>
       </c>
       <c r="O41" t="str">
         <f>IF(N41="","",IF(N41&gt;=Instellingen!$B$22,"Absolute top",IF(N41&gt;=Instellingen!$B$23,"Kopman",IF(N41&gt;=Instellingen!$B$24,"Sterke keuze",IF(N41&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3840,11 +3840,11 @@
       </c>
       <c r="L42">
         <f>IF(K42="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K42/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>884</v>
+        <v>815</v>
       </c>
       <c r="N42">
         <f>IF(L42="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L42+IF(M42="",0,M42))))</f>
-        <v>884</v>
+        <v>815</v>
       </c>
       <c r="O42" t="str">
         <f>IF(N42="","",IF(N42&gt;=Instellingen!$B$22,"Absolute top",IF(N42&gt;=Instellingen!$B$23,"Kopman",IF(N42&gt;=Instellingen!$B$24,"Sterke keuze",IF(N42&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3897,14 +3897,14 @@
       </c>
       <c r="L43">
         <f>IF(K43="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K43/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>881</v>
+        <v>812</v>
       </c>
       <c r="M43">
         <v>100</v>
       </c>
       <c r="N43">
         <f>IF(L43="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L43+IF(M43="",0,M43))))</f>
-        <v>981</v>
+        <v>912</v>
       </c>
       <c r="O43" t="str">
         <f>IF(N43="","",IF(N43&gt;=Instellingen!$B$22,"Absolute top",IF(N43&gt;=Instellingen!$B$23,"Kopman",IF(N43&gt;=Instellingen!$B$24,"Sterke keuze",IF(N43&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -3957,11 +3957,11 @@
       </c>
       <c r="L44">
         <f>IF(K44="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K44/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>880</v>
+        <v>811</v>
       </c>
       <c r="N44">
         <f>IF(L44="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L44+IF(M44="",0,M44))))</f>
-        <v>880</v>
+        <v>811</v>
       </c>
       <c r="O44" t="str">
         <f>IF(N44="","",IF(N44&gt;=Instellingen!$B$22,"Absolute top",IF(N44&gt;=Instellingen!$B$23,"Kopman",IF(N44&gt;=Instellingen!$B$24,"Sterke keuze",IF(N44&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4014,14 +4014,14 @@
       </c>
       <c r="L45">
         <f>IF(K45="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K45/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>878</v>
+        <v>809</v>
       </c>
       <c r="M45">
         <v>100</v>
       </c>
       <c r="N45">
         <f>IF(L45="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L45+IF(M45="",0,M45))))</f>
-        <v>978</v>
+        <v>909</v>
       </c>
       <c r="O45" t="str">
         <f>IF(N45="","",IF(N45&gt;=Instellingen!$B$22,"Absolute top",IF(N45&gt;=Instellingen!$B$23,"Kopman",IF(N45&gt;=Instellingen!$B$24,"Sterke keuze",IF(N45&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4074,11 +4074,11 @@
       </c>
       <c r="L46">
         <f>IF(K46="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K46/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>872</v>
+        <v>803</v>
       </c>
       <c r="N46">
         <f>IF(L46="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L46+IF(M46="",0,M46))))</f>
-        <v>872</v>
+        <v>803</v>
       </c>
       <c r="O46" t="str">
         <f>IF(N46="","",IF(N46&gt;=Instellingen!$B$22,"Absolute top",IF(N46&gt;=Instellingen!$B$23,"Kopman",IF(N46&gt;=Instellingen!$B$24,"Sterke keuze",IF(N46&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4131,11 +4131,11 @@
       </c>
       <c r="L47">
         <f>IF(K47="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K47/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>865</v>
+        <v>798</v>
       </c>
       <c r="N47">
         <f>IF(L47="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L47+IF(M47="",0,M47))))</f>
-        <v>865</v>
+        <v>798</v>
       </c>
       <c r="O47" t="str">
         <f>IF(N47="","",IF(N47&gt;=Instellingen!$B$22,"Absolute top",IF(N47&gt;=Instellingen!$B$23,"Kopman",IF(N47&gt;=Instellingen!$B$24,"Sterke keuze",IF(N47&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4188,11 +4188,11 @@
       </c>
       <c r="L48">
         <f>IF(K48="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K48/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>858</v>
+        <v>791</v>
       </c>
       <c r="N48">
         <f>IF(L48="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L48+IF(M48="",0,M48))))</f>
-        <v>858</v>
+        <v>791</v>
       </c>
       <c r="O48" t="str">
         <f>IF(N48="","",IF(N48&gt;=Instellingen!$B$22,"Absolute top",IF(N48&gt;=Instellingen!$B$23,"Kopman",IF(N48&gt;=Instellingen!$B$24,"Sterke keuze",IF(N48&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4245,11 +4245,11 @@
       </c>
       <c r="L49">
         <f>IF(K49="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K49/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>857</v>
+        <v>791</v>
       </c>
       <c r="N49">
         <f>IF(L49="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L49+IF(M49="",0,M49))))</f>
-        <v>857</v>
+        <v>791</v>
       </c>
       <c r="O49" t="str">
         <f>IF(N49="","",IF(N49&gt;=Instellingen!$B$22,"Absolute top",IF(N49&gt;=Instellingen!$B$23,"Kopman",IF(N49&gt;=Instellingen!$B$24,"Sterke keuze",IF(N49&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4302,11 +4302,11 @@
       </c>
       <c r="L50">
         <f>IF(K50="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K50/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>853</v>
+        <v>787</v>
       </c>
       <c r="N50">
         <f>IF(L50="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L50+IF(M50="",0,M50))))</f>
-        <v>853</v>
+        <v>787</v>
       </c>
       <c r="O50" t="str">
         <f>IF(N50="","",IF(N50&gt;=Instellingen!$B$22,"Absolute top",IF(N50&gt;=Instellingen!$B$23,"Kopman",IF(N50&gt;=Instellingen!$B$24,"Sterke keuze",IF(N50&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4359,11 +4359,11 @@
       </c>
       <c r="L51">
         <f>IF(K51="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K51/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>849</v>
+        <v>783</v>
       </c>
       <c r="N51">
         <f>IF(L51="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L51+IF(M51="",0,M51))))</f>
-        <v>849</v>
+        <v>783</v>
       </c>
       <c r="O51" t="str">
         <f>IF(N51="","",IF(N51&gt;=Instellingen!$B$22,"Absolute top",IF(N51&gt;=Instellingen!$B$23,"Kopman",IF(N51&gt;=Instellingen!$B$24,"Sterke keuze",IF(N51&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4416,11 +4416,11 @@
       </c>
       <c r="L52">
         <f>IF(K52="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K52/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>848</v>
+        <v>782</v>
       </c>
       <c r="N52">
         <f>IF(L52="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L52+IF(M52="",0,M52))))</f>
-        <v>848</v>
+        <v>782</v>
       </c>
       <c r="O52" t="str">
         <f>IF(N52="","",IF(N52&gt;=Instellingen!$B$22,"Absolute top",IF(N52&gt;=Instellingen!$B$23,"Kopman",IF(N52&gt;=Instellingen!$B$24,"Sterke keuze",IF(N52&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4473,11 +4473,11 @@
       </c>
       <c r="L53">
         <f>IF(K53="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K53/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>847</v>
+        <v>782</v>
       </c>
       <c r="N53">
         <f>IF(L53="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L53+IF(M53="",0,M53))))</f>
-        <v>847</v>
+        <v>782</v>
       </c>
       <c r="O53" t="str">
         <f>IF(N53="","",IF(N53&gt;=Instellingen!$B$22,"Absolute top",IF(N53&gt;=Instellingen!$B$23,"Kopman",IF(N53&gt;=Instellingen!$B$24,"Sterke keuze",IF(N53&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4530,11 +4530,11 @@
       </c>
       <c r="L54">
         <f>IF(K54="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K54/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>832</v>
+        <v>768</v>
       </c>
       <c r="N54">
         <f>IF(L54="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L54+IF(M54="",0,M54))))</f>
-        <v>832</v>
+        <v>768</v>
       </c>
       <c r="O54" t="str">
         <f>IF(N54="","",IF(N54&gt;=Instellingen!$B$22,"Absolute top",IF(N54&gt;=Instellingen!$B$23,"Kopman",IF(N54&gt;=Instellingen!$B$24,"Sterke keuze",IF(N54&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4587,11 +4587,11 @@
       </c>
       <c r="L55">
         <f>IF(K55="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K55/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>806</v>
+        <v>746</v>
       </c>
       <c r="N55">
         <f>IF(L55="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L55+IF(M55="",0,M55))))</f>
-        <v>806</v>
+        <v>746</v>
       </c>
       <c r="O55" t="str">
         <f>IF(N55="","",IF(N55&gt;=Instellingen!$B$22,"Absolute top",IF(N55&gt;=Instellingen!$B$23,"Kopman",IF(N55&gt;=Instellingen!$B$24,"Sterke keuze",IF(N55&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4644,11 +4644,11 @@
       </c>
       <c r="L56">
         <f>IF(K56="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K56/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>799</v>
+        <v>740</v>
       </c>
       <c r="N56">
         <f>IF(L56="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L56+IF(M56="",0,M56))))</f>
-        <v>799</v>
+        <v>740</v>
       </c>
       <c r="O56" t="str">
         <f>IF(N56="","",IF(N56&gt;=Instellingen!$B$22,"Absolute top",IF(N56&gt;=Instellingen!$B$23,"Kopman",IF(N56&gt;=Instellingen!$B$24,"Sterke keuze",IF(N56&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4701,11 +4701,11 @@
       </c>
       <c r="L57">
         <f>IF(K57="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K57/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>796</v>
+        <v>737</v>
       </c>
       <c r="N57">
         <f>IF(L57="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L57+IF(M57="",0,M57))))</f>
-        <v>796</v>
+        <v>737</v>
       </c>
       <c r="O57" t="str">
         <f>IF(N57="","",IF(N57&gt;=Instellingen!$B$22,"Absolute top",IF(N57&gt;=Instellingen!$B$23,"Kopman",IF(N57&gt;=Instellingen!$B$24,"Sterke keuze",IF(N57&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4758,11 +4758,11 @@
       </c>
       <c r="L58">
         <f>IF(K58="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K58/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>779</v>
+        <v>722</v>
       </c>
       <c r="N58">
         <f>IF(L58="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L58+IF(M58="",0,M58))))</f>
-        <v>779</v>
+        <v>722</v>
       </c>
       <c r="O58" t="str">
         <f>IF(N58="","",IF(N58&gt;=Instellingen!$B$22,"Absolute top",IF(N58&gt;=Instellingen!$B$23,"Kopman",IF(N58&gt;=Instellingen!$B$24,"Sterke keuze",IF(N58&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4815,11 +4815,11 @@
       </c>
       <c r="L59">
         <f>IF(K59="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K59/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>764</v>
+        <v>709</v>
       </c>
       <c r="N59">
         <f>IF(L59="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L59+IF(M59="",0,M59))))</f>
-        <v>764</v>
+        <v>709</v>
       </c>
       <c r="O59" t="str">
         <f>IF(N59="","",IF(N59&gt;=Instellingen!$B$22,"Absolute top",IF(N59&gt;=Instellingen!$B$23,"Kopman",IF(N59&gt;=Instellingen!$B$24,"Sterke keuze",IF(N59&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4872,11 +4872,11 @@
       </c>
       <c r="L60">
         <f>IF(K60="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K60/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>760</v>
+        <v>705</v>
       </c>
       <c r="N60">
         <f>IF(L60="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L60+IF(M60="",0,M60))))</f>
-        <v>760</v>
+        <v>705</v>
       </c>
       <c r="O60" t="str">
         <f>IF(N60="","",IF(N60&gt;=Instellingen!$B$22,"Absolute top",IF(N60&gt;=Instellingen!$B$23,"Kopman",IF(N60&gt;=Instellingen!$B$24,"Sterke keuze",IF(N60&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4929,11 +4929,11 @@
       </c>
       <c r="L61">
         <f>IF(K61="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K61/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>757</v>
+        <v>702</v>
       </c>
       <c r="N61">
         <f>IF(L61="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L61+IF(M61="",0,M61))))</f>
-        <v>757</v>
+        <v>702</v>
       </c>
       <c r="O61" t="str">
         <f>IF(N61="","",IF(N61&gt;=Instellingen!$B$22,"Absolute top",IF(N61&gt;=Instellingen!$B$23,"Kopman",IF(N61&gt;=Instellingen!$B$24,"Sterke keuze",IF(N61&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -4986,15 +4986,15 @@
       </c>
       <c r="L62">
         <f>IF(K62="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K62/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>753</v>
+        <v>699</v>
       </c>
       <c r="N62">
         <f>IF(L62="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L62+IF(M62="",0,M62))))</f>
-        <v>753</v>
+        <v>699</v>
       </c>
       <c r="O62" t="str">
         <f>IF(N62="","",IF(N62&gt;=Instellingen!$B$22,"Absolute top",IF(N62&gt;=Instellingen!$B$23,"Kopman",IF(N62&gt;=Instellingen!$B$24,"Sterke keuze",IF(N62&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P62" t="str">
         <f>IF(A62="","",IF(D62="","Rol invullen","Compleet"))</f>
@@ -5043,15 +5043,15 @@
       </c>
       <c r="L63">
         <f>IF(K63="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K63/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>737</v>
+        <v>685</v>
       </c>
       <c r="N63">
         <f>IF(L63="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L63+IF(M63="",0,M63))))</f>
-        <v>737</v>
+        <v>685</v>
       </c>
       <c r="O63" t="str">
         <f>IF(N63="","",IF(N63&gt;=Instellingen!$B$22,"Absolute top",IF(N63&gt;=Instellingen!$B$23,"Kopman",IF(N63&gt;=Instellingen!$B$24,"Sterke keuze",IF(N63&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P63" t="str">
         <f>IF(A63="","",IF(D63="","Rol invullen","Compleet"))</f>
@@ -5100,15 +5100,15 @@
       </c>
       <c r="L64">
         <f>IF(K64="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K64/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>736</v>
+        <v>684</v>
       </c>
       <c r="N64">
         <f>IF(L64="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L64+IF(M64="",0,M64))))</f>
-        <v>736</v>
+        <v>684</v>
       </c>
       <c r="O64" t="str">
         <f>IF(N64="","",IF(N64&gt;=Instellingen!$B$22,"Absolute top",IF(N64&gt;=Instellingen!$B$23,"Kopman",IF(N64&gt;=Instellingen!$B$24,"Sterke keuze",IF(N64&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P64" t="str">
         <f>IF(A64="","",IF(D64="","Rol invullen","Compleet"))</f>
@@ -5157,15 +5157,15 @@
       </c>
       <c r="L65">
         <f>IF(K65="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K65/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>736</v>
+        <v>684</v>
       </c>
       <c r="N65">
         <f>IF(L65="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L65+IF(M65="",0,M65))))</f>
-        <v>736</v>
+        <v>684</v>
       </c>
       <c r="O65" t="str">
         <f>IF(N65="","",IF(N65&gt;=Instellingen!$B$22,"Absolute top",IF(N65&gt;=Instellingen!$B$23,"Kopman",IF(N65&gt;=Instellingen!$B$24,"Sterke keuze",IF(N65&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P65" t="str">
         <f>IF(A65="","",IF(D65="","Rol invullen","Compleet"))</f>
@@ -5214,15 +5214,15 @@
       </c>
       <c r="L66">
         <f>IF(K66="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K66/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>734</v>
+        <v>683</v>
       </c>
       <c r="N66">
         <f>IF(L66="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L66+IF(M66="",0,M66))))</f>
-        <v>734</v>
+        <v>683</v>
       </c>
       <c r="O66" t="str">
         <f>IF(N66="","",IF(N66&gt;=Instellingen!$B$22,"Absolute top",IF(N66&gt;=Instellingen!$B$23,"Kopman",IF(N66&gt;=Instellingen!$B$24,"Sterke keuze",IF(N66&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P66" t="str">
         <f>IF(A66="","",IF(D66="","Rol invullen","Compleet"))</f>
@@ -5271,15 +5271,15 @@
       </c>
       <c r="L67">
         <f>IF(K67="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K67/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>733</v>
+        <v>681</v>
       </c>
       <c r="N67">
         <f>IF(L67="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L67+IF(M67="",0,M67))))</f>
-        <v>733</v>
+        <v>681</v>
       </c>
       <c r="O67" t="str">
         <f>IF(N67="","",IF(N67&gt;=Instellingen!$B$22,"Absolute top",IF(N67&gt;=Instellingen!$B$23,"Kopman",IF(N67&gt;=Instellingen!$B$24,"Sterke keuze",IF(N67&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P67" t="str">
         <f>IF(A67="","",IF(D67="","Rol invullen","Compleet"))</f>
@@ -5328,14 +5328,14 @@
       </c>
       <c r="L68">
         <f>IF(K68="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K68/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>732</v>
+        <v>681</v>
       </c>
       <c r="M68">
         <v>125</v>
       </c>
       <c r="N68">
         <f>IF(L68="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L68+IF(M68="",0,M68))))</f>
-        <v>857</v>
+        <v>806</v>
       </c>
       <c r="O68" t="str">
         <f>IF(N68="","",IF(N68&gt;=Instellingen!$B$22,"Absolute top",IF(N68&gt;=Instellingen!$B$23,"Kopman",IF(N68&gt;=Instellingen!$B$24,"Sterke keuze",IF(N68&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -5388,15 +5388,15 @@
       </c>
       <c r="L69">
         <f>IF(K69="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K69/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>725</v>
+        <v>674</v>
       </c>
       <c r="N69">
         <f>IF(L69="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L69+IF(M69="",0,M69))))</f>
-        <v>725</v>
+        <v>674</v>
       </c>
       <c r="O69" t="str">
         <f>IF(N69="","",IF(N69&gt;=Instellingen!$B$22,"Absolute top",IF(N69&gt;=Instellingen!$B$23,"Kopman",IF(N69&gt;=Instellingen!$B$24,"Sterke keuze",IF(N69&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P69" t="str">
         <f>IF(A69="","",IF(D69="","Rol invullen","Compleet"))</f>
@@ -5445,15 +5445,15 @@
       </c>
       <c r="L70">
         <f>IF(K70="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K70/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>721</v>
+        <v>671</v>
       </c>
       <c r="N70">
         <f>IF(L70="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L70+IF(M70="",0,M70))))</f>
-        <v>721</v>
+        <v>671</v>
       </c>
       <c r="O70" t="str">
         <f>IF(N70="","",IF(N70&gt;=Instellingen!$B$22,"Absolute top",IF(N70&gt;=Instellingen!$B$23,"Kopman",IF(N70&gt;=Instellingen!$B$24,"Sterke keuze",IF(N70&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P70" t="str">
         <f>IF(A70="","",IF(D70="","Rol invullen","Compleet"))</f>
@@ -5502,15 +5502,15 @@
       </c>
       <c r="L71">
         <f>IF(K71="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K71/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>720</v>
+        <v>670</v>
       </c>
       <c r="N71">
         <f>IF(L71="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L71+IF(M71="",0,M71))))</f>
-        <v>720</v>
+        <v>670</v>
       </c>
       <c r="O71" t="str">
         <f>IF(N71="","",IF(N71&gt;=Instellingen!$B$22,"Absolute top",IF(N71&gt;=Instellingen!$B$23,"Kopman",IF(N71&gt;=Instellingen!$B$24,"Sterke keuze",IF(N71&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P71" t="str">
         <f>IF(A71="","",IF(D71="","Rol invullen","Compleet"))</f>
@@ -5559,15 +5559,15 @@
       </c>
       <c r="L72">
         <f>IF(K72="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K72/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>711</v>
+        <v>662</v>
       </c>
       <c r="N72">
         <f>IF(L72="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L72+IF(M72="",0,M72))))</f>
-        <v>711</v>
+        <v>662</v>
       </c>
       <c r="O72" t="str">
         <f>IF(N72="","",IF(N72&gt;=Instellingen!$B$22,"Absolute top",IF(N72&gt;=Instellingen!$B$23,"Kopman",IF(N72&gt;=Instellingen!$B$24,"Sterke keuze",IF(N72&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P72" t="str">
         <f>IF(A72="","",IF(D72="","Rol invullen","Compleet"))</f>
@@ -5616,15 +5616,15 @@
       </c>
       <c r="L73">
         <f>IF(K73="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K73/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>711</v>
+        <v>662</v>
       </c>
       <c r="N73">
         <f>IF(L73="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L73+IF(M73="",0,M73))))</f>
-        <v>711</v>
+        <v>662</v>
       </c>
       <c r="O73" t="str">
         <f>IF(N73="","",IF(N73&gt;=Instellingen!$B$22,"Absolute top",IF(N73&gt;=Instellingen!$B$23,"Kopman",IF(N73&gt;=Instellingen!$B$24,"Sterke keuze",IF(N73&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P73" t="str">
         <f>IF(A73="","",IF(D73="","Rol invullen","Compleet"))</f>
@@ -5673,15 +5673,15 @@
       </c>
       <c r="L74">
         <f>IF(K74="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K74/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>707</v>
+        <v>658</v>
       </c>
       <c r="N74">
         <f>IF(L74="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L74+IF(M74="",0,M74))))</f>
-        <v>707</v>
+        <v>658</v>
       </c>
       <c r="O74" t="str">
         <f>IF(N74="","",IF(N74&gt;=Instellingen!$B$22,"Absolute top",IF(N74&gt;=Instellingen!$B$23,"Kopman",IF(N74&gt;=Instellingen!$B$24,"Sterke keuze",IF(N74&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P74" t="str">
         <f>IF(A74="","",IF(D74="","Rol invullen","Compleet"))</f>
@@ -5730,15 +5730,15 @@
       </c>
       <c r="L75">
         <f>IF(K75="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K75/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>706</v>
+        <v>658</v>
       </c>
       <c r="N75">
         <f>IF(L75="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L75+IF(M75="",0,M75))))</f>
-        <v>706</v>
+        <v>658</v>
       </c>
       <c r="O75" t="str">
         <f>IF(N75="","",IF(N75&gt;=Instellingen!$B$22,"Absolute top",IF(N75&gt;=Instellingen!$B$23,"Kopman",IF(N75&gt;=Instellingen!$B$24,"Sterke keuze",IF(N75&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
-        <v>Bruikbaar</v>
+        <v>Gok</v>
       </c>
       <c r="P75" t="str">
         <f>IF(A75="","",IF(D75="","Rol invullen","Compleet"))</f>
@@ -5787,11 +5787,11 @@
       </c>
       <c r="L76">
         <f>IF(K76="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K76/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>699</v>
+        <v>651</v>
       </c>
       <c r="N76">
         <f>IF(L76="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L76+IF(M76="",0,M76))))</f>
-        <v>699</v>
+        <v>651</v>
       </c>
       <c r="O76" t="str">
         <f>IF(N76="","",IF(N76&gt;=Instellingen!$B$22,"Absolute top",IF(N76&gt;=Instellingen!$B$23,"Kopman",IF(N76&gt;=Instellingen!$B$24,"Sterke keuze",IF(N76&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -5844,11 +5844,11 @@
       </c>
       <c r="L77">
         <f>IF(K77="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K77/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>699</v>
+        <v>651</v>
       </c>
       <c r="N77">
         <f>IF(L77="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L77+IF(M77="",0,M77))))</f>
-        <v>699</v>
+        <v>651</v>
       </c>
       <c r="O77" t="str">
         <f>IF(N77="","",IF(N77&gt;=Instellingen!$B$22,"Absolute top",IF(N77&gt;=Instellingen!$B$23,"Kopman",IF(N77&gt;=Instellingen!$B$24,"Sterke keuze",IF(N77&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -5901,11 +5901,11 @@
       </c>
       <c r="L78">
         <f>IF(K78="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K78/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>683</v>
+        <v>637</v>
       </c>
       <c r="N78">
         <f>IF(L78="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L78+IF(M78="",0,M78))))</f>
-        <v>683</v>
+        <v>637</v>
       </c>
       <c r="O78" t="str">
         <f>IF(N78="","",IF(N78&gt;=Instellingen!$B$22,"Absolute top",IF(N78&gt;=Instellingen!$B$23,"Kopman",IF(N78&gt;=Instellingen!$B$24,"Sterke keuze",IF(N78&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -5958,11 +5958,11 @@
       </c>
       <c r="L79">
         <f>IF(K79="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K79/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>682</v>
+        <v>636</v>
       </c>
       <c r="N79">
         <f>IF(L79="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L79+IF(M79="",0,M79))))</f>
-        <v>682</v>
+        <v>636</v>
       </c>
       <c r="O79" t="str">
         <f>IF(N79="","",IF(N79&gt;=Instellingen!$B$22,"Absolute top",IF(N79&gt;=Instellingen!$B$23,"Kopman",IF(N79&gt;=Instellingen!$B$24,"Sterke keuze",IF(N79&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6015,11 +6015,11 @@
       </c>
       <c r="L80">
         <f>IF(K80="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K80/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>678</v>
+        <v>633</v>
       </c>
       <c r="N80">
         <f>IF(L80="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L80+IF(M80="",0,M80))))</f>
-        <v>678</v>
+        <v>633</v>
       </c>
       <c r="O80" t="str">
         <f>IF(N80="","",IF(N80&gt;=Instellingen!$B$22,"Absolute top",IF(N80&gt;=Instellingen!$B$23,"Kopman",IF(N80&gt;=Instellingen!$B$24,"Sterke keuze",IF(N80&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6072,11 +6072,11 @@
       </c>
       <c r="L81">
         <f>IF(K81="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K81/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>676</v>
+        <v>632</v>
       </c>
       <c r="N81">
         <f>IF(L81="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L81+IF(M81="",0,M81))))</f>
-        <v>676</v>
+        <v>632</v>
       </c>
       <c r="O81" t="str">
         <f>IF(N81="","",IF(N81&gt;=Instellingen!$B$22,"Absolute top",IF(N81&gt;=Instellingen!$B$23,"Kopman",IF(N81&gt;=Instellingen!$B$24,"Sterke keuze",IF(N81&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6129,11 +6129,11 @@
       </c>
       <c r="L82">
         <f>IF(K82="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K82/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>675</v>
+        <v>630</v>
       </c>
       <c r="N82">
         <f>IF(L82="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L82+IF(M82="",0,M82))))</f>
-        <v>675</v>
+        <v>630</v>
       </c>
       <c r="O82" t="str">
         <f>IF(N82="","",IF(N82&gt;=Instellingen!$B$22,"Absolute top",IF(N82&gt;=Instellingen!$B$23,"Kopman",IF(N82&gt;=Instellingen!$B$24,"Sterke keuze",IF(N82&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6186,11 +6186,11 @@
       </c>
       <c r="L83">
         <f>IF(K83="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K83/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>675</v>
+        <v>630</v>
       </c>
       <c r="N83">
         <f>IF(L83="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L83+IF(M83="",0,M83))))</f>
-        <v>675</v>
+        <v>630</v>
       </c>
       <c r="O83" t="str">
         <f>IF(N83="","",IF(N83&gt;=Instellingen!$B$22,"Absolute top",IF(N83&gt;=Instellingen!$B$23,"Kopman",IF(N83&gt;=Instellingen!$B$24,"Sterke keuze",IF(N83&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6243,11 +6243,11 @@
       </c>
       <c r="L84">
         <f>IF(K84="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K84/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>674</v>
+        <v>629</v>
       </c>
       <c r="N84">
         <f>IF(L84="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L84+IF(M84="",0,M84))))</f>
-        <v>674</v>
+        <v>629</v>
       </c>
       <c r="O84" t="str">
         <f>IF(N84="","",IF(N84&gt;=Instellingen!$B$22,"Absolute top",IF(N84&gt;=Instellingen!$B$23,"Kopman",IF(N84&gt;=Instellingen!$B$24,"Sterke keuze",IF(N84&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6300,11 +6300,11 @@
       </c>
       <c r="L85">
         <f>IF(K85="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K85/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>674</v>
+        <v>629</v>
       </c>
       <c r="N85">
         <f>IF(L85="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L85+IF(M85="",0,M85))))</f>
-        <v>674</v>
+        <v>629</v>
       </c>
       <c r="O85" t="str">
         <f>IF(N85="","",IF(N85&gt;=Instellingen!$B$22,"Absolute top",IF(N85&gt;=Instellingen!$B$23,"Kopman",IF(N85&gt;=Instellingen!$B$24,"Sterke keuze",IF(N85&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6357,11 +6357,11 @@
       </c>
       <c r="L86">
         <f>IF(K86="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K86/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>669</v>
+        <v>625</v>
       </c>
       <c r="N86">
         <f>IF(L86="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L86+IF(M86="",0,M86))))</f>
-        <v>669</v>
+        <v>625</v>
       </c>
       <c r="O86" t="str">
         <f>IF(N86="","",IF(N86&gt;=Instellingen!$B$22,"Absolute top",IF(N86&gt;=Instellingen!$B$23,"Kopman",IF(N86&gt;=Instellingen!$B$24,"Sterke keuze",IF(N86&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6414,11 +6414,11 @@
       </c>
       <c r="L87">
         <f>IF(K87="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K87/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>666</v>
+        <v>622</v>
       </c>
       <c r="N87">
         <f>IF(L87="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L87+IF(M87="",0,M87))))</f>
-        <v>666</v>
+        <v>622</v>
       </c>
       <c r="O87" t="str">
         <f>IF(N87="","",IF(N87&gt;=Instellingen!$B$22,"Absolute top",IF(N87&gt;=Instellingen!$B$23,"Kopman",IF(N87&gt;=Instellingen!$B$24,"Sterke keuze",IF(N87&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6471,11 +6471,11 @@
       </c>
       <c r="L88">
         <f>IF(K88="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K88/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>666</v>
+        <v>623</v>
       </c>
       <c r="N88">
         <f>IF(L88="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L88+IF(M88="",0,M88))))</f>
-        <v>666</v>
+        <v>623</v>
       </c>
       <c r="O88" t="str">
         <f>IF(N88="","",IF(N88&gt;=Instellingen!$B$22,"Absolute top",IF(N88&gt;=Instellingen!$B$23,"Kopman",IF(N88&gt;=Instellingen!$B$24,"Sterke keuze",IF(N88&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6528,11 +6528,11 @@
       </c>
       <c r="L89">
         <f>IF(K89="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K89/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>665</v>
+        <v>622</v>
       </c>
       <c r="N89">
         <f>IF(L89="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L89+IF(M89="",0,M89))))</f>
-        <v>665</v>
+        <v>622</v>
       </c>
       <c r="O89" t="str">
         <f>IF(N89="","",IF(N89&gt;=Instellingen!$B$22,"Absolute top",IF(N89&gt;=Instellingen!$B$23,"Kopman",IF(N89&gt;=Instellingen!$B$24,"Sterke keuze",IF(N89&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6585,11 +6585,11 @@
       </c>
       <c r="L90">
         <f>IF(K90="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K90/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>661</v>
+        <v>618</v>
       </c>
       <c r="N90">
         <f>IF(L90="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L90+IF(M90="",0,M90))))</f>
-        <v>661</v>
+        <v>618</v>
       </c>
       <c r="O90" t="str">
         <f>IF(N90="","",IF(N90&gt;=Instellingen!$B$22,"Absolute top",IF(N90&gt;=Instellingen!$B$23,"Kopman",IF(N90&gt;=Instellingen!$B$24,"Sterke keuze",IF(N90&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6642,11 +6642,11 @@
       </c>
       <c r="L91">
         <f>IF(K91="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K91/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>661</v>
+        <v>618</v>
       </c>
       <c r="N91">
         <f>IF(L91="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L91+IF(M91="",0,M91))))</f>
-        <v>661</v>
+        <v>618</v>
       </c>
       <c r="O91" t="str">
         <f>IF(N91="","",IF(N91&gt;=Instellingen!$B$22,"Absolute top",IF(N91&gt;=Instellingen!$B$23,"Kopman",IF(N91&gt;=Instellingen!$B$24,"Sterke keuze",IF(N91&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6699,11 +6699,11 @@
       </c>
       <c r="L92">
         <f>IF(K92="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K92/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>661</v>
+        <v>618</v>
       </c>
       <c r="N92">
         <f>IF(L92="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L92+IF(M92="",0,M92))))</f>
-        <v>661</v>
+        <v>618</v>
       </c>
       <c r="O92" t="str">
         <f>IF(N92="","",IF(N92&gt;=Instellingen!$B$22,"Absolute top",IF(N92&gt;=Instellingen!$B$23,"Kopman",IF(N92&gt;=Instellingen!$B$24,"Sterke keuze",IF(N92&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6756,11 +6756,11 @@
       </c>
       <c r="L93">
         <f>IF(K93="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K93/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>658</v>
+        <v>616</v>
       </c>
       <c r="N93">
         <f>IF(L93="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L93+IF(M93="",0,M93))))</f>
-        <v>658</v>
+        <v>616</v>
       </c>
       <c r="O93" t="str">
         <f>IF(N93="","",IF(N93&gt;=Instellingen!$B$22,"Absolute top",IF(N93&gt;=Instellingen!$B$23,"Kopman",IF(N93&gt;=Instellingen!$B$24,"Sterke keuze",IF(N93&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6813,11 +6813,11 @@
       </c>
       <c r="L94">
         <f>IF(K94="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K94/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>653</v>
+        <v>611</v>
       </c>
       <c r="N94">
         <f>IF(L94="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L94+IF(M94="",0,M94))))</f>
-        <v>653</v>
+        <v>611</v>
       </c>
       <c r="O94" t="str">
         <f>IF(N94="","",IF(N94&gt;=Instellingen!$B$22,"Absolute top",IF(N94&gt;=Instellingen!$B$23,"Kopman",IF(N94&gt;=Instellingen!$B$24,"Sterke keuze",IF(N94&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6870,11 +6870,11 @@
       </c>
       <c r="L95">
         <f>IF(K95="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K95/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>653</v>
+        <v>611</v>
       </c>
       <c r="N95">
         <f>IF(L95="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L95+IF(M95="",0,M95))))</f>
-        <v>653</v>
+        <v>611</v>
       </c>
       <c r="O95" t="str">
         <f>IF(N95="","",IF(N95&gt;=Instellingen!$B$22,"Absolute top",IF(N95&gt;=Instellingen!$B$23,"Kopman",IF(N95&gt;=Instellingen!$B$24,"Sterke keuze",IF(N95&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6927,11 +6927,11 @@
       </c>
       <c r="L96">
         <f>IF(K96="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K96/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>651</v>
+        <v>609</v>
       </c>
       <c r="N96">
         <f>IF(L96="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L96+IF(M96="",0,M96))))</f>
-        <v>651</v>
+        <v>609</v>
       </c>
       <c r="O96" t="str">
         <f>IF(N96="","",IF(N96&gt;=Instellingen!$B$22,"Absolute top",IF(N96&gt;=Instellingen!$B$23,"Kopman",IF(N96&gt;=Instellingen!$B$24,"Sterke keuze",IF(N96&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -6984,11 +6984,11 @@
       </c>
       <c r="L97">
         <f>IF(K97="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K97/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>650</v>
+        <v>609</v>
       </c>
       <c r="N97">
         <f>IF(L97="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L97+IF(M97="",0,M97))))</f>
-        <v>650</v>
+        <v>609</v>
       </c>
       <c r="O97" t="str">
         <f>IF(N97="","",IF(N97&gt;=Instellingen!$B$22,"Absolute top",IF(N97&gt;=Instellingen!$B$23,"Kopman",IF(N97&gt;=Instellingen!$B$24,"Sterke keuze",IF(N97&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7041,11 +7041,11 @@
       </c>
       <c r="L98">
         <f>IF(K98="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K98/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>649</v>
+        <v>607</v>
       </c>
       <c r="N98">
         <f>IF(L98="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L98+IF(M98="",0,M98))))</f>
-        <v>649</v>
+        <v>607</v>
       </c>
       <c r="O98" t="str">
         <f>IF(N98="","",IF(N98&gt;=Instellingen!$B$22,"Absolute top",IF(N98&gt;=Instellingen!$B$23,"Kopman",IF(N98&gt;=Instellingen!$B$24,"Sterke keuze",IF(N98&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7098,11 +7098,11 @@
       </c>
       <c r="L99">
         <f>IF(K99="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K99/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>648</v>
+        <v>606</v>
       </c>
       <c r="N99">
         <f>IF(L99="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L99+IF(M99="",0,M99))))</f>
-        <v>648</v>
+        <v>606</v>
       </c>
       <c r="O99" t="str">
         <f>IF(N99="","",IF(N99&gt;=Instellingen!$B$22,"Absolute top",IF(N99&gt;=Instellingen!$B$23,"Kopman",IF(N99&gt;=Instellingen!$B$24,"Sterke keuze",IF(N99&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7155,11 +7155,11 @@
       </c>
       <c r="L100">
         <f>IF(K100="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K100/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>647</v>
+        <v>605</v>
       </c>
       <c r="N100">
         <f>IF(L100="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L100+IF(M100="",0,M100))))</f>
-        <v>647</v>
+        <v>605</v>
       </c>
       <c r="O100" t="str">
         <f>IF(N100="","",IF(N100&gt;=Instellingen!$B$22,"Absolute top",IF(N100&gt;=Instellingen!$B$23,"Kopman",IF(N100&gt;=Instellingen!$B$24,"Sterke keuze",IF(N100&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7212,11 +7212,11 @@
       </c>
       <c r="L101">
         <f>IF(K101="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K101/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>647</v>
+        <v>605</v>
       </c>
       <c r="N101">
         <f>IF(L101="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L101+IF(M101="",0,M101))))</f>
-        <v>647</v>
+        <v>605</v>
       </c>
       <c r="O101" t="str">
         <f>IF(N101="","",IF(N101&gt;=Instellingen!$B$22,"Absolute top",IF(N101&gt;=Instellingen!$B$23,"Kopman",IF(N101&gt;=Instellingen!$B$24,"Sterke keuze",IF(N101&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7269,11 +7269,11 @@
       </c>
       <c r="L102">
         <f>IF(K102="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K102/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>645</v>
+        <v>604</v>
       </c>
       <c r="N102">
         <f>IF(L102="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L102+IF(M102="",0,M102))))</f>
-        <v>645</v>
+        <v>604</v>
       </c>
       <c r="O102" t="str">
         <f>IF(N102="","",IF(N102&gt;=Instellingen!$B$22,"Absolute top",IF(N102&gt;=Instellingen!$B$23,"Kopman",IF(N102&gt;=Instellingen!$B$24,"Sterke keuze",IF(N102&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7326,11 +7326,11 @@
       </c>
       <c r="L103">
         <f>IF(K103="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K103/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>645</v>
+        <v>604</v>
       </c>
       <c r="N103">
         <f>IF(L103="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L103+IF(M103="",0,M103))))</f>
-        <v>645</v>
+        <v>604</v>
       </c>
       <c r="O103" t="str">
         <f>IF(N103="","",IF(N103&gt;=Instellingen!$B$22,"Absolute top",IF(N103&gt;=Instellingen!$B$23,"Kopman",IF(N103&gt;=Instellingen!$B$24,"Sterke keuze",IF(N103&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7383,11 +7383,11 @@
       </c>
       <c r="L104">
         <f>IF(K104="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K104/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>644</v>
+        <v>603</v>
       </c>
       <c r="N104">
         <f>IF(L104="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L104+IF(M104="",0,M104))))</f>
-        <v>644</v>
+        <v>603</v>
       </c>
       <c r="O104" t="str">
         <f>IF(N104="","",IF(N104&gt;=Instellingen!$B$22,"Absolute top",IF(N104&gt;=Instellingen!$B$23,"Kopman",IF(N104&gt;=Instellingen!$B$24,"Sterke keuze",IF(N104&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7440,11 +7440,11 @@
       </c>
       <c r="L105">
         <f>IF(K105="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K105/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>643</v>
+        <v>603</v>
       </c>
       <c r="N105">
         <f>IF(L105="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L105+IF(M105="",0,M105))))</f>
-        <v>643</v>
+        <v>603</v>
       </c>
       <c r="O105" t="str">
         <f>IF(N105="","",IF(N105&gt;=Instellingen!$B$22,"Absolute top",IF(N105&gt;=Instellingen!$B$23,"Kopman",IF(N105&gt;=Instellingen!$B$24,"Sterke keuze",IF(N105&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7497,11 +7497,11 @@
       </c>
       <c r="L106">
         <f>IF(K106="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K106/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>642</v>
+        <v>602</v>
       </c>
       <c r="N106">
         <f>IF(L106="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L106+IF(M106="",0,M106))))</f>
-        <v>642</v>
+        <v>602</v>
       </c>
       <c r="O106" t="str">
         <f>IF(N106="","",IF(N106&gt;=Instellingen!$B$22,"Absolute top",IF(N106&gt;=Instellingen!$B$23,"Kopman",IF(N106&gt;=Instellingen!$B$24,"Sterke keuze",IF(N106&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7554,11 +7554,11 @@
       </c>
       <c r="L107">
         <f>IF(K107="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K107/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>641</v>
+        <v>600</v>
       </c>
       <c r="N107">
         <f>IF(L107="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L107+IF(M107="",0,M107))))</f>
-        <v>641</v>
+        <v>600</v>
       </c>
       <c r="O107" t="str">
         <f>IF(N107="","",IF(N107&gt;=Instellingen!$B$22,"Absolute top",IF(N107&gt;=Instellingen!$B$23,"Kopman",IF(N107&gt;=Instellingen!$B$24,"Sterke keuze",IF(N107&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7611,11 +7611,11 @@
       </c>
       <c r="L108">
         <f>IF(K108="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K108/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>641</v>
+        <v>601</v>
       </c>
       <c r="N108">
         <f>IF(L108="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L108+IF(M108="",0,M108))))</f>
-        <v>641</v>
+        <v>601</v>
       </c>
       <c r="O108" t="str">
         <f>IF(N108="","",IF(N108&gt;=Instellingen!$B$22,"Absolute top",IF(N108&gt;=Instellingen!$B$23,"Kopman",IF(N108&gt;=Instellingen!$B$24,"Sterke keuze",IF(N108&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7668,11 +7668,11 @@
       </c>
       <c r="L109">
         <f>IF(K109="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K109/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>641</v>
+        <v>601</v>
       </c>
       <c r="N109">
         <f>IF(L109="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L109+IF(M109="",0,M109))))</f>
-        <v>641</v>
+        <v>601</v>
       </c>
       <c r="O109" t="str">
         <f>IF(N109="","",IF(N109&gt;=Instellingen!$B$22,"Absolute top",IF(N109&gt;=Instellingen!$B$23,"Kopman",IF(N109&gt;=Instellingen!$B$24,"Sterke keuze",IF(N109&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7725,11 +7725,11 @@
       </c>
       <c r="L110">
         <f>IF(K110="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K110/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>640</v>
+        <v>599</v>
       </c>
       <c r="N110">
         <f>IF(L110="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L110+IF(M110="",0,M110))))</f>
-        <v>640</v>
+        <v>599</v>
       </c>
       <c r="O110" t="str">
         <f>IF(N110="","",IF(N110&gt;=Instellingen!$B$22,"Absolute top",IF(N110&gt;=Instellingen!$B$23,"Kopman",IF(N110&gt;=Instellingen!$B$24,"Sterke keuze",IF(N110&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7782,11 +7782,11 @@
       </c>
       <c r="L111">
         <f>IF(K111="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K111/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>639</v>
+        <v>598</v>
       </c>
       <c r="N111">
         <f>IF(L111="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L111+IF(M111="",0,M111))))</f>
-        <v>639</v>
+        <v>598</v>
       </c>
       <c r="O111" t="str">
         <f>IF(N111="","",IF(N111&gt;=Instellingen!$B$22,"Absolute top",IF(N111&gt;=Instellingen!$B$23,"Kopman",IF(N111&gt;=Instellingen!$B$24,"Sterke keuze",IF(N111&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7839,11 +7839,11 @@
       </c>
       <c r="L112">
         <f>IF(K112="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K112/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>637</v>
+        <v>597</v>
       </c>
       <c r="N112">
         <f>IF(L112="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L112+IF(M112="",0,M112))))</f>
-        <v>637</v>
+        <v>597</v>
       </c>
       <c r="O112" t="str">
         <f>IF(N112="","",IF(N112&gt;=Instellingen!$B$22,"Absolute top",IF(N112&gt;=Instellingen!$B$23,"Kopman",IF(N112&gt;=Instellingen!$B$24,"Sterke keuze",IF(N112&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7896,11 +7896,11 @@
       </c>
       <c r="L113">
         <f>IF(K113="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K113/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>637</v>
+        <v>597</v>
       </c>
       <c r="N113">
         <f>IF(L113="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L113+IF(M113="",0,M113))))</f>
-        <v>637</v>
+        <v>597</v>
       </c>
       <c r="O113" t="str">
         <f>IF(N113="","",IF(N113&gt;=Instellingen!$B$22,"Absolute top",IF(N113&gt;=Instellingen!$B$23,"Kopman",IF(N113&gt;=Instellingen!$B$24,"Sterke keuze",IF(N113&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -7953,11 +7953,11 @@
       </c>
       <c r="L114">
         <f>IF(K114="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K114/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>637</v>
+        <v>597</v>
       </c>
       <c r="N114">
         <f>IF(L114="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L114+IF(M114="",0,M114))))</f>
-        <v>637</v>
+        <v>597</v>
       </c>
       <c r="O114" t="str">
         <f>IF(N114="","",IF(N114&gt;=Instellingen!$B$22,"Absolute top",IF(N114&gt;=Instellingen!$B$23,"Kopman",IF(N114&gt;=Instellingen!$B$24,"Sterke keuze",IF(N114&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8010,11 +8010,11 @@
       </c>
       <c r="L115">
         <f>IF(K115="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K115/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>635</v>
+        <v>595</v>
       </c>
       <c r="N115">
         <f>IF(L115="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L115+IF(M115="",0,M115))))</f>
-        <v>635</v>
+        <v>595</v>
       </c>
       <c r="O115" t="str">
         <f>IF(N115="","",IF(N115&gt;=Instellingen!$B$22,"Absolute top",IF(N115&gt;=Instellingen!$B$23,"Kopman",IF(N115&gt;=Instellingen!$B$24,"Sterke keuze",IF(N115&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8067,11 +8067,11 @@
       </c>
       <c r="L116">
         <f>IF(K116="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K116/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>633</v>
+        <v>593</v>
       </c>
       <c r="N116">
         <f>IF(L116="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L116+IF(M116="",0,M116))))</f>
-        <v>633</v>
+        <v>593</v>
       </c>
       <c r="O116" t="str">
         <f>IF(N116="","",IF(N116&gt;=Instellingen!$B$22,"Absolute top",IF(N116&gt;=Instellingen!$B$23,"Kopman",IF(N116&gt;=Instellingen!$B$24,"Sterke keuze",IF(N116&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8124,11 +8124,11 @@
       </c>
       <c r="L117">
         <f>IF(K117="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K117/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>633</v>
+        <v>593</v>
       </c>
       <c r="N117">
         <f>IF(L117="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L117+IF(M117="",0,M117))))</f>
-        <v>633</v>
+        <v>593</v>
       </c>
       <c r="O117" t="str">
         <f>IF(N117="","",IF(N117&gt;=Instellingen!$B$22,"Absolute top",IF(N117&gt;=Instellingen!$B$23,"Kopman",IF(N117&gt;=Instellingen!$B$24,"Sterke keuze",IF(N117&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8181,11 +8181,11 @@
       </c>
       <c r="L118">
         <f>IF(K118="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K118/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>632</v>
+        <v>593</v>
       </c>
       <c r="N118">
         <f>IF(L118="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L118+IF(M118="",0,M118))))</f>
-        <v>632</v>
+        <v>593</v>
       </c>
       <c r="O118" t="str">
         <f>IF(N118="","",IF(N118&gt;=Instellingen!$B$22,"Absolute top",IF(N118&gt;=Instellingen!$B$23,"Kopman",IF(N118&gt;=Instellingen!$B$24,"Sterke keuze",IF(N118&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8238,11 +8238,11 @@
       </c>
       <c r="L119">
         <f>IF(K119="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K119/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>629</v>
+        <v>590</v>
       </c>
       <c r="N119">
         <f>IF(L119="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L119+IF(M119="",0,M119))))</f>
-        <v>629</v>
+        <v>590</v>
       </c>
       <c r="O119" t="str">
         <f>IF(N119="","",IF(N119&gt;=Instellingen!$B$22,"Absolute top",IF(N119&gt;=Instellingen!$B$23,"Kopman",IF(N119&gt;=Instellingen!$B$24,"Sterke keuze",IF(N119&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8295,11 +8295,11 @@
       </c>
       <c r="L120">
         <f>IF(K120="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K120/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>629</v>
+        <v>590</v>
       </c>
       <c r="N120">
         <f>IF(L120="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L120+IF(M120="",0,M120))))</f>
-        <v>629</v>
+        <v>590</v>
       </c>
       <c r="O120" t="str">
         <f>IF(N120="","",IF(N120&gt;=Instellingen!$B$22,"Absolute top",IF(N120&gt;=Instellingen!$B$23,"Kopman",IF(N120&gt;=Instellingen!$B$24,"Sterke keuze",IF(N120&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8352,11 +8352,11 @@
       </c>
       <c r="L121">
         <f>IF(K121="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K121/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>627</v>
+        <v>588</v>
       </c>
       <c r="N121">
         <f>IF(L121="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L121+IF(M121="",0,M121))))</f>
-        <v>627</v>
+        <v>588</v>
       </c>
       <c r="O121" t="str">
         <f>IF(N121="","",IF(N121&gt;=Instellingen!$B$22,"Absolute top",IF(N121&gt;=Instellingen!$B$23,"Kopman",IF(N121&gt;=Instellingen!$B$24,"Sterke keuze",IF(N121&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8409,11 +8409,11 @@
       </c>
       <c r="L122">
         <f>IF(K122="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K122/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>625</v>
+        <v>586</v>
       </c>
       <c r="N122">
         <f>IF(L122="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L122+IF(M122="",0,M122))))</f>
-        <v>625</v>
+        <v>586</v>
       </c>
       <c r="O122" t="str">
         <f>IF(N122="","",IF(N122&gt;=Instellingen!$B$22,"Absolute top",IF(N122&gt;=Instellingen!$B$23,"Kopman",IF(N122&gt;=Instellingen!$B$24,"Sterke keuze",IF(N122&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8466,11 +8466,11 @@
       </c>
       <c r="L123">
         <f>IF(K123="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K123/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>624</v>
+        <v>585</v>
       </c>
       <c r="N123">
         <f>IF(L123="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L123+IF(M123="",0,M123))))</f>
-        <v>624</v>
+        <v>585</v>
       </c>
       <c r="O123" t="str">
         <f>IF(N123="","",IF(N123&gt;=Instellingen!$B$22,"Absolute top",IF(N123&gt;=Instellingen!$B$23,"Kopman",IF(N123&gt;=Instellingen!$B$24,"Sterke keuze",IF(N123&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8523,11 +8523,11 @@
       </c>
       <c r="L124">
         <f>IF(K124="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K124/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>621</v>
+        <v>583</v>
       </c>
       <c r="N124">
         <f>IF(L124="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L124+IF(M124="",0,M124))))</f>
-        <v>621</v>
+        <v>583</v>
       </c>
       <c r="O124" t="str">
         <f>IF(N124="","",IF(N124&gt;=Instellingen!$B$22,"Absolute top",IF(N124&gt;=Instellingen!$B$23,"Kopman",IF(N124&gt;=Instellingen!$B$24,"Sterke keuze",IF(N124&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8580,11 +8580,11 @@
       </c>
       <c r="L125">
         <f>IF(K125="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K125/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>620</v>
+        <v>582</v>
       </c>
       <c r="N125">
         <f>IF(L125="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L125+IF(M125="",0,M125))))</f>
-        <v>620</v>
+        <v>582</v>
       </c>
       <c r="O125" t="str">
         <f>IF(N125="","",IF(N125&gt;=Instellingen!$B$22,"Absolute top",IF(N125&gt;=Instellingen!$B$23,"Kopman",IF(N125&gt;=Instellingen!$B$24,"Sterke keuze",IF(N125&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8637,11 +8637,11 @@
       </c>
       <c r="L126">
         <f>IF(K126="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K126/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>620</v>
+        <v>582</v>
       </c>
       <c r="N126">
         <f>IF(L126="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L126+IF(M126="",0,M126))))</f>
-        <v>620</v>
+        <v>582</v>
       </c>
       <c r="O126" t="str">
         <f>IF(N126="","",IF(N126&gt;=Instellingen!$B$22,"Absolute top",IF(N126&gt;=Instellingen!$B$23,"Kopman",IF(N126&gt;=Instellingen!$B$24,"Sterke keuze",IF(N126&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8694,11 +8694,11 @@
       </c>
       <c r="L127">
         <f>IF(K127="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K127/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>619</v>
+        <v>581</v>
       </c>
       <c r="N127">
         <f>IF(L127="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L127+IF(M127="",0,M127))))</f>
-        <v>619</v>
+        <v>581</v>
       </c>
       <c r="O127" t="str">
         <f>IF(N127="","",IF(N127&gt;=Instellingen!$B$22,"Absolute top",IF(N127&gt;=Instellingen!$B$23,"Kopman",IF(N127&gt;=Instellingen!$B$24,"Sterke keuze",IF(N127&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8751,11 +8751,11 @@
       </c>
       <c r="L128">
         <f>IF(K128="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K128/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>619</v>
+        <v>581</v>
       </c>
       <c r="N128">
         <f>IF(L128="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L128+IF(M128="",0,M128))))</f>
-        <v>619</v>
+        <v>581</v>
       </c>
       <c r="O128" t="str">
         <f>IF(N128="","",IF(N128&gt;=Instellingen!$B$22,"Absolute top",IF(N128&gt;=Instellingen!$B$23,"Kopman",IF(N128&gt;=Instellingen!$B$24,"Sterke keuze",IF(N128&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8808,11 +8808,11 @@
       </c>
       <c r="L129">
         <f>IF(K129="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K129/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>616</v>
+        <v>578</v>
       </c>
       <c r="N129">
         <f>IF(L129="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L129+IF(M129="",0,M129))))</f>
-        <v>616</v>
+        <v>578</v>
       </c>
       <c r="O129" t="str">
         <f>IF(N129="","",IF(N129&gt;=Instellingen!$B$22,"Absolute top",IF(N129&gt;=Instellingen!$B$23,"Kopman",IF(N129&gt;=Instellingen!$B$24,"Sterke keuze",IF(N129&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8865,11 +8865,11 @@
       </c>
       <c r="L130">
         <f>IF(K130="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K130/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>603</v>
+        <v>567</v>
       </c>
       <c r="N130">
         <f>IF(L130="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L130+IF(M130="",0,M130))))</f>
-        <v>603</v>
+        <v>567</v>
       </c>
       <c r="O130" t="str">
         <f>IF(N130="","",IF(N130&gt;=Instellingen!$B$22,"Absolute top",IF(N130&gt;=Instellingen!$B$23,"Kopman",IF(N130&gt;=Instellingen!$B$24,"Sterke keuze",IF(N130&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8922,11 +8922,11 @@
       </c>
       <c r="L131">
         <f>IF(K131="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K131/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>600</v>
+        <v>565</v>
       </c>
       <c r="N131">
         <f>IF(L131="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L131+IF(M131="",0,M131))))</f>
-        <v>600</v>
+        <v>565</v>
       </c>
       <c r="O131" t="str">
         <f>IF(N131="","",IF(N131&gt;=Instellingen!$B$22,"Absolute top",IF(N131&gt;=Instellingen!$B$23,"Kopman",IF(N131&gt;=Instellingen!$B$24,"Sterke keuze",IF(N131&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -8979,11 +8979,11 @@
       </c>
       <c r="L132">
         <f>IF(K132="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K132/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>597</v>
+        <v>562</v>
       </c>
       <c r="N132">
         <f>IF(L132="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L132+IF(M132="",0,M132))))</f>
-        <v>597</v>
+        <v>562</v>
       </c>
       <c r="O132" t="str">
         <f>IF(N132="","",IF(N132&gt;=Instellingen!$B$22,"Absolute top",IF(N132&gt;=Instellingen!$B$23,"Kopman",IF(N132&gt;=Instellingen!$B$24,"Sterke keuze",IF(N132&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9036,11 +9036,11 @@
       </c>
       <c r="L133">
         <f>IF(K133="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K133/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>596</v>
+        <v>560</v>
       </c>
       <c r="N133">
         <f>IF(L133="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L133+IF(M133="",0,M133))))</f>
-        <v>596</v>
+        <v>560</v>
       </c>
       <c r="O133" t="str">
         <f>IF(N133="","",IF(N133&gt;=Instellingen!$B$22,"Absolute top",IF(N133&gt;=Instellingen!$B$23,"Kopman",IF(N133&gt;=Instellingen!$B$24,"Sterke keuze",IF(N133&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9093,11 +9093,11 @@
       </c>
       <c r="L134">
         <f>IF(K134="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K134/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>591</v>
+        <v>556</v>
       </c>
       <c r="N134">
         <f>IF(L134="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L134+IF(M134="",0,M134))))</f>
-        <v>591</v>
+        <v>556</v>
       </c>
       <c r="O134" t="str">
         <f>IF(N134="","",IF(N134&gt;=Instellingen!$B$22,"Absolute top",IF(N134&gt;=Instellingen!$B$23,"Kopman",IF(N134&gt;=Instellingen!$B$24,"Sterke keuze",IF(N134&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9150,11 +9150,11 @@
       </c>
       <c r="L135">
         <f>IF(K135="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K135/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>590</v>
+        <v>555</v>
       </c>
       <c r="N135">
         <f>IF(L135="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L135+IF(M135="",0,M135))))</f>
-        <v>590</v>
+        <v>555</v>
       </c>
       <c r="O135" t="str">
         <f>IF(N135="","",IF(N135&gt;=Instellingen!$B$22,"Absolute top",IF(N135&gt;=Instellingen!$B$23,"Kopman",IF(N135&gt;=Instellingen!$B$24,"Sterke keuze",IF(N135&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9207,11 +9207,11 @@
       </c>
       <c r="L136">
         <f>IF(K136="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K136/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>589</v>
+        <v>554</v>
       </c>
       <c r="N136">
         <f>IF(L136="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L136+IF(M136="",0,M136))))</f>
-        <v>589</v>
+        <v>554</v>
       </c>
       <c r="O136" t="str">
         <f>IF(N136="","",IF(N136&gt;=Instellingen!$B$22,"Absolute top",IF(N136&gt;=Instellingen!$B$23,"Kopman",IF(N136&gt;=Instellingen!$B$24,"Sterke keuze",IF(N136&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9264,11 +9264,11 @@
       </c>
       <c r="L137">
         <f>IF(K137="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K137/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>586</v>
+        <v>552</v>
       </c>
       <c r="N137">
         <f>IF(L137="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L137+IF(M137="",0,M137))))</f>
-        <v>586</v>
+        <v>552</v>
       </c>
       <c r="O137" t="str">
         <f>IF(N137="","",IF(N137&gt;=Instellingen!$B$22,"Absolute top",IF(N137&gt;=Instellingen!$B$23,"Kopman",IF(N137&gt;=Instellingen!$B$24,"Sterke keuze",IF(N137&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9321,11 +9321,11 @@
       </c>
       <c r="L138">
         <f>IF(K138="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K138/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>579</v>
+        <v>546</v>
       </c>
       <c r="N138">
         <f>IF(L138="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L138+IF(M138="",0,M138))))</f>
-        <v>579</v>
+        <v>546</v>
       </c>
       <c r="O138" t="str">
         <f>IF(N138="","",IF(N138&gt;=Instellingen!$B$22,"Absolute top",IF(N138&gt;=Instellingen!$B$23,"Kopman",IF(N138&gt;=Instellingen!$B$24,"Sterke keuze",IF(N138&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9378,11 +9378,11 @@
       </c>
       <c r="L139">
         <f>IF(K139="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K139/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>576</v>
+        <v>543</v>
       </c>
       <c r="N139">
         <f>IF(L139="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L139+IF(M139="",0,M139))))</f>
-        <v>576</v>
+        <v>543</v>
       </c>
       <c r="O139" t="str">
         <f>IF(N139="","",IF(N139&gt;=Instellingen!$B$22,"Absolute top",IF(N139&gt;=Instellingen!$B$23,"Kopman",IF(N139&gt;=Instellingen!$B$24,"Sterke keuze",IF(N139&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9435,11 +9435,11 @@
       </c>
       <c r="L140">
         <f>IF(K140="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K140/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>575</v>
+        <v>542</v>
       </c>
       <c r="N140">
         <f>IF(L140="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L140+IF(M140="",0,M140))))</f>
-        <v>575</v>
+        <v>542</v>
       </c>
       <c r="O140" t="str">
         <f>IF(N140="","",IF(N140&gt;=Instellingen!$B$22,"Absolute top",IF(N140&gt;=Instellingen!$B$23,"Kopman",IF(N140&gt;=Instellingen!$B$24,"Sterke keuze",IF(N140&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9492,11 +9492,11 @@
       </c>
       <c r="L141">
         <f>IF(K141="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K141/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>574</v>
+        <v>541</v>
       </c>
       <c r="N141">
         <f>IF(L141="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L141+IF(M141="",0,M141))))</f>
-        <v>574</v>
+        <v>541</v>
       </c>
       <c r="O141" t="str">
         <f>IF(N141="","",IF(N141&gt;=Instellingen!$B$22,"Absolute top",IF(N141&gt;=Instellingen!$B$23,"Kopman",IF(N141&gt;=Instellingen!$B$24,"Sterke keuze",IF(N141&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9549,11 +9549,11 @@
       </c>
       <c r="L142">
         <f>IF(K142="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K142/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>572</v>
+        <v>540</v>
       </c>
       <c r="N142">
         <f>IF(L142="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L142+IF(M142="",0,M142))))</f>
-        <v>572</v>
+        <v>540</v>
       </c>
       <c r="O142" t="str">
         <f>IF(N142="","",IF(N142&gt;=Instellingen!$B$22,"Absolute top",IF(N142&gt;=Instellingen!$B$23,"Kopman",IF(N142&gt;=Instellingen!$B$24,"Sterke keuze",IF(N142&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9606,11 +9606,11 @@
       </c>
       <c r="L143">
         <f>IF(K143="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K143/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>564</v>
+        <v>533</v>
       </c>
       <c r="N143">
         <f>IF(L143="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L143+IF(M143="",0,M143))))</f>
-        <v>564</v>
+        <v>533</v>
       </c>
       <c r="O143" t="str">
         <f>IF(N143="","",IF(N143&gt;=Instellingen!$B$22,"Absolute top",IF(N143&gt;=Instellingen!$B$23,"Kopman",IF(N143&gt;=Instellingen!$B$24,"Sterke keuze",IF(N143&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9663,11 +9663,11 @@
       </c>
       <c r="L144">
         <f>IF(K144="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K144/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>557</v>
+        <v>527</v>
       </c>
       <c r="N144">
         <f>IF(L144="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L144+IF(M144="",0,M144))))</f>
-        <v>557</v>
+        <v>527</v>
       </c>
       <c r="O144" t="str">
         <f>IF(N144="","",IF(N144&gt;=Instellingen!$B$22,"Absolute top",IF(N144&gt;=Instellingen!$B$23,"Kopman",IF(N144&gt;=Instellingen!$B$24,"Sterke keuze",IF(N144&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9720,11 +9720,11 @@
       </c>
       <c r="L145">
         <f>IF(K145="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K145/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>543</v>
+        <v>514</v>
       </c>
       <c r="N145">
         <f>IF(L145="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L145+IF(M145="",0,M145))))</f>
-        <v>543</v>
+        <v>514</v>
       </c>
       <c r="O145" t="str">
         <f>IF(N145="","",IF(N145&gt;=Instellingen!$B$22,"Absolute top",IF(N145&gt;=Instellingen!$B$23,"Kopman",IF(N145&gt;=Instellingen!$B$24,"Sterke keuze",IF(N145&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9777,11 +9777,11 @@
       </c>
       <c r="L146">
         <f>IF(K146="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K146/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>532</v>
+        <v>504</v>
       </c>
       <c r="N146">
         <f>IF(L146="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L146+IF(M146="",0,M146))))</f>
-        <v>532</v>
+        <v>504</v>
       </c>
       <c r="O146" t="str">
         <f>IF(N146="","",IF(N146&gt;=Instellingen!$B$22,"Absolute top",IF(N146&gt;=Instellingen!$B$23,"Kopman",IF(N146&gt;=Instellingen!$B$24,"Sterke keuze",IF(N146&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9834,11 +9834,11 @@
       </c>
       <c r="L147">
         <f>IF(K147="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K147/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>530</v>
+        <v>502</v>
       </c>
       <c r="N147">
         <f>IF(L147="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L147+IF(M147="",0,M147))))</f>
-        <v>530</v>
+        <v>502</v>
       </c>
       <c r="O147" t="str">
         <f>IF(N147="","",IF(N147&gt;=Instellingen!$B$22,"Absolute top",IF(N147&gt;=Instellingen!$B$23,"Kopman",IF(N147&gt;=Instellingen!$B$24,"Sterke keuze",IF(N147&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9891,11 +9891,11 @@
       </c>
       <c r="L148">
         <f>IF(K148="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K148/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>527</v>
+        <v>500</v>
       </c>
       <c r="N148">
         <f>IF(L148="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L148+IF(M148="",0,M148))))</f>
-        <v>527</v>
+        <v>500</v>
       </c>
       <c r="O148" t="str">
         <f>IF(N148="","",IF(N148&gt;=Instellingen!$B$22,"Absolute top",IF(N148&gt;=Instellingen!$B$23,"Kopman",IF(N148&gt;=Instellingen!$B$24,"Sterke keuze",IF(N148&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -9948,11 +9948,11 @@
       </c>
       <c r="L149">
         <f>IF(K149="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K149/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>503</v>
+        <v>479</v>
       </c>
       <c r="N149">
         <f>IF(L149="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L149+IF(M149="",0,M149))))</f>
-        <v>503</v>
+        <v>479</v>
       </c>
       <c r="O149" t="str">
         <f>IF(N149="","",IF(N149&gt;=Instellingen!$B$22,"Absolute top",IF(N149&gt;=Instellingen!$B$23,"Kopman",IF(N149&gt;=Instellingen!$B$24,"Sterke keuze",IF(N149&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10005,11 +10005,11 @@
       </c>
       <c r="L150">
         <f>IF(K150="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K150/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>500</v>
+        <v>476</v>
       </c>
       <c r="N150">
         <f>IF(L150="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L150+IF(M150="",0,M150))))</f>
-        <v>500</v>
+        <v>476</v>
       </c>
       <c r="O150" t="str">
         <f>IF(N150="","",IF(N150&gt;=Instellingen!$B$22,"Absolute top",IF(N150&gt;=Instellingen!$B$23,"Kopman",IF(N150&gt;=Instellingen!$B$24,"Sterke keuze",IF(N150&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10062,11 +10062,11 @@
       </c>
       <c r="L151">
         <f>IF(K151="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K151/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>492</v>
+        <v>469</v>
       </c>
       <c r="N151">
         <f>IF(L151="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L151+IF(M151="",0,M151))))</f>
-        <v>492</v>
+        <v>469</v>
       </c>
       <c r="O151" t="str">
         <f>IF(N151="","",IF(N151&gt;=Instellingen!$B$22,"Absolute top",IF(N151&gt;=Instellingen!$B$23,"Kopman",IF(N151&gt;=Instellingen!$B$24,"Sterke keuze",IF(N151&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10119,11 +10119,11 @@
       </c>
       <c r="L152">
         <f>IF(K152="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K152/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>491</v>
+        <v>468</v>
       </c>
       <c r="N152">
         <f>IF(L152="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L152+IF(M152="",0,M152))))</f>
-        <v>491</v>
+        <v>468</v>
       </c>
       <c r="O152" t="str">
         <f>IF(N152="","",IF(N152&gt;=Instellingen!$B$22,"Absolute top",IF(N152&gt;=Instellingen!$B$23,"Kopman",IF(N152&gt;=Instellingen!$B$24,"Sterke keuze",IF(N152&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10176,11 +10176,11 @@
       </c>
       <c r="L153">
         <f>IF(K153="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K153/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>473</v>
+        <v>453</v>
       </c>
       <c r="N153">
         <f>IF(L153="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L153+IF(M153="",0,M153))))</f>
-        <v>473</v>
+        <v>453</v>
       </c>
       <c r="O153" t="str">
         <f>IF(N153="","",IF(N153&gt;=Instellingen!$B$22,"Absolute top",IF(N153&gt;=Instellingen!$B$23,"Kopman",IF(N153&gt;=Instellingen!$B$24,"Sterke keuze",IF(N153&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10233,11 +10233,11 @@
       </c>
       <c r="L154">
         <f>IF(K154="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K154/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>464</v>
+        <v>445</v>
       </c>
       <c r="N154">
         <f>IF(L154="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L154+IF(M154="",0,M154))))</f>
-        <v>464</v>
+        <v>445</v>
       </c>
       <c r="O154" t="str">
         <f>IF(N154="","",IF(N154&gt;=Instellingen!$B$22,"Absolute top",IF(N154&gt;=Instellingen!$B$23,"Kopman",IF(N154&gt;=Instellingen!$B$24,"Sterke keuze",IF(N154&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10290,11 +10290,11 @@
       </c>
       <c r="L155">
         <f>IF(K155="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K155/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>450</v>
+        <v>432</v>
       </c>
       <c r="N155">
         <f>IF(L155="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L155+IF(M155="",0,M155))))</f>
-        <v>450</v>
+        <v>432</v>
       </c>
       <c r="O155" t="str">
         <f>IF(N155="","",IF(N155&gt;=Instellingen!$B$22,"Absolute top",IF(N155&gt;=Instellingen!$B$23,"Kopman",IF(N155&gt;=Instellingen!$B$24,"Sterke keuze",IF(N155&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10347,11 +10347,11 @@
       </c>
       <c r="L156">
         <f>IF(K156="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K156/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="N156">
         <f>IF(L156="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L156+IF(M156="",0,M156))))</f>
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="O156" t="str">
         <f>IF(N156="","",IF(N156&gt;=Instellingen!$B$22,"Absolute top",IF(N156&gt;=Instellingen!$B$23,"Kopman",IF(N156&gt;=Instellingen!$B$24,"Sterke keuze",IF(N156&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10404,11 +10404,11 @@
       </c>
       <c r="L157">
         <f>IF(K157="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K157/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="N157">
         <f>IF(L157="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L157+IF(M157="",0,M157))))</f>
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="O157" t="str">
         <f>IF(N157="","",IF(N157&gt;=Instellingen!$B$22,"Absolute top",IF(N157&gt;=Instellingen!$B$23,"Kopman",IF(N157&gt;=Instellingen!$B$24,"Sterke keuze",IF(N157&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10461,11 +10461,11 @@
       </c>
       <c r="L158">
         <f>IF(K158="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K158/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>446</v>
+        <v>429</v>
       </c>
       <c r="N158">
         <f>IF(L158="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L158+IF(M158="",0,M158))))</f>
-        <v>446</v>
+        <v>429</v>
       </c>
       <c r="O158" t="str">
         <f>IF(N158="","",IF(N158&gt;=Instellingen!$B$22,"Absolute top",IF(N158&gt;=Instellingen!$B$23,"Kopman",IF(N158&gt;=Instellingen!$B$24,"Sterke keuze",IF(N158&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10518,11 +10518,11 @@
       </c>
       <c r="L159">
         <f>IF(K159="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K159/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>445</v>
+        <v>428</v>
       </c>
       <c r="N159">
         <f>IF(L159="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L159+IF(M159="",0,M159))))</f>
-        <v>445</v>
+        <v>428</v>
       </c>
       <c r="O159" t="str">
         <f>IF(N159="","",IF(N159&gt;=Instellingen!$B$22,"Absolute top",IF(N159&gt;=Instellingen!$B$23,"Kopman",IF(N159&gt;=Instellingen!$B$24,"Sterke keuze",IF(N159&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10575,11 +10575,11 @@
       </c>
       <c r="L160">
         <f>IF(K160="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K160/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>439</v>
+        <v>422</v>
       </c>
       <c r="N160">
         <f>IF(L160="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L160+IF(M160="",0,M160))))</f>
-        <v>439</v>
+        <v>422</v>
       </c>
       <c r="O160" t="str">
         <f>IF(N160="","",IF(N160&gt;=Instellingen!$B$22,"Absolute top",IF(N160&gt;=Instellingen!$B$23,"Kopman",IF(N160&gt;=Instellingen!$B$24,"Sterke keuze",IF(N160&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10632,11 +10632,11 @@
       </c>
       <c r="L161">
         <f>IF(K161="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K161/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>434</v>
+        <v>418</v>
       </c>
       <c r="N161">
         <f>IF(L161="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L161+IF(M161="",0,M161))))</f>
-        <v>434</v>
+        <v>418</v>
       </c>
       <c r="O161" t="str">
         <f>IF(N161="","",IF(N161&gt;=Instellingen!$B$22,"Absolute top",IF(N161&gt;=Instellingen!$B$23,"Kopman",IF(N161&gt;=Instellingen!$B$24,"Sterke keuze",IF(N161&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10689,11 +10689,11 @@
       </c>
       <c r="L162">
         <f>IF(K162="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K162/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>433</v>
+        <v>418</v>
       </c>
       <c r="N162">
         <f>IF(L162="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L162+IF(M162="",0,M162))))</f>
-        <v>433</v>
+        <v>418</v>
       </c>
       <c r="O162" t="str">
         <f>IF(N162="","",IF(N162&gt;=Instellingen!$B$22,"Absolute top",IF(N162&gt;=Instellingen!$B$23,"Kopman",IF(N162&gt;=Instellingen!$B$24,"Sterke keuze",IF(N162&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10746,11 +10746,11 @@
       </c>
       <c r="L163">
         <f>IF(K163="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K163/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>430</v>
+        <v>414</v>
       </c>
       <c r="N163">
         <f>IF(L163="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L163+IF(M163="",0,M163))))</f>
-        <v>430</v>
+        <v>414</v>
       </c>
       <c r="O163" t="str">
         <f>IF(N163="","",IF(N163&gt;=Instellingen!$B$22,"Absolute top",IF(N163&gt;=Instellingen!$B$23,"Kopman",IF(N163&gt;=Instellingen!$B$24,"Sterke keuze",IF(N163&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10803,11 +10803,11 @@
       </c>
       <c r="L164">
         <f>IF(K164="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K164/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="N164">
         <f>IF(L164="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L164+IF(M164="",0,M164))))</f>
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="O164" t="str">
         <f>IF(N164="","",IF(N164&gt;=Instellingen!$B$22,"Absolute top",IF(N164&gt;=Instellingen!$B$23,"Kopman",IF(N164&gt;=Instellingen!$B$24,"Sterke keuze",IF(N164&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10860,11 +10860,11 @@
       </c>
       <c r="L165">
         <f>IF(K165="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K165/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>420</v>
+        <v>406</v>
       </c>
       <c r="N165">
         <f>IF(L165="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L165+IF(M165="",0,M165))))</f>
-        <v>420</v>
+        <v>406</v>
       </c>
       <c r="O165" t="str">
         <f>IF(N165="","",IF(N165&gt;=Instellingen!$B$22,"Absolute top",IF(N165&gt;=Instellingen!$B$23,"Kopman",IF(N165&gt;=Instellingen!$B$24,"Sterke keuze",IF(N165&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10917,11 +10917,11 @@
       </c>
       <c r="L166">
         <f>IF(K166="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K166/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="N166">
         <f>IF(L166="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L166+IF(M166="",0,M166))))</f>
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="O166" t="str">
         <f>IF(N166="","",IF(N166&gt;=Instellingen!$B$22,"Absolute top",IF(N166&gt;=Instellingen!$B$23,"Kopman",IF(N166&gt;=Instellingen!$B$24,"Sterke keuze",IF(N166&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -10974,11 +10974,11 @@
       </c>
       <c r="L167">
         <f>IF(K167="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K167/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>413</v>
+        <v>400</v>
       </c>
       <c r="N167">
         <f>IF(L167="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L167+IF(M167="",0,M167))))</f>
-        <v>413</v>
+        <v>400</v>
       </c>
       <c r="O167" t="str">
         <f>IF(N167="","",IF(N167&gt;=Instellingen!$B$22,"Absolute top",IF(N167&gt;=Instellingen!$B$23,"Kopman",IF(N167&gt;=Instellingen!$B$24,"Sterke keuze",IF(N167&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11031,11 +11031,11 @@
       </c>
       <c r="L168">
         <f>IF(K168="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K168/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="N168">
         <f>IF(L168="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L168+IF(M168="",0,M168))))</f>
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="O168" t="str">
         <f>IF(N168="","",IF(N168&gt;=Instellingen!$B$22,"Absolute top",IF(N168&gt;=Instellingen!$B$23,"Kopman",IF(N168&gt;=Instellingen!$B$24,"Sterke keuze",IF(N168&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11088,11 +11088,11 @@
       </c>
       <c r="L169">
         <f>IF(K169="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K169/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>406</v>
+        <v>393</v>
       </c>
       <c r="N169">
         <f>IF(L169="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L169+IF(M169="",0,M169))))</f>
-        <v>406</v>
+        <v>393</v>
       </c>
       <c r="O169" t="str">
         <f>IF(N169="","",IF(N169&gt;=Instellingen!$B$22,"Absolute top",IF(N169&gt;=Instellingen!$B$23,"Kopman",IF(N169&gt;=Instellingen!$B$24,"Sterke keuze",IF(N169&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11145,11 +11145,11 @@
       </c>
       <c r="L170">
         <f>IF(K170="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K170/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="N170">
         <f>IF(L170="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L170+IF(M170="",0,M170))))</f>
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="O170" t="str">
         <f>IF(N170="","",IF(N170&gt;=Instellingen!$B$22,"Absolute top",IF(N170&gt;=Instellingen!$B$23,"Kopman",IF(N170&gt;=Instellingen!$B$24,"Sterke keuze",IF(N170&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11202,11 +11202,11 @@
       </c>
       <c r="L171">
         <f>IF(K171="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K171/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="N171">
         <f>IF(L171="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L171+IF(M171="",0,M171))))</f>
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="O171" t="str">
         <f>IF(N171="","",IF(N171&gt;=Instellingen!$B$22,"Absolute top",IF(N171&gt;=Instellingen!$B$23,"Kopman",IF(N171&gt;=Instellingen!$B$24,"Sterke keuze",IF(N171&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11259,11 +11259,11 @@
       </c>
       <c r="L172">
         <f>IF(K172="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K172/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="N172">
         <f>IF(L172="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L172+IF(M172="",0,M172))))</f>
-        <v>403</v>
+        <v>391</v>
       </c>
       <c r="O172" t="str">
         <f>IF(N172="","",IF(N172&gt;=Instellingen!$B$22,"Absolute top",IF(N172&gt;=Instellingen!$B$23,"Kopman",IF(N172&gt;=Instellingen!$B$24,"Sterke keuze",IF(N172&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11316,11 +11316,11 @@
       </c>
       <c r="L173">
         <f>IF(K173="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K173/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="N173">
         <f>IF(L173="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L173+IF(M173="",0,M173))))</f>
-        <v>401</v>
+        <v>389</v>
       </c>
       <c r="O173" t="str">
         <f>IF(N173="","",IF(N173&gt;=Instellingen!$B$22,"Absolute top",IF(N173&gt;=Instellingen!$B$23,"Kopman",IF(N173&gt;=Instellingen!$B$24,"Sterke keuze",IF(N173&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11373,11 +11373,11 @@
       </c>
       <c r="L174">
         <f>IF(K174="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K174/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="N174">
         <f>IF(L174="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L174+IF(M174="",0,M174))))</f>
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="O174" t="str">
         <f>IF(N174="","",IF(N174&gt;=Instellingen!$B$22,"Absolute top",IF(N174&gt;=Instellingen!$B$23,"Kopman",IF(N174&gt;=Instellingen!$B$24,"Sterke keuze",IF(N174&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11430,11 +11430,11 @@
       </c>
       <c r="L175">
         <f>IF(K175="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K175/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="N175">
         <f>IF(L175="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L175+IF(M175="",0,M175))))</f>
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="O175" t="str">
         <f>IF(N175="","",IF(N175&gt;=Instellingen!$B$22,"Absolute top",IF(N175&gt;=Instellingen!$B$23,"Kopman",IF(N175&gt;=Instellingen!$B$24,"Sterke keuze",IF(N175&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11487,11 +11487,11 @@
       </c>
       <c r="L176">
         <f>IF(K176="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K176/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="N176">
         <f>IF(L176="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L176+IF(M176="",0,M176))))</f>
-        <v>396</v>
+        <v>384</v>
       </c>
       <c r="O176" t="str">
         <f>IF(N176="","",IF(N176&gt;=Instellingen!$B$22,"Absolute top",IF(N176&gt;=Instellingen!$B$23,"Kopman",IF(N176&gt;=Instellingen!$B$24,"Sterke keuze",IF(N176&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11544,11 +11544,11 @@
       </c>
       <c r="L177">
         <f>IF(K177="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K177/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="N177">
         <f>IF(L177="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L177+IF(M177="",0,M177))))</f>
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="O177" t="str">
         <f>IF(N177="","",IF(N177&gt;=Instellingen!$B$22,"Absolute top",IF(N177&gt;=Instellingen!$B$23,"Kopman",IF(N177&gt;=Instellingen!$B$24,"Sterke keuze",IF(N177&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11601,11 +11601,11 @@
       </c>
       <c r="L178">
         <f>IF(K178="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K178/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="N178">
         <f>IF(L178="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L178+IF(M178="",0,M178))))</f>
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="O178" t="str">
         <f>IF(N178="","",IF(N178&gt;=Instellingen!$B$22,"Absolute top",IF(N178&gt;=Instellingen!$B$23,"Kopman",IF(N178&gt;=Instellingen!$B$24,"Sterke keuze",IF(N178&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11658,11 +11658,11 @@
       </c>
       <c r="L179">
         <f>IF(K179="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K179/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="N179">
         <f>IF(L179="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L179+IF(M179="",0,M179))))</f>
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="O179" t="str">
         <f>IF(N179="","",IF(N179&gt;=Instellingen!$B$22,"Absolute top",IF(N179&gt;=Instellingen!$B$23,"Kopman",IF(N179&gt;=Instellingen!$B$24,"Sterke keuze",IF(N179&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11715,11 +11715,11 @@
       </c>
       <c r="L180">
         <f>IF(K180="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K180/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="N180">
         <f>IF(L180="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L180+IF(M180="",0,M180))))</f>
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="O180" t="str">
         <f>IF(N180="","",IF(N180&gt;=Instellingen!$B$22,"Absolute top",IF(N180&gt;=Instellingen!$B$23,"Kopman",IF(N180&gt;=Instellingen!$B$24,"Sterke keuze",IF(N180&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11772,11 +11772,11 @@
       </c>
       <c r="L181">
         <f>IF(K181="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K181/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="N181">
         <f>IF(L181="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L181+IF(M181="",0,M181))))</f>
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="O181" t="str">
         <f>IF(N181="","",IF(N181&gt;=Instellingen!$B$22,"Absolute top",IF(N181&gt;=Instellingen!$B$23,"Kopman",IF(N181&gt;=Instellingen!$B$24,"Sterke keuze",IF(N181&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11829,11 +11829,11 @@
       </c>
       <c r="L182">
         <f>IF(K182="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K182/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="N182">
         <f>IF(L182="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L182+IF(M182="",0,M182))))</f>
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="O182" t="str">
         <f>IF(N182="","",IF(N182&gt;=Instellingen!$B$22,"Absolute top",IF(N182&gt;=Instellingen!$B$23,"Kopman",IF(N182&gt;=Instellingen!$B$24,"Sterke keuze",IF(N182&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11886,11 +11886,11 @@
       </c>
       <c r="L183">
         <f>IF(K183="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K183/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="N183">
         <f>IF(L183="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L183+IF(M183="",0,M183))))</f>
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="O183" t="str">
         <f>IF(N183="","",IF(N183&gt;=Instellingen!$B$22,"Absolute top",IF(N183&gt;=Instellingen!$B$23,"Kopman",IF(N183&gt;=Instellingen!$B$24,"Sterke keuze",IF(N183&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -11943,11 +11943,11 @@
       </c>
       <c r="L184">
         <f>IF(K184="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K184/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="N184">
         <f>IF(L184="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L184+IF(M184="",0,M184))))</f>
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="O184" t="str">
         <f>IF(N184="","",IF(N184&gt;=Instellingen!$B$22,"Absolute top",IF(N184&gt;=Instellingen!$B$23,"Kopman",IF(N184&gt;=Instellingen!$B$24,"Sterke keuze",IF(N184&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -12000,11 +12000,11 @@
       </c>
       <c r="L185">
         <f>IF(K185="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K185/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="N185">
         <f>IF(L185="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L185+IF(M185="",0,M185))))</f>
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="O185" t="str">
         <f>IF(N185="","",IF(N185&gt;=Instellingen!$B$22,"Absolute top",IF(N185&gt;=Instellingen!$B$23,"Kopman",IF(N185&gt;=Instellingen!$B$24,"Sterke keuze",IF(N185&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -12057,11 +12057,11 @@
       </c>
       <c r="L186">
         <f>IF(K186="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K186/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="N186">
         <f>IF(L186="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L186+IF(M186="",0,M186))))</f>
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="O186" t="str">
         <f>IF(N186="","",IF(N186&gt;=Instellingen!$B$22,"Absolute top",IF(N186&gt;=Instellingen!$B$23,"Kopman",IF(N186&gt;=Instellingen!$B$24,"Sterke keuze",IF(N186&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -12114,11 +12114,11 @@
       </c>
       <c r="L187">
         <f>IF(K187="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K187/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="N187">
         <f>IF(L187="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L187+IF(M187="",0,M187))))</f>
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="O187" t="str">
         <f>IF(N187="","",IF(N187&gt;=Instellingen!$B$22,"Absolute top",IF(N187&gt;=Instellingen!$B$23,"Kopman",IF(N187&gt;=Instellingen!$B$24,"Sterke keuze",IF(N187&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -12171,11 +12171,11 @@
       </c>
       <c r="L188">
         <f>IF(K188="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K188/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="N188">
         <f>IF(L188="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L188+IF(M188="",0,M188))))</f>
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="O188" t="str">
         <f>IF(N188="","",IF(N188&gt;=Instellingen!$B$22,"Absolute top",IF(N188&gt;=Instellingen!$B$23,"Kopman",IF(N188&gt;=Instellingen!$B$24,"Sterke keuze",IF(N188&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -12228,11 +12228,11 @@
       </c>
       <c r="L189">
         <f>IF(K189="","",ROUND((Instellingen!$B$16+(Instellingen!$B$17-Instellingen!$B$16)*POWER(K189/100,Instellingen!$B$18))/Instellingen!$B$19,0)*Instellingen!$B$19)</f>
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="N189">
         <f>IF(L189="","",MAX(Instellingen!$B$16,MIN(Instellingen!$B$17,L189+IF(M189="",0,M189))))</f>
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="O189" t="str">
         <f>IF(N189="","",IF(N189&gt;=Instellingen!$B$22,"Absolute top",IF(N189&gt;=Instellingen!$B$23,"Kopman",IF(N189&gt;=Instellingen!$B$24,"Sterke keuze",IF(N189&gt;=Instellingen!$B$25,"Bruikbaar","Gok")))))</f>
@@ -12421,7 +12421,7 @@
         <v>432</v>
       </c>
       <c r="B17">
-        <v>4500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="18" spans="1:2">

</xml_diff>